<commit_message>
Fr and Es databooks after SQLNS
</commit_message>
<xml_diff>
--- a/tests/scen_results_test_2025_SQLNS.xlsx
+++ b/tests/scen_results_test_2025_SQLNS.xlsx
@@ -28,7 +28,7 @@
     <t>2.1.0</t>
   </si>
   <si>
-    <t>2025-07-29</t>
+    <t>2025-07-30</t>
   </si>
   <si>
     <t>Scenario</t>
@@ -5512,46 +5512,46 @@
         <v>0</v>
       </c>
       <c r="E89" s="3">
-        <v>1175600.063393105</v>
+        <v>1175565.880896696</v>
       </c>
       <c r="F89" s="3">
-        <v>1183743.005585368</v>
+        <v>1183518.384179026</v>
       </c>
       <c r="G89" s="3">
-        <v>1193020.311775068</v>
+        <v>1192489.221514715</v>
       </c>
       <c r="H89" s="3">
-        <v>1203901.43102918</v>
+        <v>1202982.826393005</v>
       </c>
       <c r="I89" s="3">
-        <v>1217059.690064977</v>
+        <v>1215760.738302144</v>
       </c>
       <c r="J89" s="3">
-        <v>1232840.037843361</v>
+        <v>1231221.638793531</v>
       </c>
       <c r="K89" s="3">
-        <v>1251358.937711696</v>
+        <v>1249486.851368815</v>
       </c>
       <c r="L89" s="3">
-        <v>1272049.442430496</v>
+        <v>1269978.171949176</v>
       </c>
       <c r="M89" s="3">
-        <v>1294440.847530728</v>
+        <v>1292211.878962416</v>
       </c>
       <c r="N89" s="3">
-        <v>1318665.693677976</v>
+        <v>1316308.572233856</v>
       </c>
       <c r="O89" s="3">
-        <v>1344238.202706082</v>
+        <v>1341773.701577473</v>
       </c>
       <c r="P89" s="3">
-        <v>1370660.494547966</v>
+        <v>1368103.495015938</v>
       </c>
       <c r="Q89" s="3">
-        <v>1397906.015652684</v>
+        <v>1395266.971130894</v>
       </c>
       <c r="R89" s="3">
-        <v>16455484.17394869</v>
+        <v>16434668.33231769</v>
       </c>
     </row>
     <row r="90" spans="1:18">
@@ -5568,46 +5568,46 @@
         <v>0</v>
       </c>
       <c r="E90" s="3">
-        <v>191472.8305431889</v>
+        <v>193717.2897501557</v>
       </c>
       <c r="F90" s="3">
-        <v>193394.5823647756</v>
+        <v>196050.3548677525</v>
       </c>
       <c r="G90" s="3">
-        <v>194692.7329594506</v>
+        <v>198688.1528207878</v>
       </c>
       <c r="H90" s="3">
-        <v>197634.6725811554</v>
+        <v>201673.0660779111</v>
       </c>
       <c r="I90" s="3">
-        <v>201253.4211039281</v>
+        <v>205349.9627065802</v>
       </c>
       <c r="J90" s="3">
-        <v>205135.4083235969</v>
+        <v>209304.8811946179</v>
       </c>
       <c r="K90" s="3">
-        <v>208638.5103990861</v>
+        <v>212885.7032708055</v>
       </c>
       <c r="L90" s="3">
-        <v>213148.4308803786</v>
+        <v>217473.564624953</v>
       </c>
       <c r="M90" s="3">
-        <v>217444.1566823388</v>
+        <v>221860.04927644</v>
       </c>
       <c r="N90" s="3">
-        <v>221723.5148123398</v>
+        <v>226229.3672156177</v>
       </c>
       <c r="O90" s="3">
-        <v>226036.1532042855</v>
+        <v>230630.82545264</v>
       </c>
       <c r="P90" s="3">
-        <v>230898.5241090136</v>
+        <v>235584.677369059</v>
       </c>
       <c r="Q90" s="3">
-        <v>235400.59926692</v>
+        <v>240184.5197252505</v>
       </c>
       <c r="R90" s="3">
-        <v>2736873.537230458</v>
+        <v>2789632.414352571</v>
       </c>
     </row>
     <row r="91" spans="1:18">
@@ -5624,46 +5624,46 @@
         <v>0</v>
       </c>
       <c r="E91" s="3">
-        <v>761142.2120035558</v>
+        <v>761120.4456709523</v>
       </c>
       <c r="F91" s="3">
-        <v>762174.9538583929</v>
+        <v>762032.3815374386</v>
       </c>
       <c r="G91" s="3">
-        <v>763133.8099363408</v>
+        <v>762798.7698819487</v>
       </c>
       <c r="H91" s="3">
-        <v>764811.6043704802</v>
+        <v>764235.2280460199</v>
       </c>
       <c r="I91" s="3">
-        <v>769098.3251957578</v>
+        <v>768285.3629104018</v>
       </c>
       <c r="J91" s="3">
-        <v>776057.3462067296</v>
+        <v>775045.8158652957</v>
       </c>
       <c r="K91" s="3">
-        <v>785527.2591387869</v>
+        <v>784358.0866136401</v>
       </c>
       <c r="L91" s="3">
-        <v>796944.3796279803</v>
+        <v>795651.4369433123</v>
       </c>
       <c r="M91" s="3">
-        <v>809850.7674568847</v>
+        <v>808459.8161108734</v>
       </c>
       <c r="N91" s="3">
-        <v>824207.1652813572</v>
+        <v>822736.5405229733</v>
       </c>
       <c r="O91" s="3">
-        <v>839622.3253960484</v>
+        <v>838084.9132841204</v>
       </c>
       <c r="P91" s="3">
-        <v>855722.5111426678</v>
+        <v>854127.5413838323</v>
       </c>
       <c r="Q91" s="3">
-        <v>872446.1151962263</v>
+        <v>870800.0701168043</v>
       </c>
       <c r="R91" s="3">
-        <v>10380738.77481121</v>
+        <v>10367736.40888762</v>
       </c>
     </row>
     <row r="92" spans="1:18">
@@ -5680,46 +5680,46 @@
         <v>0</v>
       </c>
       <c r="E92" s="3">
-        <v>57453.76174088936</v>
+        <v>57452.1020101484</v>
       </c>
       <c r="F92" s="3">
-        <v>57725.95983959809</v>
+        <v>57715.06698039382</v>
       </c>
       <c r="G92" s="3">
-        <v>58029.61719015912</v>
+        <v>58003.92329925164</v>
       </c>
       <c r="H92" s="3">
-        <v>58402.17932397294</v>
+        <v>58357.83048055138</v>
       </c>
       <c r="I92" s="3">
-        <v>58919.68737305373</v>
+        <v>58857.03711334529</v>
       </c>
       <c r="J92" s="3">
-        <v>59594.25429564246</v>
+        <v>59516.23702996883</v>
       </c>
       <c r="K92" s="3">
-        <v>60424.54679375751</v>
+        <v>60334.32737498623</v>
       </c>
       <c r="L92" s="3">
-        <v>61377.02450449887</v>
+        <v>61277.22459609614</v>
       </c>
       <c r="M92" s="3">
-        <v>62424.13903836967</v>
+        <v>62316.75354938609</v>
       </c>
       <c r="N92" s="3">
-        <v>63568.65765965312</v>
+        <v>63455.10697140875</v>
       </c>
       <c r="O92" s="3">
-        <v>64784.56325905063</v>
+        <v>64665.84587845208</v>
       </c>
       <c r="P92" s="3">
-        <v>66045.99919042762</v>
+        <v>65922.83037368671</v>
       </c>
       <c r="Q92" s="3">
-        <v>67350.35014764602</v>
+        <v>67223.23229613119</v>
       </c>
       <c r="R92" s="3">
-        <v>796100.7403567191</v>
+        <v>795097.5179538066</v>
       </c>
     </row>
     <row r="93" spans="1:18">
@@ -5736,46 +5736,46 @@
         <v>0</v>
       </c>
       <c r="E93" s="3">
-        <v>393429.8258240776</v>
+        <v>393418.4603789521</v>
       </c>
       <c r="F93" s="3">
-        <v>395293.7742814057</v>
+        <v>395219.1825476425</v>
       </c>
       <c r="G93" s="3">
-        <v>397373.1482844555</v>
+        <v>397197.2025723183</v>
       </c>
       <c r="H93" s="3">
-        <v>399924.366011087</v>
+        <v>399620.6755787436</v>
       </c>
       <c r="I93" s="3">
-        <v>403468.1392200658</v>
+        <v>403039.1250003166</v>
       </c>
       <c r="J93" s="3">
-        <v>408087.4145959355</v>
+        <v>407553.1707393941</v>
       </c>
       <c r="K93" s="3">
-        <v>413773.0620282072</v>
+        <v>413155.2607017559</v>
       </c>
       <c r="L93" s="3">
-        <v>420295.4050129589</v>
+        <v>419611.9987504201</v>
       </c>
       <c r="M93" s="3">
-        <v>427465.7986685837</v>
+        <v>426730.4481371879</v>
       </c>
       <c r="N93" s="3">
-        <v>435303.192568999</v>
+        <v>434525.6242054222</v>
       </c>
       <c r="O93" s="3">
-        <v>443629.4276786668</v>
+        <v>442816.479022984</v>
       </c>
       <c r="P93" s="3">
-        <v>452267.4437759954</v>
+        <v>451424.0127342494</v>
       </c>
       <c r="Q93" s="3">
-        <v>461199.3318606477</v>
+        <v>460328.8587590575</v>
       </c>
       <c r="R93" s="3">
-        <v>5451510.329811086</v>
+        <v>5444640.499128445</v>
       </c>
     </row>
     <row r="94" spans="1:18">
@@ -5792,46 +5792,46 @@
         <v>0</v>
       </c>
       <c r="E94" s="3">
-        <v>1543312.449572583</v>
+        <v>1543267.866188696</v>
       </c>
       <c r="F94" s="3">
-        <v>1550624.185162356</v>
+        <v>1550331.583168822</v>
       </c>
       <c r="G94" s="3">
-        <v>1558780.973426952</v>
+        <v>1558090.788824345</v>
       </c>
       <c r="H94" s="3">
-        <v>1568788.669388573</v>
+        <v>1567597.378860281</v>
       </c>
       <c r="I94" s="3">
-        <v>1582689.876040669</v>
+        <v>1581006.976212229</v>
       </c>
       <c r="J94" s="3">
-        <v>1600809.969454155</v>
+        <v>1598714.283919433</v>
       </c>
       <c r="K94" s="3">
-        <v>1623113.134822276</v>
+        <v>1620689.677280699</v>
       </c>
       <c r="L94" s="3">
-        <v>1648698.417045517</v>
+        <v>1646017.610142068</v>
       </c>
       <c r="M94" s="3">
-        <v>1676825.816319029</v>
+        <v>1673941.246936101</v>
       </c>
       <c r="N94" s="3">
-        <v>1707569.666390334</v>
+        <v>1704519.488551407</v>
       </c>
       <c r="O94" s="3">
-        <v>1740231.100423464</v>
+        <v>1737042.135838609</v>
       </c>
       <c r="P94" s="3">
-        <v>1774115.561914638</v>
+        <v>1770807.023665521</v>
       </c>
       <c r="Q94" s="3">
-        <v>1809152.798988263</v>
+        <v>1805738.182488642</v>
       </c>
       <c r="R94" s="3">
-        <v>21384712.61894881</v>
+        <v>21357764.24207686</v>
       </c>
     </row>
     <row r="95" spans="1:18">
@@ -5848,46 +5848,46 @@
         <v>0</v>
       </c>
       <c r="E95" s="3">
-        <v>1879288.513655771</v>
+        <v>1879234.2245575</v>
       </c>
       <c r="F95" s="3">
-        <v>1888191.999604163</v>
+        <v>1887835.69873607</v>
       </c>
       <c r="G95" s="3">
-        <v>1898124.504521249</v>
+        <v>1897284.068097412</v>
       </c>
       <c r="H95" s="3">
-        <v>1910310.856075688</v>
+        <v>1908860.223958474</v>
       </c>
       <c r="I95" s="3">
-        <v>1927238.327887682</v>
+        <v>1925189.0640992</v>
       </c>
       <c r="J95" s="3">
-        <v>1949303.129754448</v>
+        <v>1946751.217628859</v>
       </c>
       <c r="K95" s="3">
-        <v>1976461.650056725</v>
+        <v>1973510.610607469</v>
       </c>
       <c r="L95" s="3">
-        <v>2007616.797553977</v>
+        <v>2004352.384296392</v>
       </c>
       <c r="M95" s="3">
-        <v>2041867.475949243</v>
+        <v>2038354.941523903</v>
       </c>
       <c r="N95" s="3">
-        <v>2079304.20129968</v>
+        <v>2075590.00578542</v>
       </c>
       <c r="O95" s="3">
-        <v>2119075.96484308</v>
+        <v>2115192.768983141</v>
       </c>
       <c r="P95" s="3">
-        <v>2160337.006500206</v>
+        <v>2156308.206026084</v>
       </c>
       <c r="Q95" s="3">
-        <v>2203001.780701264</v>
+        <v>2198843.808951568</v>
       </c>
       <c r="R95" s="3">
-        <v>26040122.20840318</v>
+        <v>26007307.22325149</v>
       </c>
     </row>
     <row r="96" spans="1:18">
@@ -5904,46 +5904,46 @@
         <v>0</v>
       </c>
       <c r="E96" s="3">
-        <v>908998.6845796451</v>
+        <v>908972.2539547763</v>
       </c>
       <c r="F96" s="3">
-        <v>915294.9786781769</v>
+        <v>915121.2966844005</v>
       </c>
       <c r="G96" s="3">
-        <v>922468.386868152</v>
+        <v>922057.7367133191</v>
       </c>
       <c r="H96" s="3">
-        <v>930881.897037754</v>
+        <v>930171.612620516</v>
       </c>
       <c r="I96" s="3">
-        <v>941056.1395606538</v>
+        <v>940051.7627487472</v>
       </c>
       <c r="J96" s="3">
-        <v>953257.8362255536</v>
+        <v>952006.4560553504</v>
       </c>
       <c r="K96" s="3">
-        <v>967577.0389411376</v>
+        <v>966129.5024224792</v>
       </c>
       <c r="L96" s="3">
-        <v>983575.3721824561</v>
+        <v>981973.8223003522</v>
       </c>
       <c r="M96" s="3">
-        <v>1000888.877358063</v>
+        <v>999165.3919996863</v>
       </c>
       <c r="N96" s="3">
-        <v>1019620.037697096</v>
+        <v>1017797.461840885</v>
       </c>
       <c r="O96" s="3">
-        <v>1039393.239308583</v>
+        <v>1037487.635222798</v>
       </c>
       <c r="P96" s="3">
-        <v>1059823.510857336</v>
+        <v>1057846.385061361</v>
       </c>
       <c r="Q96" s="3">
-        <v>1080890.320579508</v>
+        <v>1078849.755872553</v>
       </c>
       <c r="R96" s="3">
-        <v>12723726.31987412</v>
+        <v>12707631.07349722</v>
       </c>
     </row>
     <row r="97" spans="1:18">
@@ -5960,43 +5960,43 @@
         <v>0.3411657413950535</v>
       </c>
       <c r="E97" s="3">
-        <v>0.3405327737840404</v>
+        <v>0.3405340873450804</v>
       </c>
       <c r="F97" s="3">
-        <v>0.3390861359569305</v>
+        <v>0.3390804563325584</v>
       </c>
       <c r="G97" s="3">
-        <v>0.3367206064907633</v>
+        <v>0.3367079483137003</v>
       </c>
       <c r="H97" s="3">
-        <v>0.3354859927532072</v>
+        <v>0.3354624348694093</v>
       </c>
       <c r="I97" s="3">
-        <v>0.3344924328313715</v>
+        <v>0.3344596609879122</v>
       </c>
       <c r="J97" s="3">
-        <v>0.3337716185609467</v>
+        <v>0.333731885647425</v>
       </c>
       <c r="K97" s="3">
-        <v>0.3333907063170999</v>
+        <v>0.3333460278302761</v>
       </c>
       <c r="L97" s="3">
-        <v>0.3329389246615942</v>
+        <v>0.3328905003373809</v>
       </c>
       <c r="M97" s="3">
-        <v>0.3326971410058649</v>
+        <v>0.3326461907756119</v>
       </c>
       <c r="N97" s="3">
-        <v>0.3325633487689346</v>
+        <v>0.3325106449139235</v>
       </c>
       <c r="O97" s="3">
-        <v>0.332489429441744</v>
+        <v>0.3324355039623403</v>
       </c>
       <c r="P97" s="3">
-        <v>0.3323482025383582</v>
+        <v>0.3322933222827822</v>
       </c>
       <c r="Q97" s="3">
-        <v>0.3323412730054667</v>
+        <v>0.3322858514356819</v>
       </c>
       <c r="R97" s="3" t="s">
         <v>19</v>
@@ -6016,43 +6016,43 @@
         <v>0.04535037632743646</v>
       </c>
       <c r="E98" s="3">
-        <v>0.04471514483398276</v>
+        <v>0.04471402746527998</v>
       </c>
       <c r="F98" s="3">
-        <v>0.04469102236004265</v>
+        <v>0.04469100957032307</v>
       </c>
       <c r="G98" s="3">
-        <v>0.04452473753480909</v>
+        <v>0.04452614989542812</v>
       </c>
       <c r="H98" s="3">
-        <v>0.04460951990774174</v>
+        <v>0.04461341486476176</v>
       </c>
       <c r="I98" s="3">
-        <v>0.0447004800860787</v>
+        <v>0.04470671944286383</v>
       </c>
       <c r="J98" s="3">
-        <v>0.04477299864325959</v>
+        <v>0.04478109024917162</v>
       </c>
       <c r="K98" s="3">
-        <v>0.04479703586749677</v>
+        <v>0.04480646777677671</v>
       </c>
       <c r="L98" s="3">
-        <v>0.04485463655093411</v>
+        <v>0.04486507995002207</v>
       </c>
       <c r="M98" s="3">
-        <v>0.04488079854141676</v>
+        <v>0.0448919304391977</v>
       </c>
       <c r="N98" s="3">
-        <v>0.0448909440931286</v>
+        <v>0.04490255220605267</v>
       </c>
       <c r="O98" s="3">
-        <v>0.04489252477688747</v>
+        <v>0.0449044639418132</v>
       </c>
       <c r="P98" s="3">
-        <v>0.04491360991395767</v>
+        <v>0.04492580440248491</v>
       </c>
       <c r="Q98" s="3">
-        <v>0.04490877875029793</v>
+        <v>0.04492112281752544</v>
       </c>
       <c r="R98" s="3" t="s">
         <v>19</v>
@@ -6072,43 +6072,43 @@
         <v>0.2195512735036556</v>
       </c>
       <c r="E99" s="3">
-        <v>0.2116278167611485</v>
+        <v>0.2116161424393409</v>
       </c>
       <c r="F99" s="3">
-        <v>0.2095892577150464</v>
+        <v>0.2095722836169491</v>
       </c>
       <c r="G99" s="3">
-        <v>0.2043105720657347</v>
+        <v>0.204288277113638</v>
       </c>
       <c r="H99" s="3">
-        <v>0.204288072325831</v>
+        <v>0.2042630129326373</v>
       </c>
       <c r="I99" s="3">
-        <v>0.2042451564307447</v>
+        <v>0.2042191252206733</v>
       </c>
       <c r="J99" s="3">
-        <v>0.2042341716327887</v>
+        <v>0.2042078160950068</v>
       </c>
       <c r="K99" s="3">
-        <v>0.2042765101150407</v>
+        <v>0.2042500986589632</v>
       </c>
       <c r="L99" s="3">
-        <v>0.2042198329762524</v>
+        <v>0.2041933332112627</v>
       </c>
       <c r="M99" s="3">
-        <v>0.204239705527474</v>
+        <v>0.2042132152168388</v>
       </c>
       <c r="N99" s="3">
-        <v>0.2042542257453231</v>
+        <v>0.2042277467359465</v>
       </c>
       <c r="O99" s="3">
-        <v>0.2042636097369087</v>
+        <v>0.2042371459215793</v>
       </c>
       <c r="P99" s="3">
-        <v>0.2042345501550655</v>
+        <v>0.2042080550753823</v>
       </c>
       <c r="Q99" s="3">
-        <v>0.2042626701275111</v>
+        <v>0.2042362104067417</v>
       </c>
       <c r="R99" s="3" t="s">
         <v>19</v>
@@ -6408,43 +6408,43 @@
         <v>0</v>
       </c>
       <c r="E105" s="3">
-        <v>89.05713048520413</v>
+        <v>90.10106500007241</v>
       </c>
       <c r="F105" s="3">
-        <v>88.47526733516426</v>
+        <v>89.60175738342717</v>
       </c>
       <c r="G105" s="3">
-        <v>87.94539391007815</v>
+        <v>89.29526516520423</v>
       </c>
       <c r="H105" s="3">
-        <v>87.62061087357053</v>
+        <v>89.07878957346189</v>
       </c>
       <c r="I105" s="3">
-        <v>87.36144996004451</v>
+        <v>88.88203805564171</v>
       </c>
       <c r="J105" s="3">
-        <v>87.1563805505225</v>
+        <v>88.71750422811526</v>
       </c>
       <c r="K105" s="3">
-        <v>87.01388489219885</v>
+        <v>88.60433816803817</v>
       </c>
       <c r="L105" s="3">
-        <v>86.87070287638311</v>
+        <v>88.48176273341795</v>
       </c>
       <c r="M105" s="3">
-        <v>86.75938818838166</v>
+        <v>88.38662658686357</v>
       </c>
       <c r="N105" s="3">
-        <v>86.66970159602538</v>
+        <v>88.3099784572116</v>
       </c>
       <c r="O105" s="3">
-        <v>86.59704095555011</v>
+        <v>88.24802506705804</v>
       </c>
       <c r="P105" s="3">
-        <v>86.52621715543194</v>
+        <v>88.18567605075478</v>
       </c>
       <c r="Q105" s="3">
-        <v>86.47309754282645</v>
+        <v>88.14004468728503</v>
       </c>
       <c r="R105" s="3" t="s">
         <v>19</v>
@@ -6464,43 +6464,43 @@
         <v>0.01226890863757641</v>
       </c>
       <c r="E106" s="3">
-        <v>0.01199268792946653</v>
+        <v>0.01199305976851651</v>
       </c>
       <c r="F106" s="3">
-        <v>0.01200268483333958</v>
+        <v>0.01200384463315342</v>
       </c>
       <c r="G106" s="3">
-        <v>0.01194479880198366</v>
+        <v>0.01194700408937189</v>
       </c>
       <c r="H106" s="3">
-        <v>0.01197360945692622</v>
+        <v>0.01197683243829079</v>
       </c>
       <c r="I106" s="3">
-        <v>0.01200592741176612</v>
+        <v>0.01200997528556574</v>
       </c>
       <c r="J106" s="3">
-        <v>0.01202984588003761</v>
+        <v>0.01203450785177757</v>
       </c>
       <c r="K106" s="3">
-        <v>0.01203406437194114</v>
+        <v>0.01203915579402608</v>
       </c>
       <c r="L106" s="3">
-        <v>0.01205683008764843</v>
+        <v>0.01206224895183924</v>
       </c>
       <c r="M106" s="3">
-        <v>0.01206358402330606</v>
+        <v>0.01206922012767576</v>
       </c>
       <c r="N106" s="3">
-        <v>0.01206560654229435</v>
+        <v>0.01207139252957222</v>
       </c>
       <c r="O106" s="3">
-        <v>0.01206532978780221</v>
+        <v>0.01207121940973669</v>
       </c>
       <c r="P106" s="3">
-        <v>0.0120743396189716</v>
+        <v>0.01208031254997203</v>
       </c>
       <c r="Q106" s="3">
-        <v>0.01207057734796241</v>
+        <v>0.01207659481503813</v>
       </c>
       <c r="R106" s="3" t="s">
         <v>19</v>
@@ -6520,43 +6520,43 @@
         <v>0.03308146768986005</v>
       </c>
       <c r="E107" s="3">
-        <v>0.03272245690451623</v>
+        <v>0.03272096769676348</v>
       </c>
       <c r="F107" s="3">
-        <v>0.03268833752670306</v>
+        <v>0.03268716493716965</v>
       </c>
       <c r="G107" s="3">
-        <v>0.03257993873282544</v>
+        <v>0.03257914580605623</v>
       </c>
       <c r="H107" s="3">
-        <v>0.03263591045081552</v>
+        <v>0.03263658242647097</v>
       </c>
       <c r="I107" s="3">
-        <v>0.03269455267431257</v>
+        <v>0.03269674415729809</v>
       </c>
       <c r="J107" s="3">
-        <v>0.03274315276322199</v>
+        <v>0.03274658239739406</v>
       </c>
       <c r="K107" s="3">
-        <v>0.03276297149555564</v>
+        <v>0.03276731198275063</v>
       </c>
       <c r="L107" s="3">
-        <v>0.03279780646328567</v>
+        <v>0.03280283099818283</v>
       </c>
       <c r="M107" s="3">
-        <v>0.0328172145181107</v>
+        <v>0.03282271031152194</v>
       </c>
       <c r="N107" s="3">
-        <v>0.03282533755083425</v>
+        <v>0.03283115967648045</v>
       </c>
       <c r="O107" s="3">
-        <v>0.03282719498908527</v>
+        <v>0.03283324453207652</v>
       </c>
       <c r="P107" s="3">
-        <v>0.03283927029498607</v>
+        <v>0.03284549185251288</v>
       </c>
       <c r="Q107" s="3">
-        <v>0.03283820140233552</v>
+        <v>0.03284452800248731</v>
       </c>
       <c r="R107" s="3" t="s">
         <v>19</v>
@@ -6576,43 +6576,43 @@
         <v>121000.9090850509</v>
       </c>
       <c r="E108" s="3">
-        <v>118537.9688569864</v>
+        <v>118515.3972478842</v>
       </c>
       <c r="F108" s="3">
-        <v>119365.1925572382</v>
+        <v>119322.9843380517</v>
       </c>
       <c r="G108" s="3">
-        <v>119854.4396321737</v>
+        <v>119785.6941090304</v>
       </c>
       <c r="H108" s="3">
-        <v>121504.3546946129</v>
+        <v>121415.498128547</v>
       </c>
       <c r="I108" s="3">
-        <v>123544.2148965368</v>
+        <v>123440.1345344126</v>
       </c>
       <c r="J108" s="3">
-        <v>125786.9022825334</v>
+        <v>125671.0895509145</v>
       </c>
       <c r="K108" s="3">
-        <v>127930.6587318603</v>
+        <v>127805.6427784343</v>
       </c>
       <c r="L108" s="3">
-        <v>130558.2117107613</v>
+        <v>130425.8143769097</v>
       </c>
       <c r="M108" s="3">
-        <v>133143.760183863</v>
+        <v>133005.1718505112</v>
       </c>
       <c r="N108" s="3">
-        <v>135765.0577896846</v>
+        <v>135621.1481836558</v>
       </c>
       <c r="O108" s="3">
-        <v>138417.5628101268</v>
+        <v>138268.9633246042</v>
       </c>
       <c r="P108" s="3">
-        <v>141330.8484994144</v>
+        <v>141177.9788290449</v>
       </c>
       <c r="Q108" s="3">
-        <v>144114.3106878076</v>
+        <v>143957.4162737527</v>
       </c>
       <c r="R108" s="3" t="s">
         <v>19</v>
@@ -6632,43 +6632,43 @@
         <v>326262.7331074112</v>
       </c>
       <c r="E109" s="3">
-        <v>323434.8796770674</v>
+        <v>323348.5498919341</v>
       </c>
       <c r="F109" s="3">
-        <v>325081.4094870532</v>
+        <v>324923.4048798735</v>
       </c>
       <c r="G109" s="3">
-        <v>326908.0011146667</v>
+        <v>326652.23554493</v>
       </c>
       <c r="H109" s="3">
-        <v>331178.768896934</v>
+        <v>330854.3333924154</v>
       </c>
       <c r="I109" s="3">
-        <v>336435.7207076623</v>
+        <v>336061.5156689743</v>
       </c>
       <c r="J109" s="3">
-        <v>342370.118297525</v>
+        <v>341958.2038281238</v>
       </c>
       <c r="K109" s="3">
-        <v>348293.6766743845</v>
+        <v>347852.2449352287</v>
       </c>
       <c r="L109" s="3">
-        <v>355153.2972392905</v>
+        <v>354688.0821220139</v>
       </c>
       <c r="M109" s="3">
-        <v>362198.110549925</v>
+        <v>361712.7021797247</v>
       </c>
       <c r="N109" s="3">
-        <v>369358.4598447779</v>
+        <v>368855.5036726164</v>
       </c>
       <c r="O109" s="3">
-        <v>376604.7347396784</v>
+        <v>376086.1707452369</v>
       </c>
       <c r="P109" s="3">
-        <v>384385.5714973914</v>
+        <v>383852.6639275046</v>
       </c>
       <c r="Q109" s="3">
-        <v>392065.3190730637</v>
+        <v>391518.756933145</v>
       </c>
       <c r="R109" s="3" t="s">
         <v>19</v>
@@ -6856,46 +6856,46 @@
         <v>0</v>
       </c>
       <c r="E113" s="3">
-        <v>3030514.536511332</v>
+        <v>3028779.993334658</v>
       </c>
       <c r="F113" s="3">
-        <v>3036600.569721173</v>
+        <v>3033791.174338168</v>
       </c>
       <c r="G113" s="3">
-        <v>3072676.90400015</v>
+        <v>3068402.498074546</v>
       </c>
       <c r="H113" s="3">
-        <v>3121394.239347063</v>
+        <v>3116466.347938418</v>
       </c>
       <c r="I113" s="3">
-        <v>3178807.557529681</v>
+        <v>3173579.433077995</v>
       </c>
       <c r="J113" s="3">
-        <v>3243519.997025381</v>
+        <v>3238114.601871819</v>
       </c>
       <c r="K113" s="3">
-        <v>3307378.017961221</v>
+        <v>3301837.858392315</v>
       </c>
       <c r="L113" s="3">
-        <v>3374937.736303682</v>
+        <v>3369278.654315251</v>
       </c>
       <c r="M113" s="3">
-        <v>3447536.332650212</v>
+        <v>3441754.693268677</v>
       </c>
       <c r="N113" s="3">
-        <v>3518908.099756179</v>
+        <v>3513003.967916105</v>
       </c>
       <c r="O113" s="3">
-        <v>3589345.418096531</v>
+        <v>3583320.44104924</v>
       </c>
       <c r="P113" s="3">
-        <v>3663466.085394981</v>
+        <v>3657318.708322715</v>
       </c>
       <c r="Q113" s="3">
-        <v>3739029.037331283</v>
+        <v>3732754.019614305</v>
       </c>
       <c r="R113" s="3">
-        <v>43324114.53162886</v>
+        <v>43258402.39151421</v>
       </c>
     </row>
     <row r="114" spans="1:18">
@@ -6912,46 +6912,46 @@
         <v>9862402</v>
       </c>
       <c r="E114" s="3">
-        <v>9884186.89406015</v>
+        <v>9881998.383682199</v>
       </c>
       <c r="F114" s="3">
-        <v>9944874.352251612</v>
+        <v>9940397.263097983</v>
       </c>
       <c r="G114" s="3">
-        <v>10034027.49758075</v>
+        <v>10026421.11888053</v>
       </c>
       <c r="H114" s="3">
-        <v>10147679.78959994</v>
+        <v>10137529.99836359</v>
       </c>
       <c r="I114" s="3">
-        <v>10290268.35323527</v>
+        <v>10278133.93444446</v>
       </c>
       <c r="J114" s="3">
-        <v>10456235.56086158</v>
+        <v>10442561.59859102</v>
       </c>
       <c r="K114" s="3">
-        <v>10630710.85361202</v>
+        <v>10615830.95733776</v>
       </c>
       <c r="L114" s="3">
-        <v>10828568.60067316</v>
+        <v>10812727.78382032</v>
       </c>
       <c r="M114" s="3">
-        <v>11036832.82900321</v>
+        <v>11020196.03947059</v>
       </c>
       <c r="N114" s="3">
-        <v>11252236.45523154</v>
+        <v>11234921.55949815</v>
       </c>
       <c r="O114" s="3">
-        <v>11472339.77392512</v>
+        <v>11454432.11918391</v>
       </c>
       <c r="P114" s="3">
-        <v>11705058.24412547</v>
+        <v>11686616.40541509</v>
       </c>
       <c r="Q114" s="3">
-        <v>11939305.51400964</v>
+        <v>11920364.84444214</v>
       </c>
       <c r="R114" s="3">
-        <v>149484726.7181695</v>
+        <v>149314534.0062277</v>
       </c>
     </row>
     <row r="115" spans="1:18">
@@ -7096,46 +7096,46 @@
         <v>0</v>
       </c>
       <c r="E118" s="3">
-        <v>1175600.063393105</v>
+        <v>1175565.880896696</v>
       </c>
       <c r="F118" s="3">
-        <v>1183743.005585368</v>
+        <v>1183518.384179026</v>
       </c>
       <c r="G118" s="3">
-        <v>1193020.311775068</v>
+        <v>1192489.221514715</v>
       </c>
       <c r="H118" s="3">
-        <v>1203901.43102918</v>
+        <v>1202982.826393005</v>
       </c>
       <c r="I118" s="3">
-        <v>1217059.690064977</v>
+        <v>1215760.738302144</v>
       </c>
       <c r="J118" s="3">
-        <v>1232840.037843361</v>
+        <v>1231221.638793531</v>
       </c>
       <c r="K118" s="3">
-        <v>1251358.937711696</v>
+        <v>1249486.851368815</v>
       </c>
       <c r="L118" s="3">
-        <v>1272049.442430496</v>
+        <v>1269978.171949176</v>
       </c>
       <c r="M118" s="3">
-        <v>1294440.847530728</v>
+        <v>1292211.878962416</v>
       </c>
       <c r="N118" s="3">
-        <v>1318665.693677976</v>
+        <v>1316308.572233856</v>
       </c>
       <c r="O118" s="3">
-        <v>1344238.202706082</v>
+        <v>1341773.701577473</v>
       </c>
       <c r="P118" s="3">
-        <v>1370660.494547966</v>
+        <v>1368103.495015938</v>
       </c>
       <c r="Q118" s="3">
-        <v>1397906.015652684</v>
+        <v>1395266.971130894</v>
       </c>
       <c r="R118" s="3">
-        <v>16455484.17394869</v>
+        <v>16434668.33231769</v>
       </c>
     </row>
     <row r="119" spans="1:18">
@@ -7152,46 +7152,46 @@
         <v>0</v>
       </c>
       <c r="E119" s="3">
-        <v>191472.8305431889</v>
+        <v>193717.2897501557</v>
       </c>
       <c r="F119" s="3">
-        <v>193394.5823647756</v>
+        <v>196050.3548677525</v>
       </c>
       <c r="G119" s="3">
-        <v>194692.7329594506</v>
+        <v>198688.1528207878</v>
       </c>
       <c r="H119" s="3">
-        <v>197634.6725811554</v>
+        <v>201673.0660779111</v>
       </c>
       <c r="I119" s="3">
-        <v>201253.4211039281</v>
+        <v>205349.9627065802</v>
       </c>
       <c r="J119" s="3">
-        <v>205135.4083235969</v>
+        <v>209304.8811946179</v>
       </c>
       <c r="K119" s="3">
-        <v>208638.5103990861</v>
+        <v>212885.7032708055</v>
       </c>
       <c r="L119" s="3">
-        <v>213148.4308803786</v>
+        <v>217473.564624953</v>
       </c>
       <c r="M119" s="3">
-        <v>217444.1566823388</v>
+        <v>221860.04927644</v>
       </c>
       <c r="N119" s="3">
-        <v>221723.5148123398</v>
+        <v>226229.3672156177</v>
       </c>
       <c r="O119" s="3">
-        <v>226036.1532042855</v>
+        <v>230630.82545264</v>
       </c>
       <c r="P119" s="3">
-        <v>230898.5241090136</v>
+        <v>235584.677369059</v>
       </c>
       <c r="Q119" s="3">
-        <v>235400.59926692</v>
+        <v>240184.5197252505</v>
       </c>
       <c r="R119" s="3">
-        <v>2736873.537230458</v>
+        <v>2789632.414352571</v>
       </c>
     </row>
     <row r="120" spans="1:18">
@@ -7208,46 +7208,46 @@
         <v>0</v>
       </c>
       <c r="E120" s="3">
-        <v>761142.2120035558</v>
+        <v>761120.4456709523</v>
       </c>
       <c r="F120" s="3">
-        <v>762174.9538583929</v>
+        <v>762032.3815374386</v>
       </c>
       <c r="G120" s="3">
-        <v>763133.8099363408</v>
+        <v>762798.7698819487</v>
       </c>
       <c r="H120" s="3">
-        <v>764811.6043704802</v>
+        <v>764235.2280460199</v>
       </c>
       <c r="I120" s="3">
-        <v>769098.3251957578</v>
+        <v>768285.3629104018</v>
       </c>
       <c r="J120" s="3">
-        <v>776057.3462067296</v>
+        <v>775045.8158652957</v>
       </c>
       <c r="K120" s="3">
-        <v>785527.2591387869</v>
+        <v>784358.0866136401</v>
       </c>
       <c r="L120" s="3">
-        <v>796944.3796279803</v>
+        <v>795651.4369433123</v>
       </c>
       <c r="M120" s="3">
-        <v>809850.7674568847</v>
+        <v>808459.8161108734</v>
       </c>
       <c r="N120" s="3">
-        <v>824207.1652813572</v>
+        <v>822736.5405229733</v>
       </c>
       <c r="O120" s="3">
-        <v>839622.3253960484</v>
+        <v>838084.9132841204</v>
       </c>
       <c r="P120" s="3">
-        <v>855722.5111426678</v>
+        <v>854127.5413838323</v>
       </c>
       <c r="Q120" s="3">
-        <v>872446.1151962263</v>
+        <v>870800.0701168043</v>
       </c>
       <c r="R120" s="3">
-        <v>10380738.77481121</v>
+        <v>10367736.40888762</v>
       </c>
     </row>
     <row r="121" spans="1:18">
@@ -7264,46 +7264,46 @@
         <v>0</v>
       </c>
       <c r="E121" s="3">
-        <v>57453.76174088936</v>
+        <v>57452.1020101484</v>
       </c>
       <c r="F121" s="3">
-        <v>57725.95983959809</v>
+        <v>57715.06698039382</v>
       </c>
       <c r="G121" s="3">
-        <v>58029.61719015912</v>
+        <v>58003.92329925164</v>
       </c>
       <c r="H121" s="3">
-        <v>58402.17932397294</v>
+        <v>58357.83048055138</v>
       </c>
       <c r="I121" s="3">
-        <v>58919.68737305373</v>
+        <v>58857.03711334529</v>
       </c>
       <c r="J121" s="3">
-        <v>59594.25429564246</v>
+        <v>59516.23702996883</v>
       </c>
       <c r="K121" s="3">
-        <v>60424.54679375751</v>
+        <v>60334.32737498623</v>
       </c>
       <c r="L121" s="3">
-        <v>61377.02450449887</v>
+        <v>61277.22459609614</v>
       </c>
       <c r="M121" s="3">
-        <v>62424.13903836967</v>
+        <v>62316.75354938609</v>
       </c>
       <c r="N121" s="3">
-        <v>63568.65765965312</v>
+        <v>63455.10697140875</v>
       </c>
       <c r="O121" s="3">
-        <v>64784.56325905063</v>
+        <v>64665.84587845208</v>
       </c>
       <c r="P121" s="3">
-        <v>66045.99919042762</v>
+        <v>65922.83037368671</v>
       </c>
       <c r="Q121" s="3">
-        <v>67350.35014764602</v>
+        <v>67223.23229613119</v>
       </c>
       <c r="R121" s="3">
-        <v>796100.7403567191</v>
+        <v>795097.5179538066</v>
       </c>
     </row>
     <row r="122" spans="1:18">
@@ -7320,46 +7320,46 @@
         <v>0</v>
       </c>
       <c r="E122" s="3">
-        <v>393429.8258240776</v>
+        <v>393418.4603789521</v>
       </c>
       <c r="F122" s="3">
-        <v>395293.7742814057</v>
+        <v>395219.1825476425</v>
       </c>
       <c r="G122" s="3">
-        <v>397373.1482844555</v>
+        <v>397197.2025723183</v>
       </c>
       <c r="H122" s="3">
-        <v>399924.366011087</v>
+        <v>399620.6755787436</v>
       </c>
       <c r="I122" s="3">
-        <v>403468.1392200658</v>
+        <v>403039.1250003166</v>
       </c>
       <c r="J122" s="3">
-        <v>408087.4145959355</v>
+        <v>407553.1707393941</v>
       </c>
       <c r="K122" s="3">
-        <v>413773.0620282072</v>
+        <v>413155.2607017559</v>
       </c>
       <c r="L122" s="3">
-        <v>420295.4050129589</v>
+        <v>419611.9987504201</v>
       </c>
       <c r="M122" s="3">
-        <v>427465.7986685837</v>
+        <v>426730.4481371879</v>
       </c>
       <c r="N122" s="3">
-        <v>435303.192568999</v>
+        <v>434525.6242054222</v>
       </c>
       <c r="O122" s="3">
-        <v>443629.4276786668</v>
+        <v>442816.479022984</v>
       </c>
       <c r="P122" s="3">
-        <v>452267.4437759954</v>
+        <v>451424.0127342494</v>
       </c>
       <c r="Q122" s="3">
-        <v>461199.3318606477</v>
+        <v>460328.8587590575</v>
       </c>
       <c r="R122" s="3">
-        <v>5451510.329811086</v>
+        <v>5444640.499128445</v>
       </c>
     </row>
     <row r="123" spans="1:18">
@@ -7376,46 +7376,46 @@
         <v>0</v>
       </c>
       <c r="E123" s="3">
-        <v>1543312.449572583</v>
+        <v>1543267.866188696</v>
       </c>
       <c r="F123" s="3">
-        <v>1550624.185162356</v>
+        <v>1550331.583168822</v>
       </c>
       <c r="G123" s="3">
-        <v>1558780.973426952</v>
+        <v>1558090.788824345</v>
       </c>
       <c r="H123" s="3">
-        <v>1568788.669388573</v>
+        <v>1567597.378860281</v>
       </c>
       <c r="I123" s="3">
-        <v>1582689.876040669</v>
+        <v>1581006.976212229</v>
       </c>
       <c r="J123" s="3">
-        <v>1600809.969454155</v>
+        <v>1598714.283919433</v>
       </c>
       <c r="K123" s="3">
-        <v>1623113.134822276</v>
+        <v>1620689.677280699</v>
       </c>
       <c r="L123" s="3">
-        <v>1648698.417045517</v>
+        <v>1646017.610142068</v>
       </c>
       <c r="M123" s="3">
-        <v>1676825.816319029</v>
+        <v>1673941.246936101</v>
       </c>
       <c r="N123" s="3">
-        <v>1707569.666390334</v>
+        <v>1704519.488551407</v>
       </c>
       <c r="O123" s="3">
-        <v>1740231.100423464</v>
+        <v>1737042.135838609</v>
       </c>
       <c r="P123" s="3">
-        <v>1774115.561914638</v>
+        <v>1770807.023665521</v>
       </c>
       <c r="Q123" s="3">
-        <v>1809152.798988263</v>
+        <v>1805738.182488642</v>
       </c>
       <c r="R123" s="3">
-        <v>21384712.61894881</v>
+        <v>21357764.24207686</v>
       </c>
     </row>
     <row r="124" spans="1:18">
@@ -7432,46 +7432,46 @@
         <v>0</v>
       </c>
       <c r="E124" s="3">
-        <v>1879288.513655771</v>
+        <v>1879234.2245575</v>
       </c>
       <c r="F124" s="3">
-        <v>1888191.999604163</v>
+        <v>1887835.69873607</v>
       </c>
       <c r="G124" s="3">
-        <v>1898124.504521249</v>
+        <v>1897284.068097412</v>
       </c>
       <c r="H124" s="3">
-        <v>1910310.856075688</v>
+        <v>1908860.223958474</v>
       </c>
       <c r="I124" s="3">
-        <v>1927238.327887682</v>
+        <v>1925189.0640992</v>
       </c>
       <c r="J124" s="3">
-        <v>1949303.129754448</v>
+        <v>1946751.217628859</v>
       </c>
       <c r="K124" s="3">
-        <v>1976461.650056725</v>
+        <v>1973510.610607469</v>
       </c>
       <c r="L124" s="3">
-        <v>2007616.797553977</v>
+        <v>2004352.384296392</v>
       </c>
       <c r="M124" s="3">
-        <v>2041867.475949243</v>
+        <v>2038354.941523903</v>
       </c>
       <c r="N124" s="3">
-        <v>2079304.20129968</v>
+        <v>2075590.00578542</v>
       </c>
       <c r="O124" s="3">
-        <v>2119075.96484308</v>
+        <v>2115192.768983141</v>
       </c>
       <c r="P124" s="3">
-        <v>2160337.006500206</v>
+        <v>2156308.206026084</v>
       </c>
       <c r="Q124" s="3">
-        <v>2203001.780701264</v>
+        <v>2198843.808951568</v>
       </c>
       <c r="R124" s="3">
-        <v>26040122.20840318</v>
+        <v>26007307.22325149</v>
       </c>
     </row>
     <row r="125" spans="1:18">
@@ -7488,46 +7488,46 @@
         <v>0</v>
       </c>
       <c r="E125" s="3">
-        <v>908998.6845796451</v>
+        <v>908972.2539547763</v>
       </c>
       <c r="F125" s="3">
-        <v>915294.9786781769</v>
+        <v>915121.2966844005</v>
       </c>
       <c r="G125" s="3">
-        <v>922468.386868152</v>
+        <v>922057.7367133191</v>
       </c>
       <c r="H125" s="3">
-        <v>930881.897037754</v>
+        <v>930171.612620516</v>
       </c>
       <c r="I125" s="3">
-        <v>941056.1395606538</v>
+        <v>940051.7627487472</v>
       </c>
       <c r="J125" s="3">
-        <v>953257.8362255536</v>
+        <v>952006.4560553504</v>
       </c>
       <c r="K125" s="3">
-        <v>967577.0389411376</v>
+        <v>966129.5024224792</v>
       </c>
       <c r="L125" s="3">
-        <v>983575.3721824561</v>
+        <v>981973.8223003522</v>
       </c>
       <c r="M125" s="3">
-        <v>1000888.877358063</v>
+        <v>999165.3919996863</v>
       </c>
       <c r="N125" s="3">
-        <v>1019620.037697096</v>
+        <v>1017797.461840885</v>
       </c>
       <c r="O125" s="3">
-        <v>1039393.239308583</v>
+        <v>1037487.635222798</v>
       </c>
       <c r="P125" s="3">
-        <v>1059823.510857336</v>
+        <v>1057846.385061361</v>
       </c>
       <c r="Q125" s="3">
-        <v>1080890.320579508</v>
+        <v>1078849.755872553</v>
       </c>
       <c r="R125" s="3">
-        <v>12723726.31987412</v>
+        <v>12707631.07349722</v>
       </c>
     </row>
     <row r="126" spans="1:18">
@@ -7544,43 +7544,43 @@
         <v>0.3411657413950535</v>
       </c>
       <c r="E126" s="3">
-        <v>0.3405327737840404</v>
+        <v>0.3405340873450804</v>
       </c>
       <c r="F126" s="3">
-        <v>0.3390861359569305</v>
+        <v>0.3390804563325584</v>
       </c>
       <c r="G126" s="3">
-        <v>0.3367206064907633</v>
+        <v>0.3367079483137003</v>
       </c>
       <c r="H126" s="3">
-        <v>0.3354859927532072</v>
+        <v>0.3354624348694093</v>
       </c>
       <c r="I126" s="3">
-        <v>0.3344924328313715</v>
+        <v>0.3344596609879122</v>
       </c>
       <c r="J126" s="3">
-        <v>0.3337716185609467</v>
+        <v>0.333731885647425</v>
       </c>
       <c r="K126" s="3">
-        <v>0.3333907063170999</v>
+        <v>0.3333460278302761</v>
       </c>
       <c r="L126" s="3">
-        <v>0.3329389246615942</v>
+        <v>0.3328905003373809</v>
       </c>
       <c r="M126" s="3">
-        <v>0.3326971410058649</v>
+        <v>0.3326461907756119</v>
       </c>
       <c r="N126" s="3">
-        <v>0.3325633487689346</v>
+        <v>0.3325106449139235</v>
       </c>
       <c r="O126" s="3">
-        <v>0.332489429441744</v>
+        <v>0.3324355039623403</v>
       </c>
       <c r="P126" s="3">
-        <v>0.3323482025383582</v>
+        <v>0.3322933222827822</v>
       </c>
       <c r="Q126" s="3">
-        <v>0.3323412730054667</v>
+        <v>0.3322858514356819</v>
       </c>
       <c r="R126" s="3" t="s">
         <v>19</v>
@@ -7600,43 +7600,43 @@
         <v>0.04535037632743646</v>
       </c>
       <c r="E127" s="3">
-        <v>0.04471514483398276</v>
+        <v>0.04471402746527998</v>
       </c>
       <c r="F127" s="3">
-        <v>0.04469102236004265</v>
+        <v>0.04469100957032307</v>
       </c>
       <c r="G127" s="3">
-        <v>0.04452473753480909</v>
+        <v>0.04452614989542812</v>
       </c>
       <c r="H127" s="3">
-        <v>0.04460951990774174</v>
+        <v>0.04461341486476176</v>
       </c>
       <c r="I127" s="3">
-        <v>0.0447004800860787</v>
+        <v>0.04470671944286383</v>
       </c>
       <c r="J127" s="3">
-        <v>0.04477299864325959</v>
+        <v>0.04478109024917162</v>
       </c>
       <c r="K127" s="3">
-        <v>0.04479703586749677</v>
+        <v>0.04480646777677671</v>
       </c>
       <c r="L127" s="3">
-        <v>0.04485463655093411</v>
+        <v>0.04486507995002207</v>
       </c>
       <c r="M127" s="3">
-        <v>0.04488079854141676</v>
+        <v>0.0448919304391977</v>
       </c>
       <c r="N127" s="3">
-        <v>0.0448909440931286</v>
+        <v>0.04490255220605267</v>
       </c>
       <c r="O127" s="3">
-        <v>0.04489252477688747</v>
+        <v>0.0449044639418132</v>
       </c>
       <c r="P127" s="3">
-        <v>0.04491360991395767</v>
+        <v>0.04492580440248491</v>
       </c>
       <c r="Q127" s="3">
-        <v>0.04490877875029793</v>
+        <v>0.04492112281752544</v>
       </c>
       <c r="R127" s="3" t="s">
         <v>19</v>
@@ -7656,43 +7656,43 @@
         <v>0.2195512735036556</v>
       </c>
       <c r="E128" s="3">
-        <v>0.2116278167611485</v>
+        <v>0.2116161424393409</v>
       </c>
       <c r="F128" s="3">
-        <v>0.2095892577150464</v>
+        <v>0.2095722836169491</v>
       </c>
       <c r="G128" s="3">
-        <v>0.2043105720657347</v>
+        <v>0.204288277113638</v>
       </c>
       <c r="H128" s="3">
-        <v>0.204288072325831</v>
+        <v>0.2042630129326373</v>
       </c>
       <c r="I128" s="3">
-        <v>0.2042451564307447</v>
+        <v>0.2042191252206733</v>
       </c>
       <c r="J128" s="3">
-        <v>0.2042341716327887</v>
+        <v>0.2042078160950068</v>
       </c>
       <c r="K128" s="3">
-        <v>0.2042765101150407</v>
+        <v>0.2042500986589632</v>
       </c>
       <c r="L128" s="3">
-        <v>0.2042198329762524</v>
+        <v>0.2041933332112627</v>
       </c>
       <c r="M128" s="3">
-        <v>0.204239705527474</v>
+        <v>0.2042132152168388</v>
       </c>
       <c r="N128" s="3">
-        <v>0.2042542257453231</v>
+        <v>0.2042277467359465</v>
       </c>
       <c r="O128" s="3">
-        <v>0.2042636097369087</v>
+        <v>0.2042371459215793</v>
       </c>
       <c r="P128" s="3">
-        <v>0.2042345501550655</v>
+        <v>0.2042080550753823</v>
       </c>
       <c r="Q128" s="3">
-        <v>0.2042626701275111</v>
+        <v>0.2042362104067417</v>
       </c>
       <c r="R128" s="3" t="s">
         <v>19</v>
@@ -7992,43 +7992,43 @@
         <v>0</v>
       </c>
       <c r="E134" s="3">
-        <v>89.05713048520413</v>
+        <v>90.10106500007241</v>
       </c>
       <c r="F134" s="3">
-        <v>88.47526733516426</v>
+        <v>89.60175738342717</v>
       </c>
       <c r="G134" s="3">
-        <v>87.94539391007815</v>
+        <v>89.29526516520423</v>
       </c>
       <c r="H134" s="3">
-        <v>87.62061087357053</v>
+        <v>89.07878957346189</v>
       </c>
       <c r="I134" s="3">
-        <v>87.36144996004451</v>
+        <v>88.88203805564171</v>
       </c>
       <c r="J134" s="3">
-        <v>87.1563805505225</v>
+        <v>88.71750422811526</v>
       </c>
       <c r="K134" s="3">
-        <v>87.01388489219885</v>
+        <v>88.60433816803817</v>
       </c>
       <c r="L134" s="3">
-        <v>86.87070287638311</v>
+        <v>88.48176273341795</v>
       </c>
       <c r="M134" s="3">
-        <v>86.75938818838166</v>
+        <v>88.38662658686357</v>
       </c>
       <c r="N134" s="3">
-        <v>86.66970159602538</v>
+        <v>88.3099784572116</v>
       </c>
       <c r="O134" s="3">
-        <v>86.59704095555011</v>
+        <v>88.24802506705804</v>
       </c>
       <c r="P134" s="3">
-        <v>86.52621715543194</v>
+        <v>88.18567605075478</v>
       </c>
       <c r="Q134" s="3">
-        <v>86.47309754282645</v>
+        <v>88.14004468728503</v>
       </c>
       <c r="R134" s="3" t="s">
         <v>19</v>
@@ -8048,43 +8048,43 @@
         <v>0.01226890863757641</v>
       </c>
       <c r="E135" s="3">
-        <v>0.01199268792946653</v>
+        <v>0.01199305976851651</v>
       </c>
       <c r="F135" s="3">
-        <v>0.01200268483333958</v>
+        <v>0.01200384463315342</v>
       </c>
       <c r="G135" s="3">
-        <v>0.01194479880198366</v>
+        <v>0.01194700408937189</v>
       </c>
       <c r="H135" s="3">
-        <v>0.01197360945692622</v>
+        <v>0.01197683243829079</v>
       </c>
       <c r="I135" s="3">
-        <v>0.01200592741176612</v>
+        <v>0.01200997528556574</v>
       </c>
       <c r="J135" s="3">
-        <v>0.01202984588003761</v>
+        <v>0.01203450785177757</v>
       </c>
       <c r="K135" s="3">
-        <v>0.01203406437194114</v>
+        <v>0.01203915579402608</v>
       </c>
       <c r="L135" s="3">
-        <v>0.01205683008764843</v>
+        <v>0.01206224895183924</v>
       </c>
       <c r="M135" s="3">
-        <v>0.01206358402330606</v>
+        <v>0.01206922012767576</v>
       </c>
       <c r="N135" s="3">
-        <v>0.01206560654229435</v>
+        <v>0.01207139252957222</v>
       </c>
       <c r="O135" s="3">
-        <v>0.01206532978780221</v>
+        <v>0.01207121940973669</v>
       </c>
       <c r="P135" s="3">
-        <v>0.0120743396189716</v>
+        <v>0.01208031254997203</v>
       </c>
       <c r="Q135" s="3">
-        <v>0.01207057734796241</v>
+        <v>0.01207659481503813</v>
       </c>
       <c r="R135" s="3" t="s">
         <v>19</v>
@@ -8104,43 +8104,43 @@
         <v>0.03308146768986005</v>
       </c>
       <c r="E136" s="3">
-        <v>0.03272245690451623</v>
+        <v>0.03272096769676348</v>
       </c>
       <c r="F136" s="3">
-        <v>0.03268833752670306</v>
+        <v>0.03268716493716965</v>
       </c>
       <c r="G136" s="3">
-        <v>0.03257993873282544</v>
+        <v>0.03257914580605623</v>
       </c>
       <c r="H136" s="3">
-        <v>0.03263591045081552</v>
+        <v>0.03263658242647097</v>
       </c>
       <c r="I136" s="3">
-        <v>0.03269455267431257</v>
+        <v>0.03269674415729809</v>
       </c>
       <c r="J136" s="3">
-        <v>0.03274315276322199</v>
+        <v>0.03274658239739406</v>
       </c>
       <c r="K136" s="3">
-        <v>0.03276297149555564</v>
+        <v>0.03276731198275063</v>
       </c>
       <c r="L136" s="3">
-        <v>0.03279780646328567</v>
+        <v>0.03280283099818283</v>
       </c>
       <c r="M136" s="3">
-        <v>0.0328172145181107</v>
+        <v>0.03282271031152194</v>
       </c>
       <c r="N136" s="3">
-        <v>0.03282533755083425</v>
+        <v>0.03283115967648045</v>
       </c>
       <c r="O136" s="3">
-        <v>0.03282719498908527</v>
+        <v>0.03283324453207652</v>
       </c>
       <c r="P136" s="3">
-        <v>0.03283927029498607</v>
+        <v>0.03284549185251288</v>
       </c>
       <c r="Q136" s="3">
-        <v>0.03283820140233552</v>
+        <v>0.03284452800248731</v>
       </c>
       <c r="R136" s="3" t="s">
         <v>19</v>
@@ -8160,43 +8160,43 @@
         <v>121000.9090850509</v>
       </c>
       <c r="E137" s="3">
-        <v>118537.9688569864</v>
+        <v>118515.3972478842</v>
       </c>
       <c r="F137" s="3">
-        <v>119365.1925572382</v>
+        <v>119322.9843380517</v>
       </c>
       <c r="G137" s="3">
-        <v>119854.4396321737</v>
+        <v>119785.6941090304</v>
       </c>
       <c r="H137" s="3">
-        <v>121504.3546946129</v>
+        <v>121415.498128547</v>
       </c>
       <c r="I137" s="3">
-        <v>123544.2148965368</v>
+        <v>123440.1345344126</v>
       </c>
       <c r="J137" s="3">
-        <v>125786.9022825334</v>
+        <v>125671.0895509145</v>
       </c>
       <c r="K137" s="3">
-        <v>127930.6587318603</v>
+        <v>127805.6427784343</v>
       </c>
       <c r="L137" s="3">
-        <v>130558.2117107613</v>
+        <v>130425.8143769097</v>
       </c>
       <c r="M137" s="3">
-        <v>133143.760183863</v>
+        <v>133005.1718505112</v>
       </c>
       <c r="N137" s="3">
-        <v>135765.0577896846</v>
+        <v>135621.1481836558</v>
       </c>
       <c r="O137" s="3">
-        <v>138417.5628101268</v>
+        <v>138268.9633246042</v>
       </c>
       <c r="P137" s="3">
-        <v>141330.8484994144</v>
+        <v>141177.9788290449</v>
       </c>
       <c r="Q137" s="3">
-        <v>144114.3106878076</v>
+        <v>143957.4162737527</v>
       </c>
       <c r="R137" s="3" t="s">
         <v>19</v>
@@ -8216,43 +8216,43 @@
         <v>326262.7331074112</v>
       </c>
       <c r="E138" s="3">
-        <v>323434.8796770674</v>
+        <v>323348.5498919341</v>
       </c>
       <c r="F138" s="3">
-        <v>325081.4094870532</v>
+        <v>324923.4048798735</v>
       </c>
       <c r="G138" s="3">
-        <v>326908.0011146667</v>
+        <v>326652.23554493</v>
       </c>
       <c r="H138" s="3">
-        <v>331178.768896934</v>
+        <v>330854.3333924154</v>
       </c>
       <c r="I138" s="3">
-        <v>336435.7207076623</v>
+        <v>336061.5156689743</v>
       </c>
       <c r="J138" s="3">
-        <v>342370.118297525</v>
+        <v>341958.2038281238</v>
       </c>
       <c r="K138" s="3">
-        <v>348293.6766743845</v>
+        <v>347852.2449352287</v>
       </c>
       <c r="L138" s="3">
-        <v>355153.2972392905</v>
+        <v>354688.0821220139</v>
       </c>
       <c r="M138" s="3">
-        <v>362198.110549925</v>
+        <v>361712.7021797247</v>
       </c>
       <c r="N138" s="3">
-        <v>369358.4598447779</v>
+        <v>368855.5036726164</v>
       </c>
       <c r="O138" s="3">
-        <v>376604.7347396784</v>
+        <v>376086.1707452369</v>
       </c>
       <c r="P138" s="3">
-        <v>384385.5714973914</v>
+        <v>383852.6639275046</v>
       </c>
       <c r="Q138" s="3">
-        <v>392065.3190730637</v>
+        <v>391518.756933145</v>
       </c>
       <c r="R138" s="3" t="s">
         <v>19</v>
@@ -8440,46 +8440,46 @@
         <v>0</v>
       </c>
       <c r="E142" s="3">
-        <v>3030514.536511332</v>
+        <v>3028779.993334658</v>
       </c>
       <c r="F142" s="3">
-        <v>3036600.569721173</v>
+        <v>3033791.174338168</v>
       </c>
       <c r="G142" s="3">
-        <v>3072676.90400015</v>
+        <v>3068402.498074546</v>
       </c>
       <c r="H142" s="3">
-        <v>3121394.239347063</v>
+        <v>3116466.347938418</v>
       </c>
       <c r="I142" s="3">
-        <v>3178807.557529681</v>
+        <v>3173579.433077995</v>
       </c>
       <c r="J142" s="3">
-        <v>3243519.997025381</v>
+        <v>3238114.601871819</v>
       </c>
       <c r="K142" s="3">
-        <v>3307378.017961221</v>
+        <v>3301837.858392315</v>
       </c>
       <c r="L142" s="3">
-        <v>3374937.736303682</v>
+        <v>3369278.654315251</v>
       </c>
       <c r="M142" s="3">
-        <v>3447536.332650212</v>
+        <v>3441754.693268677</v>
       </c>
       <c r="N142" s="3">
-        <v>3518908.099756179</v>
+        <v>3513003.967916105</v>
       </c>
       <c r="O142" s="3">
-        <v>3589345.418096531</v>
+        <v>3583320.44104924</v>
       </c>
       <c r="P142" s="3">
-        <v>3663466.085394981</v>
+        <v>3657318.708322715</v>
       </c>
       <c r="Q142" s="3">
-        <v>3739029.037331283</v>
+        <v>3732754.019614305</v>
       </c>
       <c r="R142" s="3">
-        <v>43324114.53162886</v>
+        <v>43258402.39151421</v>
       </c>
     </row>
     <row r="143" spans="1:18">
@@ -8496,46 +8496,46 @@
         <v>9862402</v>
       </c>
       <c r="E143" s="3">
-        <v>9884186.89406015</v>
+        <v>9881998.383682199</v>
       </c>
       <c r="F143" s="3">
-        <v>9944874.352251612</v>
+        <v>9940397.263097983</v>
       </c>
       <c r="G143" s="3">
-        <v>10034027.49758075</v>
+        <v>10026421.11888053</v>
       </c>
       <c r="H143" s="3">
-        <v>10147679.78959994</v>
+        <v>10137529.99836359</v>
       </c>
       <c r="I143" s="3">
-        <v>10290268.35323527</v>
+        <v>10278133.93444446</v>
       </c>
       <c r="J143" s="3">
-        <v>10456235.56086158</v>
+        <v>10442561.59859102</v>
       </c>
       <c r="K143" s="3">
-        <v>10630710.85361202</v>
+        <v>10615830.95733776</v>
       </c>
       <c r="L143" s="3">
-        <v>10828568.60067316</v>
+        <v>10812727.78382032</v>
       </c>
       <c r="M143" s="3">
-        <v>11036832.82900321</v>
+        <v>11020196.03947059</v>
       </c>
       <c r="N143" s="3">
-        <v>11252236.45523154</v>
+        <v>11234921.55949815</v>
       </c>
       <c r="O143" s="3">
-        <v>11472339.77392512</v>
+        <v>11454432.11918391</v>
       </c>
       <c r="P143" s="3">
-        <v>11705058.24412547</v>
+        <v>11686616.40541509</v>
       </c>
       <c r="Q143" s="3">
-        <v>11939305.51400964</v>
+        <v>11920364.84444214</v>
       </c>
       <c r="R143" s="3">
-        <v>149484726.7181695</v>
+        <v>149314534.0062277</v>
       </c>
     </row>
     <row r="144" spans="1:18">
@@ -8680,46 +8680,46 @@
         <v>0</v>
       </c>
       <c r="E147" s="3">
-        <v>1175600.063393105</v>
+        <v>1175565.880896696</v>
       </c>
       <c r="F147" s="3">
-        <v>1183743.005585368</v>
+        <v>1183518.384179026</v>
       </c>
       <c r="G147" s="3">
-        <v>1193020.311775068</v>
+        <v>1192489.221514715</v>
       </c>
       <c r="H147" s="3">
-        <v>1203901.43102918</v>
+        <v>1202982.826393005</v>
       </c>
       <c r="I147" s="3">
-        <v>1217059.690064977</v>
+        <v>1215760.738302144</v>
       </c>
       <c r="J147" s="3">
-        <v>1232840.037843361</v>
+        <v>1231221.638793531</v>
       </c>
       <c r="K147" s="3">
-        <v>1251358.937711696</v>
+        <v>1249486.851368815</v>
       </c>
       <c r="L147" s="3">
-        <v>1272049.442430496</v>
+        <v>1269978.171949176</v>
       </c>
       <c r="M147" s="3">
-        <v>1294440.847530728</v>
+        <v>1292211.878962416</v>
       </c>
       <c r="N147" s="3">
-        <v>1318665.693677976</v>
+        <v>1316308.572233856</v>
       </c>
       <c r="O147" s="3">
-        <v>1344238.202706082</v>
+        <v>1341773.701577473</v>
       </c>
       <c r="P147" s="3">
-        <v>1370660.494547966</v>
+        <v>1368103.495015938</v>
       </c>
       <c r="Q147" s="3">
-        <v>1397906.015652684</v>
+        <v>1395266.971130894</v>
       </c>
       <c r="R147" s="3">
-        <v>16455484.17394869</v>
+        <v>16434668.33231769</v>
       </c>
     </row>
     <row r="148" spans="1:18">
@@ -8736,46 +8736,46 @@
         <v>0</v>
       </c>
       <c r="E148" s="3">
-        <v>191472.8305431889</v>
+        <v>193717.2897501557</v>
       </c>
       <c r="F148" s="3">
-        <v>193394.5823647756</v>
+        <v>196050.3548677525</v>
       </c>
       <c r="G148" s="3">
-        <v>194692.7329594506</v>
+        <v>198688.1528207878</v>
       </c>
       <c r="H148" s="3">
-        <v>197634.6725811554</v>
+        <v>201673.0660779111</v>
       </c>
       <c r="I148" s="3">
-        <v>201253.4211039281</v>
+        <v>205349.9627065802</v>
       </c>
       <c r="J148" s="3">
-        <v>205135.4083235969</v>
+        <v>209304.8811946179</v>
       </c>
       <c r="K148" s="3">
-        <v>208638.5103990861</v>
+        <v>212885.7032708055</v>
       </c>
       <c r="L148" s="3">
-        <v>213148.4308803786</v>
+        <v>217473.564624953</v>
       </c>
       <c r="M148" s="3">
-        <v>217444.1566823388</v>
+        <v>221860.04927644</v>
       </c>
       <c r="N148" s="3">
-        <v>221723.5148123398</v>
+        <v>226229.3672156177</v>
       </c>
       <c r="O148" s="3">
-        <v>226036.1532042855</v>
+        <v>230630.82545264</v>
       </c>
       <c r="P148" s="3">
-        <v>230898.5241090136</v>
+        <v>235584.677369059</v>
       </c>
       <c r="Q148" s="3">
-        <v>235400.59926692</v>
+        <v>240184.5197252505</v>
       </c>
       <c r="R148" s="3">
-        <v>2736873.537230458</v>
+        <v>2789632.414352571</v>
       </c>
     </row>
     <row r="149" spans="1:18">
@@ -8792,46 +8792,46 @@
         <v>0</v>
       </c>
       <c r="E149" s="3">
-        <v>761142.2120035558</v>
+        <v>761120.4456709523</v>
       </c>
       <c r="F149" s="3">
-        <v>762174.9538583929</v>
+        <v>762032.3815374386</v>
       </c>
       <c r="G149" s="3">
-        <v>763133.8099363408</v>
+        <v>762798.7698819487</v>
       </c>
       <c r="H149" s="3">
-        <v>764811.6043704802</v>
+        <v>764235.2280460199</v>
       </c>
       <c r="I149" s="3">
-        <v>769098.3251957578</v>
+        <v>768285.3629104018</v>
       </c>
       <c r="J149" s="3">
-        <v>776057.3462067296</v>
+        <v>775045.8158652957</v>
       </c>
       <c r="K149" s="3">
-        <v>785527.2591387869</v>
+        <v>784358.0866136401</v>
       </c>
       <c r="L149" s="3">
-        <v>796944.3796279803</v>
+        <v>795651.4369433123</v>
       </c>
       <c r="M149" s="3">
-        <v>809850.7674568847</v>
+        <v>808459.8161108734</v>
       </c>
       <c r="N149" s="3">
-        <v>824207.1652813572</v>
+        <v>822736.5405229733</v>
       </c>
       <c r="O149" s="3">
-        <v>839622.3253960484</v>
+        <v>838084.9132841204</v>
       </c>
       <c r="P149" s="3">
-        <v>855722.5111426678</v>
+        <v>854127.5413838323</v>
       </c>
       <c r="Q149" s="3">
-        <v>872446.1151962263</v>
+        <v>870800.0701168043</v>
       </c>
       <c r="R149" s="3">
-        <v>10380738.77481121</v>
+        <v>10367736.40888762</v>
       </c>
     </row>
     <row r="150" spans="1:18">
@@ -8848,46 +8848,46 @@
         <v>0</v>
       </c>
       <c r="E150" s="3">
-        <v>57453.76174088936</v>
+        <v>57452.1020101484</v>
       </c>
       <c r="F150" s="3">
-        <v>57725.95983959809</v>
+        <v>57715.06698039382</v>
       </c>
       <c r="G150" s="3">
-        <v>58029.61719015912</v>
+        <v>58003.92329925164</v>
       </c>
       <c r="H150" s="3">
-        <v>58402.17932397294</v>
+        <v>58357.83048055138</v>
       </c>
       <c r="I150" s="3">
-        <v>58919.68737305373</v>
+        <v>58857.03711334529</v>
       </c>
       <c r="J150" s="3">
-        <v>59594.25429564246</v>
+        <v>59516.23702996883</v>
       </c>
       <c r="K150" s="3">
-        <v>60424.54679375751</v>
+        <v>60334.32737498623</v>
       </c>
       <c r="L150" s="3">
-        <v>61377.02450449887</v>
+        <v>61277.22459609614</v>
       </c>
       <c r="M150" s="3">
-        <v>62424.13903836967</v>
+        <v>62316.75354938609</v>
       </c>
       <c r="N150" s="3">
-        <v>63568.65765965312</v>
+        <v>63455.10697140875</v>
       </c>
       <c r="O150" s="3">
-        <v>64784.56325905063</v>
+        <v>64665.84587845208</v>
       </c>
       <c r="P150" s="3">
-        <v>66045.99919042762</v>
+        <v>65922.83037368671</v>
       </c>
       <c r="Q150" s="3">
-        <v>67350.35014764602</v>
+        <v>67223.23229613119</v>
       </c>
       <c r="R150" s="3">
-        <v>796100.7403567191</v>
+        <v>795097.5179538066</v>
       </c>
     </row>
     <row r="151" spans="1:18">
@@ -8904,46 +8904,46 @@
         <v>0</v>
       </c>
       <c r="E151" s="3">
-        <v>393429.8258240776</v>
+        <v>393418.4603789521</v>
       </c>
       <c r="F151" s="3">
-        <v>395293.7742814057</v>
+        <v>395219.1825476425</v>
       </c>
       <c r="G151" s="3">
-        <v>397373.1482844555</v>
+        <v>397197.2025723183</v>
       </c>
       <c r="H151" s="3">
-        <v>399924.366011087</v>
+        <v>399620.6755787436</v>
       </c>
       <c r="I151" s="3">
-        <v>403468.1392200658</v>
+        <v>403039.1250003166</v>
       </c>
       <c r="J151" s="3">
-        <v>408087.4145959355</v>
+        <v>407553.1707393941</v>
       </c>
       <c r="K151" s="3">
-        <v>413773.0620282072</v>
+        <v>413155.2607017559</v>
       </c>
       <c r="L151" s="3">
-        <v>420295.4050129589</v>
+        <v>419611.9987504201</v>
       </c>
       <c r="M151" s="3">
-        <v>427465.7986685837</v>
+        <v>426730.4481371879</v>
       </c>
       <c r="N151" s="3">
-        <v>435303.192568999</v>
+        <v>434525.6242054222</v>
       </c>
       <c r="O151" s="3">
-        <v>443629.4276786668</v>
+        <v>442816.479022984</v>
       </c>
       <c r="P151" s="3">
-        <v>452267.4437759954</v>
+        <v>451424.0127342494</v>
       </c>
       <c r="Q151" s="3">
-        <v>461199.3318606477</v>
+        <v>460328.8587590575</v>
       </c>
       <c r="R151" s="3">
-        <v>5451510.329811086</v>
+        <v>5444640.499128445</v>
       </c>
     </row>
     <row r="152" spans="1:18">
@@ -8960,46 +8960,46 @@
         <v>0</v>
       </c>
       <c r="E152" s="3">
-        <v>1543312.449572583</v>
+        <v>1543267.866188696</v>
       </c>
       <c r="F152" s="3">
-        <v>1550624.185162356</v>
+        <v>1550331.583168822</v>
       </c>
       <c r="G152" s="3">
-        <v>1558780.973426952</v>
+        <v>1558090.788824345</v>
       </c>
       <c r="H152" s="3">
-        <v>1568788.669388573</v>
+        <v>1567597.378860281</v>
       </c>
       <c r="I152" s="3">
-        <v>1582689.876040669</v>
+        <v>1581006.976212229</v>
       </c>
       <c r="J152" s="3">
-        <v>1600809.969454155</v>
+        <v>1598714.283919433</v>
       </c>
       <c r="K152" s="3">
-        <v>1623113.134822276</v>
+        <v>1620689.677280699</v>
       </c>
       <c r="L152" s="3">
-        <v>1648698.417045517</v>
+        <v>1646017.610142068</v>
       </c>
       <c r="M152" s="3">
-        <v>1676825.816319029</v>
+        <v>1673941.246936101</v>
       </c>
       <c r="N152" s="3">
-        <v>1707569.666390334</v>
+        <v>1704519.488551407</v>
       </c>
       <c r="O152" s="3">
-        <v>1740231.100423464</v>
+        <v>1737042.135838609</v>
       </c>
       <c r="P152" s="3">
-        <v>1774115.561914638</v>
+        <v>1770807.023665521</v>
       </c>
       <c r="Q152" s="3">
-        <v>1809152.798988263</v>
+        <v>1805738.182488642</v>
       </c>
       <c r="R152" s="3">
-        <v>21384712.61894881</v>
+        <v>21357764.24207686</v>
       </c>
     </row>
     <row r="153" spans="1:18">
@@ -9016,46 +9016,46 @@
         <v>0</v>
       </c>
       <c r="E153" s="3">
-        <v>1879288.513655771</v>
+        <v>1879234.2245575</v>
       </c>
       <c r="F153" s="3">
-        <v>1888191.999604163</v>
+        <v>1887835.69873607</v>
       </c>
       <c r="G153" s="3">
-        <v>1898124.504521249</v>
+        <v>1897284.068097412</v>
       </c>
       <c r="H153" s="3">
-        <v>1910310.856075688</v>
+        <v>1908860.223958474</v>
       </c>
       <c r="I153" s="3">
-        <v>1927238.327887682</v>
+        <v>1925189.0640992</v>
       </c>
       <c r="J153" s="3">
-        <v>1949303.129754448</v>
+        <v>1946751.217628859</v>
       </c>
       <c r="K153" s="3">
-        <v>1976461.650056725</v>
+        <v>1973510.610607469</v>
       </c>
       <c r="L153" s="3">
-        <v>2007616.797553977</v>
+        <v>2004352.384296392</v>
       </c>
       <c r="M153" s="3">
-        <v>2041867.475949243</v>
+        <v>2038354.941523903</v>
       </c>
       <c r="N153" s="3">
-        <v>2079304.20129968</v>
+        <v>2075590.00578542</v>
       </c>
       <c r="O153" s="3">
-        <v>2119075.96484308</v>
+        <v>2115192.768983141</v>
       </c>
       <c r="P153" s="3">
-        <v>2160337.006500206</v>
+        <v>2156308.206026084</v>
       </c>
       <c r="Q153" s="3">
-        <v>2203001.780701264</v>
+        <v>2198843.808951568</v>
       </c>
       <c r="R153" s="3">
-        <v>26040122.20840318</v>
+        <v>26007307.22325149</v>
       </c>
     </row>
     <row r="154" spans="1:18">
@@ -9072,46 +9072,46 @@
         <v>0</v>
       </c>
       <c r="E154" s="3">
-        <v>908998.6845796451</v>
+        <v>908972.2539547763</v>
       </c>
       <c r="F154" s="3">
-        <v>915294.9786781769</v>
+        <v>915121.2966844005</v>
       </c>
       <c r="G154" s="3">
-        <v>922468.386868152</v>
+        <v>922057.7367133191</v>
       </c>
       <c r="H154" s="3">
-        <v>930881.897037754</v>
+        <v>930171.612620516</v>
       </c>
       <c r="I154" s="3">
-        <v>941056.1395606538</v>
+        <v>940051.7627487472</v>
       </c>
       <c r="J154" s="3">
-        <v>953257.8362255536</v>
+        <v>952006.4560553504</v>
       </c>
       <c r="K154" s="3">
-        <v>967577.0389411376</v>
+        <v>966129.5024224792</v>
       </c>
       <c r="L154" s="3">
-        <v>983575.3721824561</v>
+        <v>981973.8223003522</v>
       </c>
       <c r="M154" s="3">
-        <v>1000888.877358063</v>
+        <v>999165.3919996863</v>
       </c>
       <c r="N154" s="3">
-        <v>1019620.037697096</v>
+        <v>1017797.461840885</v>
       </c>
       <c r="O154" s="3">
-        <v>1039393.239308583</v>
+        <v>1037487.635222798</v>
       </c>
       <c r="P154" s="3">
-        <v>1059823.510857336</v>
+        <v>1057846.385061361</v>
       </c>
       <c r="Q154" s="3">
-        <v>1080890.320579508</v>
+        <v>1078849.755872553</v>
       </c>
       <c r="R154" s="3">
-        <v>12723726.31987412</v>
+        <v>12707631.07349722</v>
       </c>
     </row>
     <row r="155" spans="1:18">
@@ -9128,43 +9128,43 @@
         <v>0.3411657413950535</v>
       </c>
       <c r="E155" s="3">
-        <v>0.3405327737840404</v>
+        <v>0.3405340873450804</v>
       </c>
       <c r="F155" s="3">
-        <v>0.3390861359569305</v>
+        <v>0.3390804563325584</v>
       </c>
       <c r="G155" s="3">
-        <v>0.3367206064907633</v>
+        <v>0.3367079483137003</v>
       </c>
       <c r="H155" s="3">
-        <v>0.3354859927532072</v>
+        <v>0.3354624348694093</v>
       </c>
       <c r="I155" s="3">
-        <v>0.3344924328313715</v>
+        <v>0.3344596609879122</v>
       </c>
       <c r="J155" s="3">
-        <v>0.3337716185609467</v>
+        <v>0.333731885647425</v>
       </c>
       <c r="K155" s="3">
-        <v>0.3333907063170999</v>
+        <v>0.3333460278302761</v>
       </c>
       <c r="L155" s="3">
-        <v>0.3329389246615942</v>
+        <v>0.3328905003373809</v>
       </c>
       <c r="M155" s="3">
-        <v>0.3326971410058649</v>
+        <v>0.3326461907756119</v>
       </c>
       <c r="N155" s="3">
-        <v>0.3325633487689346</v>
+        <v>0.3325106449139235</v>
       </c>
       <c r="O155" s="3">
-        <v>0.332489429441744</v>
+        <v>0.3324355039623403</v>
       </c>
       <c r="P155" s="3">
-        <v>0.3323482025383582</v>
+        <v>0.3322933222827822</v>
       </c>
       <c r="Q155" s="3">
-        <v>0.3323412730054667</v>
+        <v>0.3322858514356819</v>
       </c>
       <c r="R155" s="3" t="s">
         <v>19</v>
@@ -9184,43 +9184,43 @@
         <v>0.04535037632743646</v>
       </c>
       <c r="E156" s="3">
-        <v>0.04471514483398276</v>
+        <v>0.04471402746527998</v>
       </c>
       <c r="F156" s="3">
-        <v>0.04469102236004265</v>
+        <v>0.04469100957032307</v>
       </c>
       <c r="G156" s="3">
-        <v>0.04452473753480909</v>
+        <v>0.04452614989542812</v>
       </c>
       <c r="H156" s="3">
-        <v>0.04460951990774174</v>
+        <v>0.04461341486476176</v>
       </c>
       <c r="I156" s="3">
-        <v>0.0447004800860787</v>
+        <v>0.04470671944286383</v>
       </c>
       <c r="J156" s="3">
-        <v>0.04477299864325959</v>
+        <v>0.04478109024917162</v>
       </c>
       <c r="K156" s="3">
-        <v>0.04479703586749677</v>
+        <v>0.04480646777677671</v>
       </c>
       <c r="L156" s="3">
-        <v>0.04485463655093411</v>
+        <v>0.04486507995002207</v>
       </c>
       <c r="M156" s="3">
-        <v>0.04488079854141676</v>
+        <v>0.0448919304391977</v>
       </c>
       <c r="N156" s="3">
-        <v>0.0448909440931286</v>
+        <v>0.04490255220605267</v>
       </c>
       <c r="O156" s="3">
-        <v>0.04489252477688747</v>
+        <v>0.0449044639418132</v>
       </c>
       <c r="P156" s="3">
-        <v>0.04491360991395767</v>
+        <v>0.04492580440248491</v>
       </c>
       <c r="Q156" s="3">
-        <v>0.04490877875029793</v>
+        <v>0.04492112281752544</v>
       </c>
       <c r="R156" s="3" t="s">
         <v>19</v>
@@ -9240,43 +9240,43 @@
         <v>0.2195512735036556</v>
       </c>
       <c r="E157" s="3">
-        <v>0.2116278167611485</v>
+        <v>0.2116161424393409</v>
       </c>
       <c r="F157" s="3">
-        <v>0.2095892577150464</v>
+        <v>0.2095722836169491</v>
       </c>
       <c r="G157" s="3">
-        <v>0.2043105720657347</v>
+        <v>0.204288277113638</v>
       </c>
       <c r="H157" s="3">
-        <v>0.204288072325831</v>
+        <v>0.2042630129326373</v>
       </c>
       <c r="I157" s="3">
-        <v>0.2042451564307447</v>
+        <v>0.2042191252206733</v>
       </c>
       <c r="J157" s="3">
-        <v>0.2042341716327887</v>
+        <v>0.2042078160950068</v>
       </c>
       <c r="K157" s="3">
-        <v>0.2042765101150407</v>
+        <v>0.2042500986589632</v>
       </c>
       <c r="L157" s="3">
-        <v>0.2042198329762524</v>
+        <v>0.2041933332112627</v>
       </c>
       <c r="M157" s="3">
-        <v>0.204239705527474</v>
+        <v>0.2042132152168388</v>
       </c>
       <c r="N157" s="3">
-        <v>0.2042542257453231</v>
+        <v>0.2042277467359465</v>
       </c>
       <c r="O157" s="3">
-        <v>0.2042636097369087</v>
+        <v>0.2042371459215793</v>
       </c>
       <c r="P157" s="3">
-        <v>0.2042345501550655</v>
+        <v>0.2042080550753823</v>
       </c>
       <c r="Q157" s="3">
-        <v>0.2042626701275111</v>
+        <v>0.2042362104067417</v>
       </c>
       <c r="R157" s="3" t="s">
         <v>19</v>
@@ -9576,43 +9576,43 @@
         <v>0</v>
       </c>
       <c r="E163" s="3">
-        <v>89.05713048520413</v>
+        <v>90.10106500007241</v>
       </c>
       <c r="F163" s="3">
-        <v>88.47526733516426</v>
+        <v>89.60175738342717</v>
       </c>
       <c r="G163" s="3">
-        <v>87.94539391007815</v>
+        <v>89.29526516520423</v>
       </c>
       <c r="H163" s="3">
-        <v>87.62061087357053</v>
+        <v>89.07878957346189</v>
       </c>
       <c r="I163" s="3">
-        <v>87.36144996004451</v>
+        <v>88.88203805564171</v>
       </c>
       <c r="J163" s="3">
-        <v>87.1563805505225</v>
+        <v>88.71750422811526</v>
       </c>
       <c r="K163" s="3">
-        <v>87.01388489219885</v>
+        <v>88.60433816803817</v>
       </c>
       <c r="L163" s="3">
-        <v>86.87070287638311</v>
+        <v>88.48176273341795</v>
       </c>
       <c r="M163" s="3">
-        <v>86.75938818838166</v>
+        <v>88.38662658686357</v>
       </c>
       <c r="N163" s="3">
-        <v>86.66970159602538</v>
+        <v>88.3099784572116</v>
       </c>
       <c r="O163" s="3">
-        <v>86.59704095555011</v>
+        <v>88.24802506705804</v>
       </c>
       <c r="P163" s="3">
-        <v>86.52621715543194</v>
+        <v>88.18567605075478</v>
       </c>
       <c r="Q163" s="3">
-        <v>86.47309754282645</v>
+        <v>88.14004468728503</v>
       </c>
       <c r="R163" s="3" t="s">
         <v>19</v>
@@ -9632,43 +9632,43 @@
         <v>0.01226890863757641</v>
       </c>
       <c r="E164" s="3">
-        <v>0.01199268792946653</v>
+        <v>0.01199305976851651</v>
       </c>
       <c r="F164" s="3">
-        <v>0.01200268483333958</v>
+        <v>0.01200384463315342</v>
       </c>
       <c r="G164" s="3">
-        <v>0.01194479880198366</v>
+        <v>0.01194700408937189</v>
       </c>
       <c r="H164" s="3">
-        <v>0.01197360945692622</v>
+        <v>0.01197683243829079</v>
       </c>
       <c r="I164" s="3">
-        <v>0.01200592741176612</v>
+        <v>0.01200997528556574</v>
       </c>
       <c r="J164" s="3">
-        <v>0.01202984588003761</v>
+        <v>0.01203450785177757</v>
       </c>
       <c r="K164" s="3">
-        <v>0.01203406437194114</v>
+        <v>0.01203915579402608</v>
       </c>
       <c r="L164" s="3">
-        <v>0.01205683008764843</v>
+        <v>0.01206224895183924</v>
       </c>
       <c r="M164" s="3">
-        <v>0.01206358402330606</v>
+        <v>0.01206922012767576</v>
       </c>
       <c r="N164" s="3">
-        <v>0.01206560654229435</v>
+        <v>0.01207139252957222</v>
       </c>
       <c r="O164" s="3">
-        <v>0.01206532978780221</v>
+        <v>0.01207121940973669</v>
       </c>
       <c r="P164" s="3">
-        <v>0.0120743396189716</v>
+        <v>0.01208031254997203</v>
       </c>
       <c r="Q164" s="3">
-        <v>0.01207057734796241</v>
+        <v>0.01207659481503813</v>
       </c>
       <c r="R164" s="3" t="s">
         <v>19</v>
@@ -9688,43 +9688,43 @@
         <v>0.03308146768986005</v>
       </c>
       <c r="E165" s="3">
-        <v>0.03272245690451623</v>
+        <v>0.03272096769676348</v>
       </c>
       <c r="F165" s="3">
-        <v>0.03268833752670306</v>
+        <v>0.03268716493716965</v>
       </c>
       <c r="G165" s="3">
-        <v>0.03257993873282544</v>
+        <v>0.03257914580605623</v>
       </c>
       <c r="H165" s="3">
-        <v>0.03263591045081552</v>
+        <v>0.03263658242647097</v>
       </c>
       <c r="I165" s="3">
-        <v>0.03269455267431257</v>
+        <v>0.03269674415729809</v>
       </c>
       <c r="J165" s="3">
-        <v>0.03274315276322199</v>
+        <v>0.03274658239739406</v>
       </c>
       <c r="K165" s="3">
-        <v>0.03276297149555564</v>
+        <v>0.03276731198275063</v>
       </c>
       <c r="L165" s="3">
-        <v>0.03279780646328567</v>
+        <v>0.03280283099818283</v>
       </c>
       <c r="M165" s="3">
-        <v>0.0328172145181107</v>
+        <v>0.03282271031152194</v>
       </c>
       <c r="N165" s="3">
-        <v>0.03282533755083425</v>
+        <v>0.03283115967648045</v>
       </c>
       <c r="O165" s="3">
-        <v>0.03282719498908527</v>
+        <v>0.03283324453207652</v>
       </c>
       <c r="P165" s="3">
-        <v>0.03283927029498607</v>
+        <v>0.03284549185251288</v>
       </c>
       <c r="Q165" s="3">
-        <v>0.03283820140233552</v>
+        <v>0.03284452800248731</v>
       </c>
       <c r="R165" s="3" t="s">
         <v>19</v>
@@ -9744,43 +9744,43 @@
         <v>121000.9090850509</v>
       </c>
       <c r="E166" s="3">
-        <v>118537.9688569864</v>
+        <v>118515.3972478842</v>
       </c>
       <c r="F166" s="3">
-        <v>119365.1925572382</v>
+        <v>119322.9843380517</v>
       </c>
       <c r="G166" s="3">
-        <v>119854.4396321737</v>
+        <v>119785.6941090304</v>
       </c>
       <c r="H166" s="3">
-        <v>121504.3546946129</v>
+        <v>121415.498128547</v>
       </c>
       <c r="I166" s="3">
-        <v>123544.2148965368</v>
+        <v>123440.1345344126</v>
       </c>
       <c r="J166" s="3">
-        <v>125786.9022825334</v>
+        <v>125671.0895509145</v>
       </c>
       <c r="K166" s="3">
-        <v>127930.6587318603</v>
+        <v>127805.6427784343</v>
       </c>
       <c r="L166" s="3">
-        <v>130558.2117107613</v>
+        <v>130425.8143769097</v>
       </c>
       <c r="M166" s="3">
-        <v>133143.760183863</v>
+        <v>133005.1718505112</v>
       </c>
       <c r="N166" s="3">
-        <v>135765.0577896846</v>
+        <v>135621.1481836558</v>
       </c>
       <c r="O166" s="3">
-        <v>138417.5628101268</v>
+        <v>138268.9633246042</v>
       </c>
       <c r="P166" s="3">
-        <v>141330.8484994144</v>
+        <v>141177.9788290449</v>
       </c>
       <c r="Q166" s="3">
-        <v>144114.3106878076</v>
+        <v>143957.4162737527</v>
       </c>
       <c r="R166" s="3" t="s">
         <v>19</v>
@@ -9800,43 +9800,43 @@
         <v>326262.7331074112</v>
       </c>
       <c r="E167" s="3">
-        <v>323434.8796770674</v>
+        <v>323348.5498919341</v>
       </c>
       <c r="F167" s="3">
-        <v>325081.4094870532</v>
+        <v>324923.4048798735</v>
       </c>
       <c r="G167" s="3">
-        <v>326908.0011146667</v>
+        <v>326652.23554493</v>
       </c>
       <c r="H167" s="3">
-        <v>331178.768896934</v>
+        <v>330854.3333924154</v>
       </c>
       <c r="I167" s="3">
-        <v>336435.7207076623</v>
+        <v>336061.5156689743</v>
       </c>
       <c r="J167" s="3">
-        <v>342370.118297525</v>
+        <v>341958.2038281238</v>
       </c>
       <c r="K167" s="3">
-        <v>348293.6766743845</v>
+        <v>347852.2449352287</v>
       </c>
       <c r="L167" s="3">
-        <v>355153.2972392905</v>
+        <v>354688.0821220139</v>
       </c>
       <c r="M167" s="3">
-        <v>362198.110549925</v>
+        <v>361712.7021797247</v>
       </c>
       <c r="N167" s="3">
-        <v>369358.4598447779</v>
+        <v>368855.5036726164</v>
       </c>
       <c r="O167" s="3">
-        <v>376604.7347396784</v>
+        <v>376086.1707452369</v>
       </c>
       <c r="P167" s="3">
-        <v>384385.5714973914</v>
+        <v>383852.6639275046</v>
       </c>
       <c r="Q167" s="3">
-        <v>392065.3190730637</v>
+        <v>391518.756933145</v>
       </c>
       <c r="R167" s="3" t="s">
         <v>19</v>
@@ -10024,46 +10024,46 @@
         <v>0</v>
       </c>
       <c r="E171" s="3">
-        <v>3030514.536511332</v>
+        <v>3028779.993334658</v>
       </c>
       <c r="F171" s="3">
-        <v>3036600.569721173</v>
+        <v>3033791.174338168</v>
       </c>
       <c r="G171" s="3">
-        <v>3072676.90400015</v>
+        <v>3068402.498074546</v>
       </c>
       <c r="H171" s="3">
-        <v>3121394.239347063</v>
+        <v>3116466.347938418</v>
       </c>
       <c r="I171" s="3">
-        <v>3178807.557529681</v>
+        <v>3173579.433077995</v>
       </c>
       <c r="J171" s="3">
-        <v>3243519.997025381</v>
+        <v>3238114.601871819</v>
       </c>
       <c r="K171" s="3">
-        <v>3307378.017961221</v>
+        <v>3301837.858392315</v>
       </c>
       <c r="L171" s="3">
-        <v>3374937.736303682</v>
+        <v>3369278.654315251</v>
       </c>
       <c r="M171" s="3">
-        <v>3447536.332650212</v>
+        <v>3441754.693268677</v>
       </c>
       <c r="N171" s="3">
-        <v>3518908.099756179</v>
+        <v>3513003.967916105</v>
       </c>
       <c r="O171" s="3">
-        <v>3589345.418096531</v>
+        <v>3583320.44104924</v>
       </c>
       <c r="P171" s="3">
-        <v>3663466.085394981</v>
+        <v>3657318.708322715</v>
       </c>
       <c r="Q171" s="3">
-        <v>3739029.037331283</v>
+        <v>3732754.019614305</v>
       </c>
       <c r="R171" s="3">
-        <v>43324114.53162886</v>
+        <v>43258402.39151421</v>
       </c>
     </row>
     <row r="172" spans="1:18">
@@ -10080,46 +10080,46 @@
         <v>9862402</v>
       </c>
       <c r="E172" s="3">
-        <v>9884186.89406015</v>
+        <v>9881998.383682199</v>
       </c>
       <c r="F172" s="3">
-        <v>9944874.352251612</v>
+        <v>9940397.263097983</v>
       </c>
       <c r="G172" s="3">
-        <v>10034027.49758075</v>
+        <v>10026421.11888053</v>
       </c>
       <c r="H172" s="3">
-        <v>10147679.78959994</v>
+        <v>10137529.99836359</v>
       </c>
       <c r="I172" s="3">
-        <v>10290268.35323527</v>
+        <v>10278133.93444446</v>
       </c>
       <c r="J172" s="3">
-        <v>10456235.56086158</v>
+        <v>10442561.59859102</v>
       </c>
       <c r="K172" s="3">
-        <v>10630710.85361202</v>
+        <v>10615830.95733776</v>
       </c>
       <c r="L172" s="3">
-        <v>10828568.60067316</v>
+        <v>10812727.78382032</v>
       </c>
       <c r="M172" s="3">
-        <v>11036832.82900321</v>
+        <v>11020196.03947059</v>
       </c>
       <c r="N172" s="3">
-        <v>11252236.45523154</v>
+        <v>11234921.55949815</v>
       </c>
       <c r="O172" s="3">
-        <v>11472339.77392512</v>
+        <v>11454432.11918391</v>
       </c>
       <c r="P172" s="3">
-        <v>11705058.24412547</v>
+        <v>11686616.40541509</v>
       </c>
       <c r="Q172" s="3">
-        <v>11939305.51400964</v>
+        <v>11920364.84444214</v>
       </c>
       <c r="R172" s="3">
-        <v>149484726.7181695</v>
+        <v>149314534.0062277</v>
       </c>
     </row>
     <row r="173" spans="1:18">
@@ -14617,7 +14617,7 @@
         <v>0.2538</v>
       </c>
       <c r="J79" s="3">
-        <v>0.2537999999999999</v>
+        <v>0.2538</v>
       </c>
       <c r="K79" s="3">
         <v>0.2537999999999999</v>
@@ -14626,7 +14626,7 @@
         <v>0.2538</v>
       </c>
       <c r="M79" s="3">
-        <v>0.2537999999999999</v>
+        <v>0.2538</v>
       </c>
       <c r="N79" s="3">
         <v>0.2538</v>
@@ -14664,40 +14664,40 @@
         <v>27009738.912</v>
       </c>
       <c r="G80" s="3">
-        <v>32834694.25163174</v>
+        <v>32816930.42392865</v>
       </c>
       <c r="H80" s="3">
-        <v>49392651.48817196</v>
+        <v>49349761.35661139</v>
       </c>
       <c r="I80" s="3">
-        <v>50004769.14793261</v>
+        <v>49939540.62476175</v>
       </c>
       <c r="J80" s="3">
-        <v>50806319.25786131</v>
+        <v>50731276.61924804</v>
       </c>
       <c r="K80" s="3">
-        <v>51752478.04183175</v>
+        <v>51672926.94237532</v>
       </c>
       <c r="L80" s="3">
-        <v>52810850.67538707</v>
+        <v>52728623.57111084</v>
       </c>
       <c r="M80" s="3">
-        <v>53841953.77601892</v>
+        <v>53757685.27702214</v>
       </c>
       <c r="N80" s="3">
-        <v>54954743.80899656</v>
+        <v>54868668.65948829</v>
       </c>
       <c r="O80" s="3">
-        <v>56134125.23825622</v>
+        <v>56046185.42999908</v>
       </c>
       <c r="P80" s="3">
-        <v>57292598.84745549</v>
+        <v>57202796.89171506</v>
       </c>
       <c r="Q80" s="3">
-        <v>58436797.76913241</v>
+        <v>58345158.93054393</v>
       </c>
       <c r="R80" s="3">
-        <v>59650813.21120584</v>
+        <v>59557312.19064193</v>
       </c>
     </row>
     <row r="81" spans="1:14">
@@ -16356,46 +16356,46 @@
         <v>0</v>
       </c>
       <c r="E32" s="3">
-        <v>85137560883.95833</v>
+        <v>85399012762.75777</v>
       </c>
       <c r="F32" s="3">
-        <v>85515585746.14221</v>
+        <v>85815799595.39043</v>
       </c>
       <c r="G32" s="3">
-        <v>85795932609.96681</v>
+        <v>86238221468.41631</v>
       </c>
       <c r="H32" s="3">
-        <v>86336848436.47656</v>
+        <v>86765354734.90605</v>
       </c>
       <c r="I32" s="3">
-        <v>87173331115.08069</v>
+        <v>87590235922.03542</v>
       </c>
       <c r="J32" s="3">
-        <v>88251164808.43306</v>
+        <v>88661170019.31863</v>
       </c>
       <c r="K32" s="3">
-        <v>89466773640.31754</v>
+        <v>89873627174.52092</v>
       </c>
       <c r="L32" s="3">
-        <v>90975380765.47096</v>
+        <v>91381743707.53951</v>
       </c>
       <c r="M32" s="3">
-        <v>92566755784.093</v>
+        <v>92976134617.68068</v>
       </c>
       <c r="N32" s="3">
-        <v>94266514484.26511</v>
+        <v>94680241067.95354</v>
       </c>
       <c r="O32" s="3">
-        <v>96052385979.42105</v>
+        <v>96471328646.32677</v>
       </c>
       <c r="P32" s="3">
-        <v>97969064120.33824</v>
+        <v>98394252587.37434</v>
       </c>
       <c r="Q32" s="3">
-        <v>99881537618.55551</v>
+        <v>100314212891.0544</v>
       </c>
       <c r="R32" s="3">
-        <v>1179388835992.519</v>
+        <v>1184561335195.275</v>
       </c>
     </row>
     <row r="33" spans="1:18">
@@ -16412,46 +16412,46 @@
         <v>0</v>
       </c>
       <c r="E33" s="3">
-        <v>22460477234.41212</v>
+        <v>22723760671.43362</v>
       </c>
       <c r="F33" s="3">
-        <v>22685905891.3996</v>
+        <v>22997437912.2804</v>
       </c>
       <c r="G33" s="3">
-        <v>22838183798.37898</v>
+        <v>23306861451.40631</v>
       </c>
       <c r="H33" s="3">
-        <v>23183284289.71689</v>
+        <v>23657002910.47453</v>
       </c>
       <c r="I33" s="3">
-        <v>23607776989.71103</v>
+        <v>24088316600.18823</v>
       </c>
       <c r="J33" s="3">
-        <v>24063148570.75623</v>
+        <v>24552243291.05359</v>
       </c>
       <c r="K33" s="3">
-        <v>24474075511.11186</v>
+        <v>24972287077.39408</v>
       </c>
       <c r="L33" s="3">
-        <v>25003106005.99574</v>
+        <v>25510460327.39064</v>
       </c>
       <c r="M33" s="3">
-        <v>25507010666.02761</v>
+        <v>26025011339.01107</v>
       </c>
       <c r="N33" s="3">
-        <v>26008995337.08569</v>
+        <v>26537548631.24413</v>
       </c>
       <c r="O33" s="3">
-        <v>26514883907.00842</v>
+        <v>27053856100.30074</v>
       </c>
       <c r="P33" s="3">
-        <v>27085258151.23456</v>
+        <v>27634961408.43101</v>
       </c>
       <c r="Q33" s="3">
-        <v>27613368360.42145</v>
+        <v>28174540074.6576</v>
       </c>
       <c r="R33" s="3">
-        <v>321045474713.2602</v>
+        <v>327234287795.266</v>
       </c>
     </row>
     <row r="34" spans="1:18">
@@ -16524,46 +16524,46 @@
         <v>0</v>
       </c>
       <c r="E35" s="3">
-        <v>58927981596.11422</v>
+        <v>58926296436.591</v>
       </c>
       <c r="F35" s="3">
-        <v>59007936947.5001</v>
+        <v>58996898932.56306</v>
       </c>
       <c r="G35" s="3">
-        <v>59082172027.91418</v>
+        <v>59056233072.16083</v>
       </c>
       <c r="H35" s="3">
-        <v>59212067647.91505</v>
+        <v>59167444326.66891</v>
       </c>
       <c r="I35" s="3">
-        <v>59543947554.08225</v>
+        <v>59481007638.47344</v>
       </c>
       <c r="J35" s="3">
-        <v>60082718174.86028</v>
+        <v>60004405028.63889</v>
       </c>
       <c r="K35" s="3">
-        <v>60815883207.85477</v>
+        <v>60725365330.96134</v>
       </c>
       <c r="L35" s="3">
-        <v>61699801949.26424</v>
+        <v>61599701729.45591</v>
       </c>
       <c r="M35" s="3">
-        <v>62699020455.95039</v>
+        <v>62591332360.31437</v>
       </c>
       <c r="N35" s="3">
-        <v>63810499406.19822</v>
+        <v>63696642958.17818</v>
       </c>
       <c r="O35" s="3">
-        <v>65003948221.95701</v>
+        <v>64884921066.17904</v>
       </c>
       <c r="P35" s="3">
-        <v>66250432038.52712</v>
+        <v>66126948743.14185</v>
       </c>
       <c r="Q35" s="3">
-        <v>67545181188.35378</v>
+        <v>67417743618.05898</v>
       </c>
       <c r="R35" s="3">
-        <v>803681590416.4916</v>
+        <v>802674941241.3859</v>
       </c>
     </row>
     <row r="36" spans="1:18">
@@ -16580,46 +16580,46 @@
         <v>0</v>
       </c>
       <c r="E36" s="3">
-        <v>529341649.0398673</v>
+        <v>529195250.3410169</v>
       </c>
       <c r="F36" s="3">
-        <v>527461403.1622463</v>
+        <v>527181246.4666829</v>
       </c>
       <c r="G36" s="3">
-        <v>518786292.3795489</v>
+        <v>518336453.5550686</v>
       </c>
       <c r="H36" s="3">
-        <v>524604643.9516553</v>
+        <v>524015642.8696463</v>
       </c>
       <c r="I36" s="3">
-        <v>531864290.4425843</v>
+        <v>531169402.5289106</v>
       </c>
       <c r="J36" s="3">
-        <v>540413429.1085882</v>
+        <v>539637065.9181825</v>
       </c>
       <c r="K36" s="3">
-        <v>549544798.1939797</v>
+        <v>548704643.0085766</v>
       </c>
       <c r="L36" s="3">
-        <v>559617561.3579296</v>
+        <v>558726401.8399116</v>
       </c>
       <c r="M36" s="3">
-        <v>570436105.107469</v>
+        <v>569502361.3476992</v>
       </c>
       <c r="N36" s="3">
-        <v>581610536.8727413</v>
+        <v>580640274.4227693</v>
       </c>
       <c r="O36" s="3">
-        <v>593014577.2619159</v>
+        <v>592012206.65328</v>
       </c>
       <c r="P36" s="3">
-        <v>604957907.6955825</v>
+        <v>603926412.9205221</v>
       </c>
       <c r="Q36" s="3">
-        <v>617149577.4171875</v>
+        <v>616090705.9746995</v>
       </c>
       <c r="R36" s="3">
-        <v>7248802771.991297</v>
+        <v>7239138067.846966</v>
       </c>
     </row>
     <row r="37" spans="1:18">
@@ -16876,46 +16876,46 @@
         <v>0</v>
       </c>
       <c r="E42" s="3">
-        <v>85137560883.95833</v>
+        <v>85399012762.75777</v>
       </c>
       <c r="F42" s="3">
-        <v>85515585746.14221</v>
+        <v>85815799595.39043</v>
       </c>
       <c r="G42" s="3">
-        <v>85795932609.96681</v>
+        <v>86238221468.41631</v>
       </c>
       <c r="H42" s="3">
-        <v>86336848436.47656</v>
+        <v>86765354734.90605</v>
       </c>
       <c r="I42" s="3">
-        <v>87173331115.08069</v>
+        <v>87590235922.03542</v>
       </c>
       <c r="J42" s="3">
-        <v>88251164808.43306</v>
+        <v>88661170019.31863</v>
       </c>
       <c r="K42" s="3">
-        <v>89466773640.31754</v>
+        <v>89873627174.52092</v>
       </c>
       <c r="L42" s="3">
-        <v>90975380765.47096</v>
+        <v>91381743707.53951</v>
       </c>
       <c r="M42" s="3">
-        <v>92566755784.093</v>
+        <v>92976134617.68068</v>
       </c>
       <c r="N42" s="3">
-        <v>94266514484.26511</v>
+        <v>94680241067.95354</v>
       </c>
       <c r="O42" s="3">
-        <v>96052385979.42105</v>
+        <v>96471328646.32677</v>
       </c>
       <c r="P42" s="3">
-        <v>97969064120.33824</v>
+        <v>98394252587.37434</v>
       </c>
       <c r="Q42" s="3">
-        <v>99881537618.55551</v>
+        <v>100314212891.0544</v>
       </c>
       <c r="R42" s="3">
-        <v>1179388835992.519</v>
+        <v>1184561335195.275</v>
       </c>
     </row>
     <row r="43" spans="1:18">
@@ -16932,46 +16932,46 @@
         <v>0</v>
       </c>
       <c r="E43" s="3">
-        <v>22460477234.41212</v>
+        <v>22723760671.43362</v>
       </c>
       <c r="F43" s="3">
-        <v>22685905891.3996</v>
+        <v>22997437912.2804</v>
       </c>
       <c r="G43" s="3">
-        <v>22838183798.37898</v>
+        <v>23306861451.40631</v>
       </c>
       <c r="H43" s="3">
-        <v>23183284289.71689</v>
+        <v>23657002910.47453</v>
       </c>
       <c r="I43" s="3">
-        <v>23607776989.71103</v>
+        <v>24088316600.18823</v>
       </c>
       <c r="J43" s="3">
-        <v>24063148570.75623</v>
+        <v>24552243291.05359</v>
       </c>
       <c r="K43" s="3">
-        <v>24474075511.11186</v>
+        <v>24972287077.39408</v>
       </c>
       <c r="L43" s="3">
-        <v>25003106005.99574</v>
+        <v>25510460327.39064</v>
       </c>
       <c r="M43" s="3">
-        <v>25507010666.02761</v>
+        <v>26025011339.01107</v>
       </c>
       <c r="N43" s="3">
-        <v>26008995337.08569</v>
+        <v>26537548631.24413</v>
       </c>
       <c r="O43" s="3">
-        <v>26514883907.00842</v>
+        <v>27053856100.30074</v>
       </c>
       <c r="P43" s="3">
-        <v>27085258151.23456</v>
+        <v>27634961408.43101</v>
       </c>
       <c r="Q43" s="3">
-        <v>27613368360.42145</v>
+        <v>28174540074.6576</v>
       </c>
       <c r="R43" s="3">
-        <v>321045474713.2602</v>
+        <v>327234287795.266</v>
       </c>
     </row>
     <row r="44" spans="1:18">
@@ -17044,46 +17044,46 @@
         <v>0</v>
       </c>
       <c r="E45" s="3">
-        <v>58927981596.11422</v>
+        <v>58926296436.591</v>
       </c>
       <c r="F45" s="3">
-        <v>59007936947.5001</v>
+        <v>58996898932.56306</v>
       </c>
       <c r="G45" s="3">
-        <v>59082172027.91418</v>
+        <v>59056233072.16083</v>
       </c>
       <c r="H45" s="3">
-        <v>59212067647.91505</v>
+        <v>59167444326.66891</v>
       </c>
       <c r="I45" s="3">
-        <v>59543947554.08225</v>
+        <v>59481007638.47344</v>
       </c>
       <c r="J45" s="3">
-        <v>60082718174.86028</v>
+        <v>60004405028.63889</v>
       </c>
       <c r="K45" s="3">
-        <v>60815883207.85477</v>
+        <v>60725365330.96134</v>
       </c>
       <c r="L45" s="3">
-        <v>61699801949.26424</v>
+        <v>61599701729.45591</v>
       </c>
       <c r="M45" s="3">
-        <v>62699020455.95039</v>
+        <v>62591332360.31437</v>
       </c>
       <c r="N45" s="3">
-        <v>63810499406.19822</v>
+        <v>63696642958.17818</v>
       </c>
       <c r="O45" s="3">
-        <v>65003948221.95701</v>
+        <v>64884921066.17904</v>
       </c>
       <c r="P45" s="3">
-        <v>66250432038.52712</v>
+        <v>66126948743.14185</v>
       </c>
       <c r="Q45" s="3">
-        <v>67545181188.35378</v>
+        <v>67417743618.05898</v>
       </c>
       <c r="R45" s="3">
-        <v>803681590416.4916</v>
+        <v>802674941241.3859</v>
       </c>
     </row>
     <row r="46" spans="1:18">
@@ -17100,46 +17100,46 @@
         <v>0</v>
       </c>
       <c r="E46" s="3">
-        <v>529341649.0398673</v>
+        <v>529195250.3410169</v>
       </c>
       <c r="F46" s="3">
-        <v>527461403.1622463</v>
+        <v>527181246.4666829</v>
       </c>
       <c r="G46" s="3">
-        <v>518786292.3795489</v>
+        <v>518336453.5550686</v>
       </c>
       <c r="H46" s="3">
-        <v>524604643.9516553</v>
+        <v>524015642.8696463</v>
       </c>
       <c r="I46" s="3">
-        <v>531864290.4425843</v>
+        <v>531169402.5289106</v>
       </c>
       <c r="J46" s="3">
-        <v>540413429.1085882</v>
+        <v>539637065.9181825</v>
       </c>
       <c r="K46" s="3">
-        <v>549544798.1939797</v>
+        <v>548704643.0085766</v>
       </c>
       <c r="L46" s="3">
-        <v>559617561.3579296</v>
+        <v>558726401.8399116</v>
       </c>
       <c r="M46" s="3">
-        <v>570436105.107469</v>
+        <v>569502361.3476992</v>
       </c>
       <c r="N46" s="3">
-        <v>581610536.8727413</v>
+        <v>580640274.4227693</v>
       </c>
       <c r="O46" s="3">
-        <v>593014577.2619159</v>
+        <v>592012206.65328</v>
       </c>
       <c r="P46" s="3">
-        <v>604957907.6955825</v>
+        <v>603926412.9205221</v>
       </c>
       <c r="Q46" s="3">
-        <v>617149577.4171875</v>
+        <v>616090705.9746995</v>
       </c>
       <c r="R46" s="3">
-        <v>7248802771.991297</v>
+        <v>7239138067.846966</v>
       </c>
     </row>
     <row r="47" spans="1:18">
@@ -17396,46 +17396,46 @@
         <v>0</v>
       </c>
       <c r="E52" s="3">
-        <v>85137560883.95833</v>
+        <v>85399012762.75777</v>
       </c>
       <c r="F52" s="3">
-        <v>85515585746.14221</v>
+        <v>85815799595.39043</v>
       </c>
       <c r="G52" s="3">
-        <v>85795932609.96681</v>
+        <v>86238221468.41631</v>
       </c>
       <c r="H52" s="3">
-        <v>86336848436.47656</v>
+        <v>86765354734.90605</v>
       </c>
       <c r="I52" s="3">
-        <v>87173331115.08069</v>
+        <v>87590235922.03542</v>
       </c>
       <c r="J52" s="3">
-        <v>88251164808.43306</v>
+        <v>88661170019.31863</v>
       </c>
       <c r="K52" s="3">
-        <v>89466773640.31754</v>
+        <v>89873627174.52092</v>
       </c>
       <c r="L52" s="3">
-        <v>90975380765.47096</v>
+        <v>91381743707.53951</v>
       </c>
       <c r="M52" s="3">
-        <v>92566755784.093</v>
+        <v>92976134617.68068</v>
       </c>
       <c r="N52" s="3">
-        <v>94266514484.26511</v>
+        <v>94680241067.95354</v>
       </c>
       <c r="O52" s="3">
-        <v>96052385979.42105</v>
+        <v>96471328646.32677</v>
       </c>
       <c r="P52" s="3">
-        <v>97969064120.33824</v>
+        <v>98394252587.37434</v>
       </c>
       <c r="Q52" s="3">
-        <v>99881537618.55551</v>
+        <v>100314212891.0544</v>
       </c>
       <c r="R52" s="3">
-        <v>1179388835992.519</v>
+        <v>1184561335195.275</v>
       </c>
     </row>
     <row r="53" spans="1:18">
@@ -17452,46 +17452,46 @@
         <v>0</v>
       </c>
       <c r="E53" s="3">
-        <v>22460477234.41212</v>
+        <v>22723760671.43362</v>
       </c>
       <c r="F53" s="3">
-        <v>22685905891.3996</v>
+        <v>22997437912.2804</v>
       </c>
       <c r="G53" s="3">
-        <v>22838183798.37898</v>
+        <v>23306861451.40631</v>
       </c>
       <c r="H53" s="3">
-        <v>23183284289.71689</v>
+        <v>23657002910.47453</v>
       </c>
       <c r="I53" s="3">
-        <v>23607776989.71103</v>
+        <v>24088316600.18823</v>
       </c>
       <c r="J53" s="3">
-        <v>24063148570.75623</v>
+        <v>24552243291.05359</v>
       </c>
       <c r="K53" s="3">
-        <v>24474075511.11186</v>
+        <v>24972287077.39408</v>
       </c>
       <c r="L53" s="3">
-        <v>25003106005.99574</v>
+        <v>25510460327.39064</v>
       </c>
       <c r="M53" s="3">
-        <v>25507010666.02761</v>
+        <v>26025011339.01107</v>
       </c>
       <c r="N53" s="3">
-        <v>26008995337.08569</v>
+        <v>26537548631.24413</v>
       </c>
       <c r="O53" s="3">
-        <v>26514883907.00842</v>
+        <v>27053856100.30074</v>
       </c>
       <c r="P53" s="3">
-        <v>27085258151.23456</v>
+        <v>27634961408.43101</v>
       </c>
       <c r="Q53" s="3">
-        <v>27613368360.42145</v>
+        <v>28174540074.6576</v>
       </c>
       <c r="R53" s="3">
-        <v>321045474713.2602</v>
+        <v>327234287795.266</v>
       </c>
     </row>
     <row r="54" spans="1:18">
@@ -17564,46 +17564,46 @@
         <v>0</v>
       </c>
       <c r="E55" s="3">
-        <v>58927981596.11422</v>
+        <v>58926296436.591</v>
       </c>
       <c r="F55" s="3">
-        <v>59007936947.5001</v>
+        <v>58996898932.56306</v>
       </c>
       <c r="G55" s="3">
-        <v>59082172027.91418</v>
+        <v>59056233072.16083</v>
       </c>
       <c r="H55" s="3">
-        <v>59212067647.91505</v>
+        <v>59167444326.66891</v>
       </c>
       <c r="I55" s="3">
-        <v>59543947554.08225</v>
+        <v>59481007638.47344</v>
       </c>
       <c r="J55" s="3">
-        <v>60082718174.86028</v>
+        <v>60004405028.63889</v>
       </c>
       <c r="K55" s="3">
-        <v>60815883207.85477</v>
+        <v>60725365330.96134</v>
       </c>
       <c r="L55" s="3">
-        <v>61699801949.26424</v>
+        <v>61599701729.45591</v>
       </c>
       <c r="M55" s="3">
-        <v>62699020455.95039</v>
+        <v>62591332360.31437</v>
       </c>
       <c r="N55" s="3">
-        <v>63810499406.19822</v>
+        <v>63696642958.17818</v>
       </c>
       <c r="O55" s="3">
-        <v>65003948221.95701</v>
+        <v>64884921066.17904</v>
       </c>
       <c r="P55" s="3">
-        <v>66250432038.52712</v>
+        <v>66126948743.14185</v>
       </c>
       <c r="Q55" s="3">
-        <v>67545181188.35378</v>
+        <v>67417743618.05898</v>
       </c>
       <c r="R55" s="3">
-        <v>803681590416.4916</v>
+        <v>802674941241.3859</v>
       </c>
     </row>
     <row r="56" spans="1:18">
@@ -17620,46 +17620,46 @@
         <v>0</v>
       </c>
       <c r="E56" s="3">
-        <v>529341649.0398673</v>
+        <v>529195250.3410169</v>
       </c>
       <c r="F56" s="3">
-        <v>527461403.1622463</v>
+        <v>527181246.4666829</v>
       </c>
       <c r="G56" s="3">
-        <v>518786292.3795489</v>
+        <v>518336453.5550686</v>
       </c>
       <c r="H56" s="3">
-        <v>524604643.9516553</v>
+        <v>524015642.8696463</v>
       </c>
       <c r="I56" s="3">
-        <v>531864290.4425843</v>
+        <v>531169402.5289106</v>
       </c>
       <c r="J56" s="3">
-        <v>540413429.1085882</v>
+        <v>539637065.9181825</v>
       </c>
       <c r="K56" s="3">
-        <v>549544798.1939797</v>
+        <v>548704643.0085766</v>
       </c>
       <c r="L56" s="3">
-        <v>559617561.3579296</v>
+        <v>558726401.8399116</v>
       </c>
       <c r="M56" s="3">
-        <v>570436105.107469</v>
+        <v>569502361.3476992</v>
       </c>
       <c r="N56" s="3">
-        <v>581610536.8727413</v>
+        <v>580640274.4227693</v>
       </c>
       <c r="O56" s="3">
-        <v>593014577.2619159</v>
+        <v>592012206.65328</v>
       </c>
       <c r="P56" s="3">
-        <v>604957907.6955825</v>
+        <v>603926412.9205221</v>
       </c>
       <c r="Q56" s="3">
-        <v>617149577.4171875</v>
+        <v>616090705.9746995</v>
       </c>
       <c r="R56" s="3">
-        <v>7248802771.991297</v>
+        <v>7239138067.846966</v>
       </c>
     </row>
     <row r="57" spans="1:18">

</xml_diff>

<commit_message>
pandas future warning fix
</commit_message>
<xml_diff>
--- a/tests/scen_results_test_2025_SQLNS.xlsx
+++ b/tests/scen_results_test_2025_SQLNS.xlsx
@@ -25,10 +25,10 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2.1.0</t>
+    <t>2.2.0</t>
   </si>
   <si>
-    <t>2025-07-30</t>
+    <t>2026-02-23</t>
   </si>
   <si>
     <t>Scenario</t>
@@ -769,25 +769,25 @@
         <v>1185682.156836694</v>
       </c>
       <c r="H2" s="3">
-        <v>1192823.933083587</v>
+        <v>1192823.933083586</v>
       </c>
       <c r="I2" s="3">
         <v>1202931.282480146</v>
       </c>
       <c r="J2" s="3">
-        <v>1216320.444463288</v>
+        <v>1216320.444463287</v>
       </c>
       <c r="K2" s="3">
-        <v>1232972.185062426</v>
+        <v>1232972.185062425</v>
       </c>
       <c r="L2" s="3">
-        <v>1252188.553667712</v>
+        <v>1252188.553667711</v>
       </c>
       <c r="M2" s="3">
         <v>1273391.233600219</v>
       </c>
       <c r="N2" s="3">
-        <v>1296622.465197729</v>
+        <v>1296622.465197728</v>
       </c>
       <c r="O2" s="3">
         <v>1321339.784881344</v>
@@ -822,16 +822,16 @@
         <v>196598.263595488</v>
       </c>
       <c r="G3" s="3">
-        <v>199458.3825701244</v>
+        <v>199458.3825701243</v>
       </c>
       <c r="H3" s="3">
         <v>202513.0761709206</v>
       </c>
       <c r="I3" s="3">
-        <v>206247.0019222059</v>
+        <v>206247.0019222058</v>
       </c>
       <c r="J3" s="3">
-        <v>210249.2629382346</v>
+        <v>210249.2629382347</v>
       </c>
       <c r="K3" s="3">
         <v>213867.341355186</v>
@@ -840,19 +840,19 @@
         <v>218490.689882769</v>
       </c>
       <c r="M3" s="3">
-        <v>222908.8082589257</v>
+        <v>222908.8082589258</v>
       </c>
       <c r="N3" s="3">
         <v>227306.0953553297</v>
       </c>
       <c r="O3" s="3">
-        <v>231733.5108810464</v>
+        <v>231733.5108810465</v>
       </c>
       <c r="P3" s="3">
         <v>236714.4801659135</v>
       </c>
       <c r="Q3" s="3">
-        <v>241339.3458974526</v>
+        <v>241339.3458974525</v>
       </c>
       <c r="R3" s="3">
         <v>2801591.749435167</v>
@@ -887,19 +887,19 @@
         <v>780747.3249886667</v>
       </c>
       <c r="J4" s="3">
-        <v>789437.3911249649</v>
+        <v>789437.3911249653</v>
       </c>
       <c r="K4" s="3">
-        <v>800244.9926218479</v>
+        <v>800244.9926218481</v>
       </c>
       <c r="L4" s="3">
         <v>812717.1334690286</v>
       </c>
       <c r="M4" s="3">
-        <v>826478.4645450347</v>
+        <v>826478.4645450348</v>
       </c>
       <c r="N4" s="3">
-        <v>841556.4014065251</v>
+        <v>841556.4014065254</v>
       </c>
       <c r="O4" s="3">
         <v>857598.8649328577</v>
@@ -937,13 +937,13 @@
         <v>58002.32623787722</v>
       </c>
       <c r="H5" s="3">
-        <v>58351.69443356231</v>
+        <v>58351.6944335623</v>
       </c>
       <c r="I5" s="3">
-        <v>58846.13535410663</v>
+        <v>58846.13535410661</v>
       </c>
       <c r="J5" s="3">
-        <v>59501.11910073717</v>
+        <v>59501.11910073716</v>
       </c>
       <c r="K5" s="3">
         <v>60315.70476780701</v>
@@ -952,7 +952,7 @@
         <v>61255.74934427656</v>
       </c>
       <c r="M5" s="3">
-        <v>62292.96218540048</v>
+        <v>62292.96218540047</v>
       </c>
       <c r="N5" s="3">
         <v>63429.40964415397</v>
@@ -967,7 +967,7 @@
         <v>67193.4105637453</v>
       </c>
       <c r="R5" s="3">
-        <v>794888.8825335219</v>
+        <v>794888.8825335217</v>
       </c>
     </row>
     <row r="6" spans="1:18">
@@ -996,22 +996,22 @@
         <v>399578.6573744518</v>
       </c>
       <c r="I6" s="3">
-        <v>402964.4723212148</v>
+        <v>402964.4723212145</v>
       </c>
       <c r="J6" s="3">
         <v>407449.6467213977</v>
       </c>
       <c r="K6" s="3">
-        <v>413027.7374747834</v>
+        <v>413027.7374747833</v>
       </c>
       <c r="L6" s="3">
-        <v>419464.9412849575</v>
+        <v>419464.9412849573</v>
       </c>
       <c r="M6" s="3">
         <v>426567.5304812268</v>
       </c>
       <c r="N6" s="3">
-        <v>434349.6549619883</v>
+        <v>434349.6549619881</v>
       </c>
       <c r="O6" s="3">
         <v>442629.597323257</v>
@@ -1023,7 +1023,7 @@
         <v>460124.6465608858</v>
       </c>
       <c r="R6" s="3">
-        <v>5443211.812919289</v>
+        <v>5443211.812919288</v>
       </c>
     </row>
     <row r="7" spans="1:18">
@@ -1049,7 +1049,7 @@
         <v>1558047.88885353</v>
       </c>
       <c r="H7" s="3">
-        <v>1567432.553487279</v>
+        <v>1567432.553487278</v>
       </c>
       <c r="I7" s="3">
         <v>1580714.135147598</v>
@@ -1061,7 +1061,7 @@
         <v>1620189.44020949</v>
       </c>
       <c r="L7" s="3">
-        <v>1645440.745851783</v>
+        <v>1645440.745851782</v>
       </c>
       <c r="M7" s="3">
         <v>1673302.167664026</v>
@@ -1079,7 +1079,7 @@
         <v>1804937.116562505</v>
       </c>
       <c r="R7" s="3">
-        <v>21352159.91554034</v>
+        <v>21352159.91554033</v>
       </c>
     </row>
     <row r="8" spans="1:18">
@@ -1102,22 +1102,22 @@
         <v>1887866.281325574</v>
       </c>
       <c r="G8" s="3">
-        <v>1897231.828887905</v>
+        <v>1897231.828887904</v>
       </c>
       <c r="H8" s="3">
-        <v>1908659.516428168</v>
+        <v>1908659.516428167</v>
       </c>
       <c r="I8" s="3">
-        <v>1924832.472114707</v>
+        <v>1924832.472114705</v>
       </c>
       <c r="J8" s="3">
-        <v>1946256.716487516</v>
+        <v>1946256.716487515</v>
       </c>
       <c r="K8" s="3">
         <v>1972901.472916466</v>
       </c>
       <c r="L8" s="3">
-        <v>2003649.937792464</v>
+        <v>2003649.937792463</v>
       </c>
       <c r="M8" s="3">
         <v>2037576.735959853</v>
@@ -1135,7 +1135,7 @@
         <v>2197868.352559647</v>
       </c>
       <c r="R8" s="3">
-        <v>26000482.84592611</v>
+        <v>26000482.8459261</v>
       </c>
     </row>
     <row r="9" spans="1:18">
@@ -1158,25 +1158,25 @@
         <v>912268.682157184</v>
       </c>
       <c r="G9" s="3">
-        <v>916794.371194003</v>
+        <v>916794.3711940027</v>
       </c>
       <c r="H9" s="3">
         <v>922316.5427352753</v>
       </c>
       <c r="I9" s="3">
-        <v>930131.7577834454</v>
+        <v>930131.7577834451</v>
       </c>
       <c r="J9" s="3">
-        <v>940484.5393196864</v>
+        <v>940484.5393196858</v>
       </c>
       <c r="K9" s="3">
-        <v>953360.0152335694</v>
+        <v>953360.0152335691</v>
       </c>
       <c r="L9" s="3">
-        <v>968218.515439997</v>
+        <v>968218.5154399967</v>
       </c>
       <c r="M9" s="3">
-        <v>984612.8733244161</v>
+        <v>984612.873324416</v>
       </c>
       <c r="N9" s="3">
         <v>1002575.750004051</v>
@@ -1261,7 +1261,7 @@
         <v>20</v>
       </c>
       <c r="D11" s="3">
-        <v>0.04535037632743646</v>
+        <v>0.04535037632743647</v>
       </c>
       <c r="E11" s="3">
         <v>0.04515789980144898</v>
@@ -1438,10 +1438,10 @@
         <v>483657.4722049777</v>
       </c>
       <c r="G14" s="3">
-        <v>492451.2444268863</v>
+        <v>492451.2444268864</v>
       </c>
       <c r="H14" s="3">
-        <v>501245.016648795</v>
+        <v>501245.0166487951</v>
       </c>
       <c r="I14" s="3">
         <v>512237.2319261809</v>
@@ -1453,16 +1453,16 @@
         <v>532023.2194254755</v>
       </c>
       <c r="L14" s="3">
-        <v>545213.8777583386</v>
+        <v>545213.8777583385</v>
       </c>
       <c r="M14" s="3">
-        <v>556206.0930357242</v>
+        <v>556206.0930357244</v>
       </c>
       <c r="N14" s="3">
-        <v>567198.3083131101</v>
+        <v>567198.3083131103</v>
       </c>
       <c r="O14" s="3">
-        <v>578190.523590496</v>
+        <v>578190.5235904962</v>
       </c>
       <c r="P14" s="3">
         <v>591381.1819233592</v>
@@ -1497,7 +1497,7 @@
         <v>0.18698022</v>
       </c>
       <c r="H15" s="3">
-        <v>0.1869802199999999</v>
+        <v>0.18698022</v>
       </c>
       <c r="I15" s="3">
         <v>0.18698022</v>
@@ -1518,7 +1518,7 @@
         <v>0.18698022</v>
       </c>
       <c r="O15" s="3">
-        <v>0.1869802199999999</v>
+        <v>0.18698022</v>
       </c>
       <c r="P15" s="3">
         <v>0.18698022</v>
@@ -1562,7 +1562,7 @@
         <v>2558725.427536433</v>
       </c>
       <c r="K16" s="3">
-        <v>2650598.148654525</v>
+        <v>2650598.148654524</v>
       </c>
       <c r="L16" s="3">
         <v>2741307.682941661</v>
@@ -1574,7 +1574,7 @@
         <v>2933535.31226689</v>
       </c>
       <c r="O16" s="3">
-        <v>3033864.776969503</v>
+        <v>3033864.776969504</v>
       </c>
       <c r="P16" s="3">
         <v>3133930.392536641</v>
@@ -1612,7 +1612,7 @@
         <v>0.1887220562459707</v>
       </c>
       <c r="I17" s="3">
-        <v>0.1887068640814534</v>
+        <v>0.1887068640814535</v>
       </c>
       <c r="J17" s="3">
         <v>0.1886876101253084</v>
@@ -1636,7 +1636,7 @@
         <v>0.188638085652016</v>
       </c>
       <c r="Q17" s="3">
-        <v>0.1886205769816762</v>
+        <v>0.1886205769816761</v>
       </c>
       <c r="R17" s="3" t="s">
         <v>19</v>
@@ -1683,16 +1683,16 @@
         <v>88.74337539911589</v>
       </c>
       <c r="N18" s="3">
-        <v>88.67335364522062</v>
+        <v>88.67335364522063</v>
       </c>
       <c r="O18" s="3">
-        <v>88.61700699358508</v>
+        <v>88.61700699358511</v>
       </c>
       <c r="P18" s="3">
-        <v>88.55940517252557</v>
+        <v>88.5594051725256</v>
       </c>
       <c r="Q18" s="3">
-        <v>88.51790677520275</v>
+        <v>88.51790677520276</v>
       </c>
       <c r="R18" s="3" t="s">
         <v>19</v>
@@ -1765,7 +1765,7 @@
         <v>29</v>
       </c>
       <c r="D20" s="3">
-        <v>0.03308146768986005</v>
+        <v>0.03308146768986006</v>
       </c>
       <c r="E20" s="3">
         <v>0.03300344769614093</v>
@@ -2222,7 +2222,7 @@
         <v>2586677.201497451</v>
       </c>
       <c r="G28" s="3">
-        <v>2633707.696070131</v>
+        <v>2633707.696070132</v>
       </c>
       <c r="H28" s="3">
         <v>2680738.190642813</v>
@@ -2243,13 +2243,13 @@
         <v>2974678.781722068</v>
       </c>
       <c r="N28" s="3">
-        <v>3033466.899937919</v>
+        <v>3033466.89993792</v>
       </c>
       <c r="O28" s="3">
-        <v>3092255.018153772</v>
+        <v>3092255.018153771</v>
       </c>
       <c r="P28" s="3">
-        <v>3162800.760012793</v>
+        <v>3162800.760012792</v>
       </c>
       <c r="Q28" s="3">
         <v>3221588.878228643</v>
@@ -2845,7 +2845,7 @@
         <v>20</v>
       </c>
       <c r="D40" s="3">
-        <v>0.04535037632743646</v>
+        <v>0.04535037632743647</v>
       </c>
       <c r="E40" s="3">
         <v>0.04514529622817693</v>
@@ -2854,13 +2854,13 @@
         <v>0.04520799432205112</v>
       </c>
       <c r="G40" s="3">
-        <v>0.04531247549066409</v>
+        <v>0.04531247549066408</v>
       </c>
       <c r="H40" s="3">
         <v>0.04540658766245453</v>
       </c>
       <c r="I40" s="3">
-        <v>0.0455063349443774</v>
+        <v>0.04550633494437741</v>
       </c>
       <c r="J40" s="3">
         <v>0.04558631933395784</v>
@@ -2881,7 +2881,7 @@
         <v>0.04571938995269134</v>
       </c>
       <c r="P40" s="3">
-        <v>0.04574125906916457</v>
+        <v>0.04574125906916458</v>
       </c>
       <c r="Q40" s="3">
         <v>0.04573697811278184</v>
@@ -2907,7 +2907,7 @@
         <v>0.2202889468938179</v>
       </c>
       <c r="F41" s="3">
-        <v>0.2199437382411898</v>
+        <v>0.2199437382411899</v>
       </c>
       <c r="G41" s="3">
         <v>0.2198974624532505</v>
@@ -2940,7 +2940,7 @@
         <v>0.2201889992151971</v>
       </c>
       <c r="Q41" s="3">
-        <v>0.2202252770729862</v>
+        <v>0.2202252770729863</v>
       </c>
       <c r="R41" s="3" t="s">
         <v>19</v>
@@ -3022,10 +3022,10 @@
         <v>483657.4722049777</v>
       </c>
       <c r="G43" s="3">
-        <v>492451.2444268863</v>
+        <v>492451.2444268864</v>
       </c>
       <c r="H43" s="3">
-        <v>501245.016648795</v>
+        <v>501245.0166487951</v>
       </c>
       <c r="I43" s="3">
         <v>512237.2319261809</v>
@@ -3037,16 +3037,16 @@
         <v>532023.2194254755</v>
       </c>
       <c r="L43" s="3">
-        <v>545213.8777583386</v>
+        <v>545213.8777583385</v>
       </c>
       <c r="M43" s="3">
-        <v>556206.0930357242</v>
+        <v>556206.0930357244</v>
       </c>
       <c r="N43" s="3">
-        <v>567198.3083131101</v>
+        <v>567198.3083131103</v>
       </c>
       <c r="O43" s="3">
-        <v>578190.523590496</v>
+        <v>578190.5235904962</v>
       </c>
       <c r="P43" s="3">
         <v>591381.1819233592</v>
@@ -3081,7 +3081,7 @@
         <v>0.18698022</v>
       </c>
       <c r="H44" s="3">
-        <v>0.1869802199999999</v>
+        <v>0.18698022</v>
       </c>
       <c r="I44" s="3">
         <v>0.18698022</v>
@@ -3102,7 +3102,7 @@
         <v>0.18698022</v>
       </c>
       <c r="O44" s="3">
-        <v>0.1869802199999999</v>
+        <v>0.18698022</v>
       </c>
       <c r="P44" s="3">
         <v>0.18698022</v>
@@ -3146,7 +3146,7 @@
         <v>2558725.427536433</v>
       </c>
       <c r="K45" s="3">
-        <v>2650598.148654525</v>
+        <v>2650598.148654524</v>
       </c>
       <c r="L45" s="3">
         <v>2741307.682941661</v>
@@ -3158,7 +3158,7 @@
         <v>2933535.31226689</v>
       </c>
       <c r="O45" s="3">
-        <v>3033864.776969503</v>
+        <v>3033864.776969504</v>
       </c>
       <c r="P45" s="3">
         <v>3133930.392536641</v>
@@ -3196,7 +3196,7 @@
         <v>0.1887220562459707</v>
       </c>
       <c r="I46" s="3">
-        <v>0.1887068640814534</v>
+        <v>0.1887068640814535</v>
       </c>
       <c r="J46" s="3">
         <v>0.1886876101253084</v>
@@ -3220,7 +3220,7 @@
         <v>0.188638085652016</v>
       </c>
       <c r="Q46" s="3">
-        <v>0.1886205769816762</v>
+        <v>0.1886205769816761</v>
       </c>
       <c r="R46" s="3" t="s">
         <v>19</v>
@@ -3329,7 +3329,7 @@
         <v>0.01236792559112337</v>
       </c>
       <c r="P48" s="3">
-        <v>0.01237721271433998</v>
+        <v>0.01237721271433999</v>
       </c>
       <c r="Q48" s="3">
         <v>0.01237362607897</v>
@@ -3349,7 +3349,7 @@
         <v>29</v>
       </c>
       <c r="D49" s="3">
-        <v>0.03308146768986005</v>
+        <v>0.03308146768986006</v>
       </c>
       <c r="E49" s="3">
         <v>0.03299568793338076</v>
@@ -3373,7 +3373,7 @@
         <v>0.03328120369497208</v>
       </c>
       <c r="L49" s="3">
-        <v>0.03331854692259711</v>
+        <v>0.03331854692259712</v>
       </c>
       <c r="M49" s="3">
         <v>0.03333998879049142</v>
@@ -3385,7 +3385,7 @@
         <v>0.03335144908739439</v>
       </c>
       <c r="P49" s="3">
-        <v>0.03336402390377671</v>
+        <v>0.03336402390377672</v>
       </c>
       <c r="Q49" s="3">
         <v>0.03336332492043433</v>
@@ -3408,7 +3408,7 @@
         <v>121000.9090850509</v>
       </c>
       <c r="E50" s="3">
-        <v>120017.7280824316</v>
+        <v>120017.7280824315</v>
       </c>
       <c r="F50" s="3">
         <v>121108.7687025134</v>
@@ -3473,7 +3473,7 @@
         <v>331311.6972334617</v>
       </c>
       <c r="H51" s="3">
-        <v>335524.8707785656</v>
+        <v>335524.8707785655</v>
       </c>
       <c r="I51" s="3">
         <v>340775.1597925952</v>
@@ -3632,13 +3632,13 @@
         <v>0</v>
       </c>
       <c r="E54" s="3">
-        <v>844949.7187397726</v>
+        <v>844949.7187397724</v>
       </c>
       <c r="F54" s="3">
         <v>859985.8637810693</v>
       </c>
       <c r="G54" s="3">
-        <v>875763.4618273739</v>
+        <v>875763.4618273737</v>
       </c>
       <c r="H54" s="3">
         <v>891441.1643479362</v>
@@ -3662,7 +3662,7 @@
         <v>1008524.606781444</v>
       </c>
       <c r="O54" s="3">
-        <v>1028114.344485683</v>
+        <v>1028114.344485682</v>
       </c>
       <c r="P54" s="3">
         <v>1051206.173424766</v>
@@ -3724,7 +3724,7 @@
         <v>3650318.769775946</v>
       </c>
       <c r="Q55" s="3">
-        <v>3725609.553937779</v>
+        <v>3725609.553937778</v>
       </c>
       <c r="R55" s="3">
         <v>43182381.36801808</v>
@@ -3747,7 +3747,7 @@
         <v>9878270.105880328</v>
       </c>
       <c r="F56" s="3">
-        <v>9933138.270005254</v>
+        <v>9933138.270005252</v>
       </c>
       <c r="G56" s="3">
         <v>10015918.12765318</v>
@@ -3765,7 +3765,7 @@
         <v>10597637.89353936</v>
       </c>
       <c r="L56" s="3">
-        <v>10793451.24362944</v>
+        <v>10793451.24362943</v>
       </c>
       <c r="M56" s="3">
         <v>11000008.58373932</v>
@@ -3777,13 +3777,13 @@
         <v>11432768.6254344</v>
       </c>
       <c r="P56" s="3">
-        <v>11664312.65030537</v>
+        <v>11664312.65030536</v>
       </c>
       <c r="Q56" s="3">
         <v>11897467.98336907</v>
       </c>
       <c r="R56" s="3">
-        <v>149102303.3619655</v>
+        <v>149102303.3619654</v>
       </c>
     </row>
     <row r="57" spans="1:18">
@@ -3806,7 +3806,7 @@
         <v>2586677.201497451</v>
       </c>
       <c r="G57" s="3">
-        <v>2633707.696070131</v>
+        <v>2633707.696070132</v>
       </c>
       <c r="H57" s="3">
         <v>2680738.190642813</v>
@@ -3827,13 +3827,13 @@
         <v>2974678.781722068</v>
       </c>
       <c r="N57" s="3">
-        <v>3033466.899937919</v>
+        <v>3033466.89993792</v>
       </c>
       <c r="O57" s="3">
-        <v>3092255.018153772</v>
+        <v>3092255.018153771</v>
       </c>
       <c r="P57" s="3">
-        <v>3162800.760012793</v>
+        <v>3162800.760012792</v>
       </c>
       <c r="Q57" s="3">
         <v>3221588.878228643</v>
@@ -4394,7 +4394,7 @@
         <v>0.3409564297396435</v>
       </c>
       <c r="K68" s="3">
-        <v>0.3408865707214276</v>
+        <v>0.3408865707214277</v>
       </c>
       <c r="L68" s="3">
         <v>0.3406475902531179</v>
@@ -4403,7 +4403,7 @@
         <v>0.3405579695368782</v>
       </c>
       <c r="N68" s="3">
-        <v>0.3405310061340829</v>
+        <v>0.340531006134083</v>
       </c>
       <c r="O68" s="3">
         <v>0.3405317904602121</v>
@@ -4429,7 +4429,7 @@
         <v>20</v>
       </c>
       <c r="D69" s="3">
-        <v>0.04535037632743646</v>
+        <v>0.04535037632743647</v>
       </c>
       <c r="E69" s="3">
         <v>0.04516415952716646</v>
@@ -4606,10 +4606,10 @@
         <v>483657.4722049777</v>
       </c>
       <c r="G72" s="3">
-        <v>492451.2444268863</v>
+        <v>492451.2444268864</v>
       </c>
       <c r="H72" s="3">
-        <v>501245.016648795</v>
+        <v>501245.0166487951</v>
       </c>
       <c r="I72" s="3">
         <v>512237.2319261809</v>
@@ -4621,16 +4621,16 @@
         <v>532023.2194254755</v>
       </c>
       <c r="L72" s="3">
-        <v>545213.8777583386</v>
+        <v>545213.8777583385</v>
       </c>
       <c r="M72" s="3">
-        <v>556206.0930357242</v>
+        <v>556206.0930357244</v>
       </c>
       <c r="N72" s="3">
-        <v>567198.3083131101</v>
+        <v>567198.3083131103</v>
       </c>
       <c r="O72" s="3">
-        <v>578190.523590496</v>
+        <v>578190.5235904962</v>
       </c>
       <c r="P72" s="3">
         <v>591381.1819233592</v>
@@ -4665,7 +4665,7 @@
         <v>0.18698022</v>
       </c>
       <c r="H73" s="3">
-        <v>0.1869802199999999</v>
+        <v>0.18698022</v>
       </c>
       <c r="I73" s="3">
         <v>0.18698022</v>
@@ -4686,7 +4686,7 @@
         <v>0.18698022</v>
       </c>
       <c r="O73" s="3">
-        <v>0.1869802199999999</v>
+        <v>0.18698022</v>
       </c>
       <c r="P73" s="3">
         <v>0.18698022</v>
@@ -4730,7 +4730,7 @@
         <v>2558725.427536433</v>
       </c>
       <c r="K74" s="3">
-        <v>2650598.148654525</v>
+        <v>2650598.148654524</v>
       </c>
       <c r="L74" s="3">
         <v>2741307.682941661</v>
@@ -4742,7 +4742,7 @@
         <v>2933535.31226689</v>
       </c>
       <c r="O74" s="3">
-        <v>3033864.776969503</v>
+        <v>3033864.776969504</v>
       </c>
       <c r="P74" s="3">
         <v>3133930.392536641</v>
@@ -4780,7 +4780,7 @@
         <v>0.1887220562459707</v>
       </c>
       <c r="I75" s="3">
-        <v>0.1887068640814534</v>
+        <v>0.1887068640814535</v>
       </c>
       <c r="J75" s="3">
         <v>0.1886876101253084</v>
@@ -4804,7 +4804,7 @@
         <v>0.188638085652016</v>
       </c>
       <c r="Q75" s="3">
-        <v>0.1886205769816762</v>
+        <v>0.1886205769816761</v>
       </c>
       <c r="R75" s="3" t="s">
         <v>19</v>
@@ -4933,7 +4933,7 @@
         <v>29</v>
       </c>
       <c r="D78" s="3">
-        <v>0.03308146768986005</v>
+        <v>0.03308146768986006</v>
       </c>
       <c r="E78" s="3">
         <v>0.033006831257611</v>
@@ -5160,13 +5160,13 @@
         <v>0.5092287374537772</v>
       </c>
       <c r="E82" s="3">
-        <v>0.5124607711022933</v>
+        <v>0.5124607711022932</v>
       </c>
       <c r="F82" s="3">
         <v>0.5127058446112905</v>
       </c>
       <c r="G82" s="3">
-        <v>0.5126984388101171</v>
+        <v>0.512698438810117</v>
       </c>
       <c r="H82" s="3">
         <v>0.5126964299094969</v>
@@ -5390,7 +5390,7 @@
         <v>2586677.201497451</v>
       </c>
       <c r="G86" s="3">
-        <v>2633707.696070131</v>
+        <v>2633707.696070132</v>
       </c>
       <c r="H86" s="3">
         <v>2680738.190642813</v>
@@ -5411,13 +5411,13 @@
         <v>2974678.781722068</v>
       </c>
       <c r="N86" s="3">
-        <v>3033466.899937919</v>
+        <v>3033466.89993792</v>
       </c>
       <c r="O86" s="3">
-        <v>3092255.018153772</v>
+        <v>3092255.018153771</v>
       </c>
       <c r="P86" s="3">
-        <v>3162800.760012793</v>
+        <v>3162800.760012792</v>
       </c>
       <c r="Q86" s="3">
         <v>3221588.878228643</v>
@@ -5524,7 +5524,7 @@
         <v>1201603.878308399</v>
       </c>
       <c r="I89" s="3">
-        <v>1214061.196545525</v>
+        <v>1214061.196545524</v>
       </c>
       <c r="J89" s="3">
         <v>1229191.403997979</v>
@@ -5536,10 +5536,10 @@
         <v>1267445.570296652</v>
       </c>
       <c r="M89" s="3">
-        <v>1289504.118729486</v>
+        <v>1289504.118729487</v>
       </c>
       <c r="N89" s="3">
-        <v>1313456.990339579</v>
+        <v>1313456.99033958</v>
       </c>
       <c r="O89" s="3">
         <v>1338800.61647759</v>
@@ -5548,7 +5548,7 @@
         <v>1365025.022754148</v>
       </c>
       <c r="Q89" s="3">
-        <v>1392094.0338322</v>
+        <v>1392094.033832199</v>
       </c>
       <c r="R89" s="3">
         <v>16408200.1587729</v>
@@ -5577,37 +5577,37 @@
         <v>198914.0184273994</v>
       </c>
       <c r="H90" s="3">
-        <v>201915.9524810384</v>
+        <v>201915.9524810385</v>
       </c>
       <c r="I90" s="3">
-        <v>205608.0331454558</v>
+        <v>205608.0331454559</v>
       </c>
       <c r="J90" s="3">
-        <v>209575.7004475182</v>
+        <v>209575.7004475183</v>
       </c>
       <c r="K90" s="3">
         <v>213164.8608082295</v>
       </c>
       <c r="L90" s="3">
-        <v>217763.6231897639</v>
+        <v>217763.623189764</v>
       </c>
       <c r="M90" s="3">
         <v>222158.6941550838</v>
       </c>
       <c r="N90" s="3">
-        <v>226535.0603257282</v>
+        <v>226535.0603257283</v>
       </c>
       <c r="O90" s="3">
         <v>230943.1007686078</v>
       </c>
       <c r="P90" s="3">
-        <v>235905.3935391532</v>
+        <v>235905.3935391533</v>
       </c>
       <c r="Q90" s="3">
         <v>240511.519622273</v>
       </c>
       <c r="R90" s="3">
-        <v>2793145.262856409</v>
+        <v>2793145.26285641</v>
       </c>
     </row>
     <row r="91" spans="1:18">
@@ -5630,7 +5630,7 @@
         <v>762580.6474017324</v>
       </c>
       <c r="G91" s="3">
-        <v>763867.3568204551</v>
+        <v>763867.3568204549</v>
       </c>
       <c r="H91" s="3">
         <v>765864.9953420266</v>
@@ -5657,10 +5657,10 @@
         <v>841356.7138497927</v>
       </c>
       <c r="P91" s="3">
-        <v>857505.007664789</v>
+        <v>857505.0076647889</v>
       </c>
       <c r="Q91" s="3">
-        <v>874274.1214844574</v>
+        <v>874274.1214844565</v>
       </c>
       <c r="R91" s="3">
         <v>10397381.05487779</v>
@@ -5698,28 +5698,28 @@
         <v>59513.2808920886</v>
       </c>
       <c r="K92" s="3">
-        <v>60330.09710752314</v>
+        <v>60330.09710752315</v>
       </c>
       <c r="L92" s="3">
-        <v>61271.9856107551</v>
+        <v>61271.98561075512</v>
       </c>
       <c r="M92" s="3">
-        <v>62310.71940248761</v>
+        <v>62310.71940248763</v>
       </c>
       <c r="N92" s="3">
-        <v>63448.4360924403</v>
+        <v>63448.43609244031</v>
       </c>
       <c r="O92" s="3">
-        <v>64658.65832396557</v>
+        <v>64658.65832396558</v>
       </c>
       <c r="P92" s="3">
-        <v>65915.21774308685</v>
+        <v>65915.21774308688</v>
       </c>
       <c r="Q92" s="3">
-        <v>67215.26068996782</v>
+        <v>67215.26068996786</v>
       </c>
       <c r="R92" s="3">
-        <v>795052.9659205902</v>
+        <v>795052.9659205904</v>
       </c>
     </row>
     <row r="93" spans="1:18">
@@ -5751,16 +5751,16 @@
         <v>403029.625752438</v>
       </c>
       <c r="J93" s="3">
-        <v>407532.927803578</v>
+        <v>407532.9278035781</v>
       </c>
       <c r="K93" s="3">
-        <v>413126.2928267073</v>
+        <v>413126.2928267075</v>
       </c>
       <c r="L93" s="3">
-        <v>419576.1234129702</v>
+        <v>419576.1234129703</v>
       </c>
       <c r="M93" s="3">
-        <v>426689.1277207119</v>
+        <v>426689.127720712</v>
       </c>
       <c r="N93" s="3">
         <v>434479.9435977282</v>
@@ -5769,10 +5769,10 @@
         <v>442767.2603430572</v>
       </c>
       <c r="P93" s="3">
-        <v>451371.8832332351</v>
+        <v>451371.8832332353</v>
       </c>
       <c r="Q93" s="3">
-        <v>460274.2710779494</v>
+        <v>460274.2710779495</v>
       </c>
       <c r="R93" s="3">
         <v>5444335.417300256</v>
@@ -5810,7 +5810,7 @@
         <v>1598634.876683859</v>
       </c>
       <c r="K94" s="3">
-        <v>1620576.044609087</v>
+        <v>1620576.044609088</v>
       </c>
       <c r="L94" s="3">
         <v>1645876.881475138</v>
@@ -5825,13 +5825,13 @@
         <v>1736849.065063348</v>
       </c>
       <c r="P94" s="3">
-        <v>1770602.534573376</v>
+        <v>1770602.534573377</v>
       </c>
       <c r="Q94" s="3">
         <v>1805524.050660504</v>
       </c>
       <c r="R94" s="3">
-        <v>21356567.49350143</v>
+        <v>21356567.49350144</v>
       </c>
     </row>
     <row r="95" spans="1:18">
@@ -5866,22 +5866,22 @@
         <v>1946654.523595349</v>
       </c>
       <c r="K95" s="3">
-        <v>1973372.240328271</v>
+        <v>1973372.240328272</v>
       </c>
       <c r="L95" s="3">
         <v>2004181.019277353</v>
       </c>
       <c r="M95" s="3">
-        <v>2038157.567102936</v>
+        <v>2038157.567102937</v>
       </c>
       <c r="N95" s="3">
         <v>2075371.80412479</v>
       </c>
       <c r="O95" s="3">
-        <v>2114957.667082439</v>
+        <v>2114957.66708244</v>
       </c>
       <c r="P95" s="3">
-        <v>2156059.200063525</v>
+        <v>2156059.200063526</v>
       </c>
       <c r="Q95" s="3">
         <v>2198583.061048486</v>
@@ -5913,22 +5913,22 @@
         <v>921311.059982967</v>
       </c>
       <c r="H96" s="3">
-        <v>929105.380970789</v>
+        <v>929105.3809707889</v>
       </c>
       <c r="I96" s="3">
-        <v>938737.6413317267</v>
+        <v>938737.6413317265</v>
       </c>
       <c r="J96" s="3">
         <v>950436.6358282076</v>
       </c>
       <c r="K96" s="3">
-        <v>964341.6820502287</v>
+        <v>964341.6820502284</v>
       </c>
       <c r="L96" s="3">
         <v>980015.5614577453</v>
       </c>
       <c r="M96" s="3">
-        <v>997071.6948602136</v>
+        <v>997071.6948602138</v>
       </c>
       <c r="N96" s="3">
         <v>1015592.558769183</v>
@@ -5963,10 +5963,10 @@
         <v>0.3408863874357196</v>
       </c>
       <c r="F97" s="3">
-        <v>0.3396364826232976</v>
+        <v>0.3396364826232977</v>
       </c>
       <c r="G97" s="3">
-        <v>0.3376049351640145</v>
+        <v>0.3376049351640146</v>
       </c>
       <c r="H97" s="3">
         <v>0.3365104365461967</v>
@@ -5975,7 +5975,7 @@
         <v>0.3356141751963702</v>
       </c>
       <c r="J97" s="3">
-        <v>0.334961467243806</v>
+        <v>0.3349614672438061</v>
       </c>
       <c r="K97" s="3">
         <v>0.3346290556153954</v>
@@ -5993,10 +5993,10 @@
         <v>0.3338116256820459</v>
       </c>
       <c r="P97" s="3">
-        <v>0.3336777467052953</v>
+        <v>0.3336777467052952</v>
       </c>
       <c r="Q97" s="3">
-        <v>0.3336767146024854</v>
+        <v>0.3336767146024851</v>
       </c>
       <c r="R97" s="3" t="s">
         <v>19</v>
@@ -6013,7 +6013,7 @@
         <v>20</v>
       </c>
       <c r="D98" s="3">
-        <v>0.04535037632743646</v>
+        <v>0.04535037632743647</v>
       </c>
       <c r="E98" s="3">
         <v>0.04476587818302722</v>
@@ -6022,22 +6022,22 @@
         <v>0.04475181087005206</v>
       </c>
       <c r="G98" s="3">
-        <v>0.0446090350003612</v>
+        <v>0.04460903500036118</v>
       </c>
       <c r="H98" s="3">
-        <v>0.04469399078728013</v>
+        <v>0.04469399078728015</v>
       </c>
       <c r="I98" s="3">
         <v>0.04478536931799604</v>
       </c>
       <c r="J98" s="3">
-        <v>0.04485828831292442</v>
+        <v>0.0448582883129244</v>
       </c>
       <c r="K98" s="3">
         <v>0.04488246713048312</v>
       </c>
       <c r="L98" s="3">
-        <v>0.04494036525056893</v>
+        <v>0.04494036525056892</v>
       </c>
       <c r="M98" s="3">
         <v>0.04496670065853924</v>
@@ -6087,13 +6087,13 @@
         <v>0.2045028982677134</v>
       </c>
       <c r="J99" s="3">
-        <v>0.2044932158200258</v>
+        <v>0.2044932158200259</v>
       </c>
       <c r="K99" s="3">
         <v>0.2045359408250811</v>
       </c>
       <c r="L99" s="3">
-        <v>0.2044803255155197</v>
+        <v>0.2044803255155196</v>
       </c>
       <c r="M99" s="3">
         <v>0.2045008410261895</v>
@@ -6190,10 +6190,10 @@
         <v>483657.4722049777</v>
       </c>
       <c r="G101" s="3">
-        <v>492451.2444268863</v>
+        <v>492451.2444268864</v>
       </c>
       <c r="H101" s="3">
-        <v>501245.016648795</v>
+        <v>501245.0166487951</v>
       </c>
       <c r="I101" s="3">
         <v>512237.2319261809</v>
@@ -6205,16 +6205,16 @@
         <v>532023.2194254755</v>
       </c>
       <c r="L101" s="3">
-        <v>545213.8777583386</v>
+        <v>545213.8777583385</v>
       </c>
       <c r="M101" s="3">
-        <v>556206.0930357242</v>
+        <v>556206.0930357244</v>
       </c>
       <c r="N101" s="3">
-        <v>567198.3083131101</v>
+        <v>567198.3083131103</v>
       </c>
       <c r="O101" s="3">
-        <v>578190.523590496</v>
+        <v>578190.5235904962</v>
       </c>
       <c r="P101" s="3">
         <v>591381.1819233592</v>
@@ -6249,7 +6249,7 @@
         <v>0.18698022</v>
       </c>
       <c r="H102" s="3">
-        <v>0.1869802199999999</v>
+        <v>0.18698022</v>
       </c>
       <c r="I102" s="3">
         <v>0.18698022</v>
@@ -6270,7 +6270,7 @@
         <v>0.18698022</v>
       </c>
       <c r="O102" s="3">
-        <v>0.1869802199999999</v>
+        <v>0.18698022</v>
       </c>
       <c r="P102" s="3">
         <v>0.18698022</v>
@@ -6314,7 +6314,7 @@
         <v>2558725.427536433</v>
       </c>
       <c r="K103" s="3">
-        <v>2650598.148654525</v>
+        <v>2650598.148654524</v>
       </c>
       <c r="L103" s="3">
         <v>2741307.682941661</v>
@@ -6326,7 +6326,7 @@
         <v>2933535.31226689</v>
       </c>
       <c r="O103" s="3">
-        <v>3033864.776969503</v>
+        <v>3033864.776969504</v>
       </c>
       <c r="P103" s="3">
         <v>3133930.392536641</v>
@@ -6364,7 +6364,7 @@
         <v>0.1887220562459707</v>
       </c>
       <c r="I104" s="3">
-        <v>0.1887068640814534</v>
+        <v>0.1887068640814535</v>
       </c>
       <c r="J104" s="3">
         <v>0.1886876101253084</v>
@@ -6388,7 +6388,7 @@
         <v>0.188638085652016</v>
       </c>
       <c r="Q104" s="3">
-        <v>0.1886205769816762</v>
+        <v>0.1886205769816761</v>
       </c>
       <c r="R104" s="3" t="s">
         <v>19</v>
@@ -6411,40 +6411,40 @@
         <v>90.18666587979455</v>
       </c>
       <c r="F105" s="3">
-        <v>89.68949561980648</v>
+        <v>89.68949561980649</v>
       </c>
       <c r="G105" s="3">
-        <v>89.38745438141994</v>
+        <v>89.38745438141999</v>
       </c>
       <c r="H105" s="3">
-        <v>89.17466480886087</v>
+        <v>89.1746648088609</v>
       </c>
       <c r="I105" s="3">
-        <v>88.98100982143319</v>
+        <v>88.98100982143322</v>
       </c>
       <c r="J105" s="3">
-        <v>88.8190729342835</v>
+        <v>88.81907293428353</v>
       </c>
       <c r="K105" s="3">
-        <v>88.70799195348746</v>
+        <v>88.70799195348751</v>
       </c>
       <c r="L105" s="3">
-        <v>88.58720208038763</v>
+        <v>88.58720208038766</v>
       </c>
       <c r="M105" s="3">
-        <v>88.49358346504745</v>
+        <v>88.49358346504748</v>
       </c>
       <c r="N105" s="3">
-        <v>88.41819622409392</v>
+        <v>88.41819622409393</v>
       </c>
       <c r="O105" s="3">
-        <v>88.35729785259279</v>
+        <v>88.35729785259281</v>
       </c>
       <c r="P105" s="3">
-        <v>88.29587489568094</v>
+        <v>88.29587489568098</v>
       </c>
       <c r="Q105" s="3">
-        <v>88.25103516133994</v>
+        <v>88.25103516133997</v>
       </c>
       <c r="R105" s="3" t="s">
         <v>19</v>
@@ -6497,7 +6497,7 @@
         <v>0.01206517507408892</v>
       </c>
       <c r="P106" s="3">
-        <v>0.01207425870372447</v>
+        <v>0.01207425870372446</v>
       </c>
       <c r="Q106" s="3">
         <v>0.01207055677785233</v>
@@ -6517,7 +6517,7 @@
         <v>29</v>
       </c>
       <c r="D107" s="3">
-        <v>0.03308146768986005</v>
+        <v>0.03308146768986006</v>
       </c>
       <c r="E107" s="3">
         <v>0.03279287260185953</v>
@@ -6538,7 +6538,7 @@
         <v>0.03287637359337099</v>
       </c>
       <c r="K107" s="3">
-        <v>0.03289759470825739</v>
+        <v>0.03289759470825738</v>
       </c>
       <c r="L107" s="3">
         <v>0.03293322471310698</v>
@@ -6553,7 +6553,7 @@
         <v>0.03296422458456055</v>
       </c>
       <c r="P107" s="3">
-        <v>0.03297644375617336</v>
+        <v>0.03297644375617335</v>
       </c>
       <c r="Q107" s="3">
         <v>0.03297560663225818</v>
@@ -6591,7 +6591,7 @@
         <v>123361.4009352947</v>
       </c>
       <c r="J108" s="3">
-        <v>125589.4525012567</v>
+        <v>125589.4525012568</v>
       </c>
       <c r="K108" s="3">
         <v>127721.8467542922</v>
@@ -6603,7 +6603,7 @@
         <v>132916.4284555344</v>
       </c>
       <c r="N108" s="3">
-        <v>135530.3786398928</v>
+        <v>135530.3786398929</v>
       </c>
       <c r="O108" s="3">
         <v>138176.2417861391</v>
@@ -6638,7 +6638,7 @@
         <v>325763.1141498805</v>
       </c>
       <c r="G109" s="3">
-        <v>327917.4746143433</v>
+        <v>327917.4746143431</v>
       </c>
       <c r="H109" s="3">
         <v>332136.6159239307</v>
@@ -6647,13 +6647,13 @@
         <v>337365.0100616488</v>
       </c>
       <c r="J109" s="3">
-        <v>343287.0113348274</v>
+        <v>343287.0113348273</v>
       </c>
       <c r="K109" s="3">
         <v>349208.1015745864</v>
       </c>
       <c r="L109" s="3">
-        <v>356070.2815478683</v>
+        <v>356070.2815478682</v>
       </c>
       <c r="M109" s="3">
         <v>363124.7150164315</v>
@@ -6665,7 +6665,7 @@
         <v>377557.5086522197</v>
       </c>
       <c r="P109" s="3">
-        <v>385353.6303532312</v>
+        <v>385353.6303532311</v>
       </c>
       <c r="Q109" s="3">
         <v>393051.3631252338</v>
@@ -6765,16 +6765,16 @@
         <v>0.5125835546772366</v>
       </c>
       <c r="L111" s="3">
-        <v>0.5126192427393643</v>
+        <v>0.5126192427393642</v>
       </c>
       <c r="M111" s="3">
         <v>0.5126001328084887</v>
       </c>
       <c r="N111" s="3">
-        <v>0.5125970152271305</v>
+        <v>0.5125970152271304</v>
       </c>
       <c r="O111" s="3">
-        <v>0.5125950248263682</v>
+        <v>0.5125950248263683</v>
       </c>
       <c r="P111" s="3">
         <v>0.5126108461189653</v>
@@ -6806,7 +6806,7 @@
         <v>861624.5974758542</v>
       </c>
       <c r="G112" s="3">
-        <v>877441.2560309536</v>
+        <v>877441.2560309531</v>
       </c>
       <c r="H112" s="3">
         <v>893149.6069284477</v>
@@ -6815,19 +6815,19 @@
         <v>912360.9219617507</v>
       </c>
       <c r="J112" s="3">
-        <v>931958.6323450616</v>
+        <v>931958.6323450612</v>
       </c>
       <c r="K112" s="3">
-        <v>948072.1303455111</v>
+        <v>948072.1303455106</v>
       </c>
       <c r="L112" s="3">
-        <v>970821.0323227596</v>
+        <v>970821.0323227593</v>
       </c>
       <c r="M112" s="3">
-        <v>990807.4727093632</v>
+        <v>990807.4727093629</v>
       </c>
       <c r="N112" s="3">
-        <v>1010457.450631027</v>
+        <v>1010457.450631026</v>
       </c>
       <c r="O112" s="3">
         <v>1030084.740525888</v>
@@ -6862,16 +6862,16 @@
         <v>3034472.358891554</v>
       </c>
       <c r="G113" s="3">
-        <v>3069171.876611042</v>
+        <v>3069171.876611041</v>
       </c>
       <c r="H113" s="3">
-        <v>3117275.211060226</v>
+        <v>3117275.211060227</v>
       </c>
       <c r="I113" s="3">
         <v>3174411.925429798</v>
       </c>
       <c r="J113" s="3">
-        <v>3238966.550769669</v>
+        <v>3238966.550769668</v>
       </c>
       <c r="K113" s="3">
         <v>3302707.730062874</v>
@@ -6880,16 +6880,16 @@
         <v>3370166.320734185</v>
       </c>
       <c r="M113" s="3">
-        <v>3442661.243637009</v>
+        <v>3442661.243637008</v>
       </c>
       <c r="N113" s="3">
         <v>3513929.470624622</v>
       </c>
       <c r="O113" s="3">
-        <v>3584264.741125174</v>
+        <v>3584264.741125173</v>
       </c>
       <c r="P113" s="3">
-        <v>3658282.328259145</v>
+        <v>3658282.328259144</v>
       </c>
       <c r="Q113" s="3">
         <v>3733737.555874001</v>
@@ -6933,7 +6933,7 @@
         <v>10615004.06553839</v>
       </c>
       <c r="L114" s="3">
-        <v>10811886.31388888</v>
+        <v>10811886.31388887</v>
       </c>
       <c r="M114" s="3">
         <v>11019342.37072727</v>
@@ -6974,7 +6974,7 @@
         <v>2586677.201497451</v>
       </c>
       <c r="G115" s="3">
-        <v>2633707.696070131</v>
+        <v>2633707.696070132</v>
       </c>
       <c r="H115" s="3">
         <v>2680738.190642813</v>
@@ -6995,13 +6995,13 @@
         <v>2974678.781722068</v>
       </c>
       <c r="N115" s="3">
-        <v>3033466.899937919</v>
+        <v>3033466.89993792</v>
       </c>
       <c r="O115" s="3">
-        <v>3092255.018153772</v>
+        <v>3092255.018153771</v>
       </c>
       <c r="P115" s="3">
-        <v>3162800.760012793</v>
+        <v>3162800.760012792</v>
       </c>
       <c r="Q115" s="3">
         <v>3221588.878228643</v>
@@ -7120,7 +7120,7 @@
         <v>1266551.215363578</v>
       </c>
       <c r="M118" s="3">
-        <v>1288600.601820457</v>
+        <v>1288600.601820458</v>
       </c>
       <c r="N118" s="3">
         <v>1312541.537046958</v>
@@ -7132,7 +7132,7 @@
         <v>1364079.712029624</v>
       </c>
       <c r="Q118" s="3">
-        <v>1391131.719938596</v>
+        <v>1391131.719938597</v>
       </c>
       <c r="R118" s="3">
         <v>16398528.62679099</v>
@@ -7155,19 +7155,19 @@
         <v>190762.0638799602</v>
       </c>
       <c r="F119" s="3">
-        <v>193056.5863448694</v>
+        <v>193056.5863448695</v>
       </c>
       <c r="G119" s="3">
-        <v>195653.556810365</v>
+        <v>195653.5568103649</v>
       </c>
       <c r="H119" s="3">
-        <v>198599.6963100175</v>
+        <v>198599.6963100174</v>
       </c>
       <c r="I119" s="3">
         <v>202220.7979808142</v>
       </c>
       <c r="J119" s="3">
-        <v>206116.0617271804</v>
+        <v>206116.0617271803</v>
       </c>
       <c r="K119" s="3">
         <v>209648.0790329246</v>
@@ -7185,7 +7185,7 @@
         <v>227122.9416281024</v>
       </c>
       <c r="P119" s="3">
-        <v>231998.2995077868</v>
+        <v>231998.2995077869</v>
       </c>
       <c r="Q119" s="3">
         <v>236531.3514382231</v>
@@ -7217,37 +7217,37 @@
         <v>762498.8613859708</v>
       </c>
       <c r="H120" s="3">
-        <v>763708.571672269</v>
+        <v>763708.5716722688</v>
       </c>
       <c r="I120" s="3">
-        <v>767547.6706694405</v>
+        <v>767547.6706694404</v>
       </c>
       <c r="J120" s="3">
-        <v>774135.8497860425</v>
+        <v>774135.8497860424</v>
       </c>
       <c r="K120" s="3">
         <v>783312.7347266955</v>
       </c>
       <c r="L120" s="3">
-        <v>794500.2191015534</v>
+        <v>794500.2191015533</v>
       </c>
       <c r="M120" s="3">
-        <v>807224.7319449444</v>
+        <v>807224.7319449438</v>
       </c>
       <c r="N120" s="3">
-        <v>821432.9417258396</v>
+        <v>821432.9417258393</v>
       </c>
       <c r="O120" s="3">
-        <v>836723.7576784656</v>
+        <v>836723.7576784655</v>
       </c>
       <c r="P120" s="3">
         <v>852716.7416212243</v>
       </c>
       <c r="Q120" s="3">
-        <v>869345.0105757772</v>
+        <v>869345.0105757773</v>
       </c>
       <c r="R120" s="3">
-        <v>10356170.8789494</v>
+        <v>10356170.87894939</v>
       </c>
     </row>
     <row r="121" spans="1:18">
@@ -7282,7 +7282,7 @@
         <v>59440.53749792602</v>
       </c>
       <c r="K121" s="3">
-        <v>60248.41793162135</v>
+        <v>60248.41793162134</v>
       </c>
       <c r="L121" s="3">
         <v>61183.3222425783</v>
@@ -7291,7 +7291,7 @@
         <v>62216.49404473905</v>
       </c>
       <c r="N121" s="3">
-        <v>63349.6250394298</v>
+        <v>63349.62503942979</v>
       </c>
       <c r="O121" s="3">
         <v>64555.9468291604</v>
@@ -7300,10 +7300,10 @@
         <v>65809.09214197034</v>
       </c>
       <c r="Q121" s="3">
-        <v>67106.04560093138</v>
+        <v>67106.04560093136</v>
       </c>
       <c r="R121" s="3">
-        <v>794142.6087822343</v>
+        <v>794142.6087822341</v>
       </c>
     </row>
     <row r="122" spans="1:18">
@@ -7329,13 +7329,13 @@
         <v>397004.6927059512</v>
       </c>
       <c r="H122" s="3">
-        <v>399302.5274940203</v>
+        <v>399302.5274940202</v>
       </c>
       <c r="I122" s="3">
         <v>402610.0348860169</v>
       </c>
       <c r="J122" s="3">
-        <v>407034.7981767608</v>
+        <v>407034.7981767607</v>
       </c>
       <c r="K122" s="3">
         <v>412566.9730715724</v>
@@ -7412,10 +7412,10 @@
         <v>1767751.808068119</v>
       </c>
       <c r="Q123" s="3">
-        <v>1802590.334895272</v>
+        <v>1802590.334895271</v>
       </c>
       <c r="R123" s="3">
-        <v>21332113.64639707</v>
+        <v>21332113.64639706</v>
       </c>
     </row>
     <row r="124" spans="1:18">
@@ -7444,13 +7444,13 @@
         <v>1907340.532257394</v>
       </c>
       <c r="I124" s="3">
-        <v>1923139.437786713</v>
+        <v>1923139.437786712</v>
       </c>
       <c r="J124" s="3">
         <v>1944275.117600827</v>
       </c>
       <c r="K124" s="3">
-        <v>1970700.548650895</v>
+        <v>1970700.548650894</v>
       </c>
       <c r="L124" s="3">
         <v>2001280.877592145</v>
@@ -7465,7 +7465,7 @@
         <v>2111598.017051545</v>
       </c>
       <c r="P124" s="3">
-        <v>2152587.876043306</v>
+        <v>2152587.876043305</v>
       </c>
       <c r="Q124" s="3">
         <v>2195010.681170736</v>
@@ -7494,25 +7494,25 @@
         <v>914477.8237756658</v>
       </c>
       <c r="G125" s="3">
-        <v>920944.5471100379</v>
+        <v>920944.547110038</v>
       </c>
       <c r="H125" s="3">
-        <v>928576.7368011813</v>
+        <v>928576.7368011812</v>
       </c>
       <c r="I125" s="3">
         <v>938084.4557845545</v>
       </c>
       <c r="J125" s="3">
-        <v>949753.6671787186</v>
+        <v>949753.6671787187</v>
       </c>
       <c r="K125" s="3">
-        <v>963655.1068277928</v>
+        <v>963655.1068277929</v>
       </c>
       <c r="L125" s="3">
-        <v>979324.0274207657</v>
+        <v>979324.027420766</v>
       </c>
       <c r="M125" s="3">
-        <v>996373.0765908066</v>
+        <v>996373.0765908067</v>
       </c>
       <c r="N125" s="3">
         <v>1014884.711037034</v>
@@ -7524,7 +7524,7 @@
         <v>1054735.111461191</v>
       </c>
       <c r="Q125" s="3">
-        <v>1075652.292712032</v>
+        <v>1075652.292712033</v>
       </c>
       <c r="R125" s="3">
         <v>12679687.09339055</v>
@@ -7550,13 +7550,13 @@
         <v>0.3389468894761283</v>
       </c>
       <c r="G126" s="3">
-        <v>0.3364961427306638</v>
+        <v>0.3364961427306637</v>
       </c>
       <c r="H126" s="3">
-        <v>0.3352073226134445</v>
+        <v>0.3352073226134446</v>
       </c>
       <c r="I126" s="3">
-        <v>0.3341735529649525</v>
+        <v>0.3341735529649524</v>
       </c>
       <c r="J126" s="3">
         <v>0.3334238082109685</v>
@@ -7565,13 +7565,13 @@
         <v>0.3330224862615002</v>
       </c>
       <c r="L126" s="3">
-        <v>0.332556255997532</v>
+        <v>0.3325562559975319</v>
       </c>
       <c r="M126" s="3">
-        <v>0.3323043783539585</v>
+        <v>0.3323043783539584</v>
       </c>
       <c r="N126" s="3">
-        <v>0.3321635783896118</v>
+        <v>0.3321635783896117</v>
       </c>
       <c r="O126" s="3">
         <v>0.3320847899197073</v>
@@ -7597,7 +7597,7 @@
         <v>20</v>
       </c>
       <c r="D127" s="3">
-        <v>0.04535037632743646</v>
+        <v>0.04535037632743647</v>
       </c>
       <c r="E127" s="3">
         <v>0.04468776814709099</v>
@@ -7627,16 +7627,16 @@
         <v>0.0448399065346138</v>
       </c>
       <c r="N127" s="3">
-        <v>0.04485041902186661</v>
+        <v>0.04485041902186662</v>
       </c>
       <c r="O127" s="3">
-        <v>0.04485227548567668</v>
+        <v>0.04485227548567667</v>
       </c>
       <c r="P127" s="3">
         <v>0.04487353479687993</v>
       </c>
       <c r="Q127" s="3">
-        <v>0.04486882366636283</v>
+        <v>0.04486882366636284</v>
       </c>
       <c r="R127" s="3" t="s">
         <v>19</v>
@@ -7683,7 +7683,7 @@
         <v>0.2038284784820326</v>
       </c>
       <c r="N128" s="3">
-        <v>0.2038425305268522</v>
+        <v>0.2038425305268521</v>
       </c>
       <c r="O128" s="3">
         <v>0.2038517323186693</v>
@@ -7774,10 +7774,10 @@
         <v>483657.4722049777</v>
       </c>
       <c r="G130" s="3">
-        <v>492451.2444268863</v>
+        <v>492451.2444268864</v>
       </c>
       <c r="H130" s="3">
-        <v>501245.016648795</v>
+        <v>501245.0166487951</v>
       </c>
       <c r="I130" s="3">
         <v>512237.2319261809</v>
@@ -7789,16 +7789,16 @@
         <v>532023.2194254755</v>
       </c>
       <c r="L130" s="3">
-        <v>545213.8777583386</v>
+        <v>545213.8777583385</v>
       </c>
       <c r="M130" s="3">
-        <v>556206.0930357242</v>
+        <v>556206.0930357244</v>
       </c>
       <c r="N130" s="3">
-        <v>567198.3083131101</v>
+        <v>567198.3083131103</v>
       </c>
       <c r="O130" s="3">
-        <v>578190.523590496</v>
+        <v>578190.5235904962</v>
       </c>
       <c r="P130" s="3">
         <v>591381.1819233592</v>
@@ -7833,7 +7833,7 @@
         <v>0.18698022</v>
       </c>
       <c r="H131" s="3">
-        <v>0.1869802199999999</v>
+        <v>0.18698022</v>
       </c>
       <c r="I131" s="3">
         <v>0.18698022</v>
@@ -7854,7 +7854,7 @@
         <v>0.18698022</v>
       </c>
       <c r="O131" s="3">
-        <v>0.1869802199999999</v>
+        <v>0.18698022</v>
       </c>
       <c r="P131" s="3">
         <v>0.18698022</v>
@@ -7898,7 +7898,7 @@
         <v>2558725.427536433</v>
       </c>
       <c r="K132" s="3">
-        <v>2650598.148654525</v>
+        <v>2650598.148654524</v>
       </c>
       <c r="L132" s="3">
         <v>2741307.682941661</v>
@@ -7910,7 +7910,7 @@
         <v>2933535.31226689</v>
       </c>
       <c r="O132" s="3">
-        <v>3033864.776969503</v>
+        <v>3033864.776969504</v>
       </c>
       <c r="P132" s="3">
         <v>3133930.392536641</v>
@@ -7948,7 +7948,7 @@
         <v>0.1887220562459707</v>
       </c>
       <c r="I133" s="3">
-        <v>0.1887068640814534</v>
+        <v>0.1887068640814535</v>
       </c>
       <c r="J133" s="3">
         <v>0.1886876101253084</v>
@@ -7972,7 +7972,7 @@
         <v>0.188638085652016</v>
       </c>
       <c r="Q133" s="3">
-        <v>0.1886205769816762</v>
+        <v>0.1886205769816761</v>
       </c>
       <c r="R133" s="3" t="s">
         <v>19</v>
@@ -7995,16 +7995,16 @@
         <v>88.72654133951639</v>
       </c>
       <c r="F134" s="3">
-        <v>88.23417246547808</v>
+        <v>88.23417246547811</v>
       </c>
       <c r="G134" s="3">
-        <v>87.93204962597794</v>
+        <v>87.93204962597795</v>
       </c>
       <c r="H134" s="3">
         <v>87.71949304906563</v>
       </c>
       <c r="I134" s="3">
-        <v>87.52613404696663</v>
+        <v>87.52613404696665</v>
       </c>
       <c r="J134" s="3">
         <v>87.36441554147325</v>
@@ -8016,10 +8016,10 @@
         <v>87.13299415932229</v>
       </c>
       <c r="M134" s="3">
-        <v>87.03950391098054</v>
+        <v>87.03950391098056</v>
       </c>
       <c r="N134" s="3">
-        <v>86.96425453377832</v>
+        <v>86.96425453377833</v>
       </c>
       <c r="O134" s="3">
         <v>86.90349756216374</v>
@@ -8101,7 +8101,7 @@
         <v>29</v>
       </c>
       <c r="D136" s="3">
-        <v>0.03308146768986005</v>
+        <v>0.03308146768986006</v>
       </c>
       <c r="E136" s="3">
         <v>0.03267881117033483</v>
@@ -8110,7 +8110,7 @@
         <v>0.03263661469404588</v>
       </c>
       <c r="G136" s="3">
-        <v>0.03250213986460572</v>
+        <v>0.03250213986460573</v>
       </c>
       <c r="H136" s="3">
         <v>0.03255885054524994</v>
@@ -8125,16 +8125,16 @@
         <v>0.03268801773372466</v>
       </c>
       <c r="L136" s="3">
-        <v>0.03272324058997546</v>
+        <v>0.03272324058997545</v>
       </c>
       <c r="M136" s="3">
         <v>0.03274287742891711</v>
       </c>
       <c r="N136" s="3">
-        <v>0.03275120440167462</v>
+        <v>0.03275120440167463</v>
       </c>
       <c r="O136" s="3">
-        <v>0.03275323450866797</v>
+        <v>0.03275323450866796</v>
       </c>
       <c r="P136" s="3">
         <v>0.03276540140416852</v>
@@ -8166,7 +8166,7 @@
         <v>118819.9168480144</v>
       </c>
       <c r="G137" s="3">
-        <v>119018.0364075176</v>
+        <v>119018.0364075175</v>
       </c>
       <c r="H137" s="3">
         <v>120636.1787344728</v>
@@ -8234,13 +8234,13 @@
         <v>341233.5563151515</v>
       </c>
       <c r="K138" s="3">
-        <v>347116.8108893561</v>
+        <v>347116.8108893562</v>
       </c>
       <c r="L138" s="3">
         <v>353939.2316736339</v>
       </c>
       <c r="M138" s="3">
-        <v>360949.1944423882</v>
+        <v>360949.1944423883</v>
       </c>
       <c r="N138" s="3">
         <v>368077.3935650637</v>
@@ -8249,10 +8249,10 @@
         <v>375293.3702503165</v>
       </c>
       <c r="P138" s="3">
-        <v>383043.6633793371</v>
+        <v>383043.6633793372</v>
       </c>
       <c r="Q138" s="3">
-        <v>390693.6372366435</v>
+        <v>390693.6372366436</v>
       </c>
       <c r="R138" s="3" t="s">
         <v>19</v>
@@ -8272,16 +8272,16 @@
         <v>0</v>
       </c>
       <c r="E139" s="3">
-        <v>67241.04651188724</v>
+        <v>67241.04651188725</v>
       </c>
       <c r="F139" s="3">
-        <v>68804.79177960554</v>
+        <v>68804.79177960556</v>
       </c>
       <c r="G139" s="3">
         <v>70055.78799378021</v>
       </c>
       <c r="H139" s="3">
-        <v>71306.78420795484</v>
+        <v>71306.78420795486</v>
       </c>
       <c r="I139" s="3">
         <v>72870.52947567316</v>
@@ -8293,7 +8293,7 @@
         <v>75685.27095756611</v>
       </c>
       <c r="L139" s="3">
-        <v>77561.76527882808</v>
+        <v>77561.7652788281</v>
       </c>
       <c r="M139" s="3">
         <v>79125.51054654639</v>
@@ -8305,10 +8305,10 @@
         <v>82253.00108198301</v>
       </c>
       <c r="P139" s="3">
-        <v>84129.49540324498</v>
+        <v>84129.49540324499</v>
       </c>
       <c r="Q139" s="3">
-        <v>85693.24067096328</v>
+        <v>85693.24067096329</v>
       </c>
       <c r="R139" s="3">
         <v>989850.7544656891</v>
@@ -8387,19 +8387,19 @@
         <v>844949.7187397976</v>
       </c>
       <c r="F141" s="3">
-        <v>859985.8637811218</v>
+        <v>859985.8637811216</v>
       </c>
       <c r="G141" s="3">
-        <v>875763.4618274552</v>
+        <v>875763.4618274551</v>
       </c>
       <c r="H141" s="3">
         <v>891441.1643480208</v>
       </c>
       <c r="I141" s="3">
-        <v>910615.7495797478</v>
+        <v>910615.7495797476</v>
       </c>
       <c r="J141" s="3">
-        <v>930175.9722622737</v>
+        <v>930175.9722622735</v>
       </c>
       <c r="K141" s="3">
         <v>946258.5765052406</v>
@@ -8408,7 +8408,7 @@
         <v>968964.0769107188</v>
       </c>
       <c r="M141" s="3">
-        <v>988912.2314474944</v>
+        <v>988912.2314474941</v>
       </c>
       <c r="N141" s="3">
         <v>1008524.60678154</v>
@@ -8443,22 +8443,22 @@
         <v>3027123.019928549</v>
       </c>
       <c r="F142" s="3">
-        <v>3030076.421524487</v>
+        <v>3030076.421524486</v>
       </c>
       <c r="G142" s="3">
-        <v>3063677.821360072</v>
+        <v>3063677.821360071</v>
       </c>
       <c r="H142" s="3">
         <v>3111297.38954731</v>
       </c>
       <c r="I142" s="3">
-        <v>3168182.124352902</v>
+        <v>3168182.124352901</v>
       </c>
       <c r="J142" s="3">
         <v>3232560.172133284</v>
       </c>
       <c r="K142" s="3">
-        <v>3296157.526507151</v>
+        <v>3296157.52650715</v>
       </c>
       <c r="L142" s="3">
         <v>3363476.491624252</v>
@@ -8467,13 +8467,13 @@
         <v>3435825.617777915</v>
       </c>
       <c r="N142" s="3">
-        <v>3506951.443145812</v>
+        <v>3506951.443145811</v>
       </c>
       <c r="O142" s="3">
         <v>3577146.554356871</v>
       </c>
       <c r="P142" s="3">
-        <v>3651017.242495343</v>
+        <v>3651017.242495342</v>
       </c>
       <c r="Q142" s="3">
         <v>3726322.529416781</v>
@@ -8499,7 +8499,7 @@
         <v>9878510.617419982</v>
       </c>
       <c r="F143" s="3">
-        <v>9933673.463728165</v>
+        <v>9933673.463728163</v>
       </c>
       <c r="G143" s="3">
         <v>10016893.87437631</v>
@@ -8526,7 +8526,7 @@
         <v>11216623.35636714</v>
       </c>
       <c r="O143" s="3">
-        <v>11435560.76993702</v>
+        <v>11435560.76993703</v>
       </c>
       <c r="P143" s="3">
         <v>11667210.0215381</v>
@@ -8558,7 +8558,7 @@
         <v>2586677.201497451</v>
       </c>
       <c r="G144" s="3">
-        <v>2633707.696070131</v>
+        <v>2633707.696070132</v>
       </c>
       <c r="H144" s="3">
         <v>2680738.190642813</v>
@@ -8579,13 +8579,13 @@
         <v>2974678.781722068</v>
       </c>
       <c r="N144" s="3">
-        <v>3033466.899937919</v>
+        <v>3033466.89993792</v>
       </c>
       <c r="O144" s="3">
-        <v>3092255.018153772</v>
+        <v>3092255.018153771</v>
       </c>
       <c r="P144" s="3">
-        <v>3162800.760012793</v>
+        <v>3162800.760012792</v>
       </c>
       <c r="Q144" s="3">
         <v>3221588.878228643</v>
@@ -8695,7 +8695,7 @@
         <v>1216198.707839487</v>
       </c>
       <c r="J147" s="3">
-        <v>1231799.725624779</v>
+        <v>1231799.725624778</v>
       </c>
       <c r="K147" s="3">
         <v>1250185.044388702</v>
@@ -8748,7 +8748,7 @@
         <v>205414.6726210008</v>
       </c>
       <c r="I148" s="3">
-        <v>209155.7802747746</v>
+        <v>209155.7802747747</v>
       </c>
       <c r="J148" s="3">
         <v>213179.5638264837</v>
@@ -8757,7 +8757,7 @@
         <v>216818.6212897463</v>
       </c>
       <c r="L148" s="3">
-        <v>221494.0810099026</v>
+        <v>221494.0810099027</v>
       </c>
       <c r="M148" s="3">
         <v>225957.9729237889</v>
@@ -8766,13 +8766,13 @@
         <v>230405.1775846198</v>
       </c>
       <c r="O148" s="3">
-        <v>234885.8451705683</v>
+        <v>234885.8451705684</v>
       </c>
       <c r="P148" s="3">
-        <v>239933.5182369304</v>
+        <v>239933.5182369305</v>
       </c>
       <c r="Q148" s="3">
-        <v>244614.7738682946</v>
+        <v>244614.7738682947</v>
       </c>
       <c r="R148" s="3">
         <v>2841225.961816652</v>
@@ -8801,22 +8801,22 @@
         <v>764091.0533268012</v>
       </c>
       <c r="H149" s="3">
-        <v>766156.0632878313</v>
+        <v>766156.0632878314</v>
       </c>
       <c r="I149" s="3">
-        <v>770712.4923051612</v>
+        <v>770712.4923051613</v>
       </c>
       <c r="J149" s="3">
         <v>777864.8597453295</v>
       </c>
       <c r="K149" s="3">
-        <v>787481.3564118391</v>
+        <v>787481.3564118394</v>
       </c>
       <c r="L149" s="3">
-        <v>799014.3321307347</v>
+        <v>799014.3321307349</v>
       </c>
       <c r="M149" s="3">
-        <v>812015.9824685317</v>
+        <v>812015.9824685318</v>
       </c>
       <c r="N149" s="3">
         <v>826454.6575815515</v>
@@ -8825,13 +8825,13 @@
         <v>841942.852128499</v>
       </c>
       <c r="P149" s="3">
-        <v>858109.2956742696</v>
+        <v>858109.2956742699</v>
       </c>
       <c r="Q149" s="3">
-        <v>874894.9510691173</v>
+        <v>874894.951069118</v>
       </c>
       <c r="R149" s="3">
-        <v>10402809.42816069</v>
+        <v>10402809.4281607</v>
       </c>
     </row>
     <row r="150" spans="1:18">
@@ -8854,22 +8854,22 @@
         <v>57720.17791769715</v>
       </c>
       <c r="G150" s="3">
-        <v>58022.25857297828</v>
+        <v>58022.25857297827</v>
       </c>
       <c r="H150" s="3">
         <v>58391.95262079508</v>
       </c>
       <c r="I150" s="3">
-        <v>58905.31192832348</v>
+        <v>58905.31192832346</v>
       </c>
       <c r="J150" s="3">
-        <v>59575.95526480076</v>
+        <v>59575.95526480075</v>
       </c>
       <c r="K150" s="3">
-        <v>60403.01178391022</v>
+        <v>60403.01178391021</v>
       </c>
       <c r="L150" s="3">
-        <v>61352.91358999241</v>
+        <v>61352.91358999239</v>
       </c>
       <c r="M150" s="3">
         <v>62397.99033640627</v>
@@ -8887,7 +8887,7 @@
         <v>67319.01748221171</v>
       </c>
       <c r="R150" s="3">
-        <v>795853.5036691326</v>
+        <v>795853.5036691325</v>
       </c>
     </row>
     <row r="151" spans="1:18">
@@ -8910,7 +8910,7 @@
         <v>395254.181042295</v>
       </c>
       <c r="G151" s="3">
-        <v>397322.7582074954</v>
+        <v>397322.7582074953</v>
       </c>
       <c r="H151" s="3">
         <v>399854.335956864</v>
@@ -8919,13 +8919,13 @@
         <v>403369.6995610251</v>
       </c>
       <c r="J151" s="3">
-        <v>407962.1071434961</v>
+        <v>407962.107143496</v>
       </c>
       <c r="K151" s="3">
-        <v>413625.5953538481</v>
+        <v>413625.595353848</v>
       </c>
       <c r="L151" s="3">
-        <v>420130.2991503084</v>
+        <v>420130.2991503082</v>
       </c>
       <c r="M151" s="3">
         <v>427286.7385174765</v>
@@ -8940,10 +8940,10 @@
         <v>452059.8945648244</v>
       </c>
       <c r="Q151" s="3">
-        <v>460984.7731488957</v>
+        <v>460984.7731488956</v>
       </c>
       <c r="R151" s="3">
-        <v>5449817.311216876</v>
+        <v>5449817.311216875</v>
       </c>
     </row>
     <row r="152" spans="1:18">
@@ -8996,7 +8996,7 @@
         <v>1773301.405842896</v>
       </c>
       <c r="Q152" s="3">
-        <v>1808311.146654667</v>
+        <v>1808311.146654666</v>
       </c>
       <c r="R152" s="3">
         <v>21378071.39222349</v>
@@ -9078,22 +9078,22 @@
         <v>915173.3316080007</v>
       </c>
       <c r="G154" s="3">
-        <v>922191.1704406879</v>
+        <v>922191.170440688</v>
       </c>
       <c r="H154" s="3">
         <v>930410.37599241</v>
       </c>
       <c r="I154" s="3">
-        <v>940390.410002799</v>
+        <v>940390.4100027987</v>
       </c>
       <c r="J154" s="3">
-        <v>952453.4449468444</v>
+        <v>952453.444946844</v>
       </c>
       <c r="K154" s="3">
-        <v>966669.3599441164</v>
+        <v>966669.3599441161</v>
       </c>
       <c r="L154" s="3">
-        <v>982585.763414868</v>
+        <v>982585.7634148679</v>
       </c>
       <c r="M154" s="3">
         <v>999833.6306313332</v>
@@ -9105,10 +9105,10 @@
         <v>1038238.006361108</v>
       </c>
       <c r="P154" s="3">
-        <v>1058627.982030107</v>
+        <v>1058627.982030106</v>
       </c>
       <c r="Q154" s="3">
-        <v>1079658.5745306</v>
+        <v>1079658.574530599</v>
       </c>
       <c r="R154" s="3">
         <v>12713720.32715764</v>
@@ -9134,16 +9134,16 @@
         <v>0.3396807803569109</v>
       </c>
       <c r="G155" s="3">
-        <v>0.3376577380460396</v>
+        <v>0.3376577380460397</v>
       </c>
       <c r="H155" s="3">
         <v>0.3365783002992578</v>
       </c>
       <c r="I155" s="3">
-        <v>0.3356929199358225</v>
+        <v>0.3356929199358226</v>
       </c>
       <c r="J155" s="3">
-        <v>0.3350478859262347</v>
+        <v>0.3350478859262346</v>
       </c>
       <c r="K155" s="3">
         <v>0.3347207001671181</v>
@@ -9158,13 +9158,13 @@
         <v>0.3339735142611333</v>
       </c>
       <c r="O155" s="3">
-        <v>0.333912299823017</v>
+        <v>0.3339122998230169</v>
       </c>
       <c r="P155" s="3">
         <v>0.3337792455845593</v>
       </c>
       <c r="Q155" s="3">
-        <v>0.3337787335343444</v>
+        <v>0.3337787335343445</v>
       </c>
       <c r="R155" s="3" t="s">
         <v>19</v>
@@ -9181,7 +9181,7 @@
         <v>20</v>
       </c>
       <c r="D156" s="3">
-        <v>0.04535037632743646</v>
+        <v>0.04535037632743647</v>
       </c>
       <c r="E156" s="3">
         <v>0.04483196923623563</v>
@@ -9190,16 +9190,16 @@
         <v>0.04483336269264667</v>
       </c>
       <c r="G156" s="3">
-        <v>0.04474721103719077</v>
+        <v>0.04474721103719076</v>
       </c>
       <c r="H156" s="3">
         <v>0.04483805491137387</v>
       </c>
       <c r="I156" s="3">
-        <v>0.04493453742934583</v>
+        <v>0.04493453742934582</v>
       </c>
       <c r="J156" s="3">
-        <v>0.04501150468810938</v>
+        <v>0.04501150468810939</v>
       </c>
       <c r="K156" s="3">
         <v>0.04503862200316668</v>
@@ -9217,10 +9217,10 @@
         <v>0.04514003418462223</v>
       </c>
       <c r="P156" s="3">
-        <v>0.04516172149941126</v>
+        <v>0.04516172149941125</v>
       </c>
       <c r="Q156" s="3">
-        <v>0.04515725955180034</v>
+        <v>0.04515725955180035</v>
       </c>
       <c r="R156" s="3" t="s">
         <v>19</v>
@@ -9243,7 +9243,7 @@
         <v>0.2121103230619991</v>
       </c>
       <c r="F157" s="3">
-        <v>0.2101581151596921</v>
+        <v>0.2101581151596922</v>
       </c>
       <c r="G157" s="3">
         <v>0.2051666277023231</v>
@@ -9358,10 +9358,10 @@
         <v>483657.4722049777</v>
       </c>
       <c r="G159" s="3">
-        <v>492451.2444268863</v>
+        <v>492451.2444268864</v>
       </c>
       <c r="H159" s="3">
-        <v>501245.016648795</v>
+        <v>501245.0166487951</v>
       </c>
       <c r="I159" s="3">
         <v>512237.2319261809</v>
@@ -9373,16 +9373,16 @@
         <v>532023.2194254755</v>
       </c>
       <c r="L159" s="3">
-        <v>545213.8777583386</v>
+        <v>545213.8777583385</v>
       </c>
       <c r="M159" s="3">
-        <v>556206.0930357242</v>
+        <v>556206.0930357244</v>
       </c>
       <c r="N159" s="3">
-        <v>567198.3083131101</v>
+        <v>567198.3083131103</v>
       </c>
       <c r="O159" s="3">
-        <v>578190.523590496</v>
+        <v>578190.5235904962</v>
       </c>
       <c r="P159" s="3">
         <v>591381.1819233592</v>
@@ -9417,7 +9417,7 @@
         <v>0.18698022</v>
       </c>
       <c r="H160" s="3">
-        <v>0.1869802199999999</v>
+        <v>0.18698022</v>
       </c>
       <c r="I160" s="3">
         <v>0.18698022</v>
@@ -9438,7 +9438,7 @@
         <v>0.18698022</v>
       </c>
       <c r="O160" s="3">
-        <v>0.1869802199999999</v>
+        <v>0.18698022</v>
       </c>
       <c r="P160" s="3">
         <v>0.18698022</v>
@@ -9482,7 +9482,7 @@
         <v>2558725.427536433</v>
       </c>
       <c r="K161" s="3">
-        <v>2650598.148654525</v>
+        <v>2650598.148654524</v>
       </c>
       <c r="L161" s="3">
         <v>2741307.682941661</v>
@@ -9494,7 +9494,7 @@
         <v>2933535.31226689</v>
       </c>
       <c r="O161" s="3">
-        <v>3033864.776969503</v>
+        <v>3033864.776969504</v>
       </c>
       <c r="P161" s="3">
         <v>3133930.392536641</v>
@@ -9532,7 +9532,7 @@
         <v>0.1887220562459707</v>
       </c>
       <c r="I162" s="3">
-        <v>0.1887068640814534</v>
+        <v>0.1887068640814535</v>
       </c>
       <c r="J162" s="3">
         <v>0.1886876101253084</v>
@@ -9556,7 +9556,7 @@
         <v>0.188638085652016</v>
       </c>
       <c r="Q162" s="3">
-        <v>0.1886205769816762</v>
+        <v>0.1886205769816761</v>
       </c>
       <c r="R162" s="3" t="s">
         <v>19</v>
@@ -9588,31 +9588,31 @@
         <v>90.73062318281197</v>
       </c>
       <c r="I163" s="3">
-        <v>90.53003642020686</v>
+        <v>90.53003642020687</v>
       </c>
       <c r="J163" s="3">
         <v>90.36200086397648</v>
       </c>
       <c r="K163" s="3">
-        <v>90.24591206390917</v>
+        <v>90.24591206390919</v>
       </c>
       <c r="L163" s="3">
-        <v>90.12059924418016</v>
+        <v>90.12059924418017</v>
       </c>
       <c r="M163" s="3">
-        <v>90.0231626347567</v>
+        <v>90.02316263475672</v>
       </c>
       <c r="N163" s="3">
-        <v>89.94454533873922</v>
+        <v>89.94454533873923</v>
       </c>
       <c r="O163" s="3">
-        <v>89.88091799051969</v>
+        <v>89.88091799051972</v>
       </c>
       <c r="P163" s="3">
-        <v>89.81705942401787</v>
+        <v>89.8170594240179</v>
       </c>
       <c r="Q163" s="3">
-        <v>89.77017256924648</v>
+        <v>89.7701725692465</v>
       </c>
       <c r="R163" s="3" t="s">
         <v>19</v>
@@ -9685,7 +9685,7 @@
         <v>29</v>
       </c>
       <c r="D165" s="3">
-        <v>0.03308146768986005</v>
+        <v>0.03308146768986006</v>
       </c>
       <c r="E165" s="3">
         <v>0.03285048886906182</v>
@@ -9724,7 +9724,7 @@
         <v>0.03309097422263469</v>
       </c>
       <c r="Q165" s="3">
-        <v>0.03309010759344662</v>
+        <v>0.03309010759344663</v>
       </c>
       <c r="R165" s="3" t="s">
         <v>19</v>
@@ -9806,7 +9806,7 @@
         <v>326414.6776217115</v>
       </c>
       <c r="G167" s="3">
-        <v>328917.8903527489</v>
+        <v>328917.8903527487</v>
       </c>
       <c r="H167" s="3">
         <v>333161.5925124681</v>
@@ -9815,16 +9815,16 @@
         <v>338416.1604801377</v>
       </c>
       <c r="J167" s="3">
-        <v>344363.7824956931</v>
+        <v>344363.782495693</v>
       </c>
       <c r="K167" s="3">
-        <v>350304.7293682682</v>
+        <v>350304.7293682681</v>
       </c>
       <c r="L167" s="3">
-        <v>357193.933193537</v>
+        <v>357193.9331935369</v>
       </c>
       <c r="M167" s="3">
-        <v>364272.9089455821</v>
+        <v>364272.908945582</v>
       </c>
       <c r="N167" s="3">
         <v>371468.3171072938</v>
@@ -9856,7 +9856,7 @@
         <v>0</v>
       </c>
       <c r="E168" s="3">
-        <v>67455.19711575106</v>
+        <v>67455.19711575107</v>
       </c>
       <c r="F168" s="3">
         <v>69023.92263007084</v>
@@ -9868,34 +9868,34 @@
         <v>71533.88345298251</v>
       </c>
       <c r="I168" s="3">
-        <v>73102.60896730229</v>
+        <v>73102.60896730231</v>
       </c>
       <c r="J168" s="3">
-        <v>74671.33448162208</v>
+        <v>74671.33448162209</v>
       </c>
       <c r="K168" s="3">
-        <v>75926.31489307791</v>
+        <v>75926.31489307793</v>
       </c>
       <c r="L168" s="3">
-        <v>77808.78551026167</v>
+        <v>77808.78551026169</v>
       </c>
       <c r="M168" s="3">
-        <v>79377.51102458146</v>
+        <v>79377.51102458147</v>
       </c>
       <c r="N168" s="3">
-        <v>80946.23653890126</v>
+        <v>80946.23653890127</v>
       </c>
       <c r="O168" s="3">
-        <v>82514.96205322104</v>
+        <v>82514.96205322105</v>
       </c>
       <c r="P168" s="3">
-        <v>84397.43267040479</v>
+        <v>84397.43267040481</v>
       </c>
       <c r="Q168" s="3">
-        <v>85966.15818472458</v>
+        <v>85966.1581847246</v>
       </c>
       <c r="R168" s="3">
-        <v>993003.2505644283</v>
+        <v>993003.2505644284</v>
       </c>
     </row>
     <row r="169" spans="1:18">
@@ -9924,10 +9924,10 @@
         <v>0.5126964299094924</v>
       </c>
       <c r="I169" s="3">
-        <v>0.5127152811860275</v>
+        <v>0.5127152811860274</v>
       </c>
       <c r="J169" s="3">
-        <v>0.5127143392612276</v>
+        <v>0.5127143392612277</v>
       </c>
       <c r="K169" s="3">
         <v>0.5126925644627411</v>
@@ -9948,7 +9948,7 @@
         <v>0.5127198849556622</v>
       </c>
       <c r="Q169" s="3">
-        <v>0.5127012631844541</v>
+        <v>0.512701263184454</v>
       </c>
       <c r="R169" s="3" t="s">
         <v>19</v>
@@ -9971,10 +9971,10 @@
         <v>847532.5702609476</v>
       </c>
       <c r="F170" s="3">
-        <v>862846.5507570901</v>
+        <v>862846.5507570899</v>
       </c>
       <c r="G170" s="3">
-        <v>878692.3062854472</v>
+        <v>878692.306285447</v>
       </c>
       <c r="H170" s="3">
         <v>894423.510292002</v>
@@ -9983,7 +9983,7 @@
         <v>913662.1955124481</v>
       </c>
       <c r="J170" s="3">
-        <v>933287.857773056</v>
+        <v>933287.8577730561</v>
       </c>
       <c r="K170" s="3">
         <v>949424.4124160392</v>
@@ -9992,7 +9992,7 @@
         <v>972205.6433318784</v>
       </c>
       <c r="M170" s="3">
-        <v>992220.647535064</v>
+        <v>992220.6475350641</v>
       </c>
       <c r="N170" s="3">
         <v>1011898.668175257</v>
@@ -10030,10 +10030,10 @@
         <v>3036996.449025948</v>
       </c>
       <c r="G171" s="3">
-        <v>3072467.326669153</v>
+        <v>3072467.326669152</v>
       </c>
       <c r="H171" s="3">
-        <v>3120909.239416876</v>
+        <v>3120909.239416875</v>
       </c>
       <c r="I171" s="3">
         <v>3178216.918012697</v>
@@ -10060,7 +10060,7 @@
         <v>3662731.610460706</v>
       </c>
       <c r="Q171" s="3">
-        <v>3738278.584486744</v>
+        <v>3738278.584486745</v>
       </c>
       <c r="R171" s="3">
         <v>43317363.47139777</v>
@@ -10083,7 +10083,7 @@
         <v>9884953.353417039</v>
       </c>
       <c r="F172" s="3">
-        <v>9946176.748959353</v>
+        <v>9946176.748959351</v>
       </c>
       <c r="G172" s="3">
         <v>10034617.12634464</v>
@@ -10142,7 +10142,7 @@
         <v>2586677.201497451</v>
       </c>
       <c r="G173" s="3">
-        <v>2633707.696070131</v>
+        <v>2633707.696070132</v>
       </c>
       <c r="H173" s="3">
         <v>2680738.190642813</v>
@@ -10163,13 +10163,13 @@
         <v>2974678.781722068</v>
       </c>
       <c r="N173" s="3">
-        <v>3033466.899937919</v>
+        <v>3033466.89993792</v>
       </c>
       <c r="O173" s="3">
-        <v>3092255.018153772</v>
+        <v>3092255.018153771</v>
       </c>
       <c r="P173" s="3">
-        <v>3162800.760012793</v>
+        <v>3162800.760012792</v>
       </c>
       <c r="Q173" s="3">
         <v>3221588.878228643</v>
@@ -11126,13 +11126,13 @@
         <v>0.8999999999999999</v>
       </c>
       <c r="I16" s="3">
-        <v>0.9</v>
+        <v>0.9000000000000002</v>
       </c>
       <c r="J16" s="3">
-        <v>0.8999999999999999</v>
+        <v>0.8999999999999998</v>
       </c>
       <c r="K16" s="3">
-        <v>0.9</v>
+        <v>0.8999999999999998</v>
       </c>
       <c r="L16" s="3">
         <v>0.9</v>
@@ -11147,13 +11147,13 @@
         <v>0.9</v>
       </c>
       <c r="P16" s="3">
-        <v>0.9</v>
+        <v>0.9000000000000002</v>
       </c>
       <c r="Q16" s="3">
-        <v>0.9</v>
+        <v>0.8999999999999998</v>
       </c>
       <c r="R16" s="3">
-        <v>0.9</v>
+        <v>0.8999999999999999</v>
       </c>
     </row>
     <row r="17" spans="1:18">
@@ -11206,10 +11206,10 @@
         <v>0.8080000000000001</v>
       </c>
       <c r="Q17" s="3">
+        <v>0.8079999999999999</v>
+      </c>
+      <c r="R17" s="3">
         <v>0.8080000000000002</v>
-      </c>
-      <c r="R17" s="3">
-        <v>0.8080000000000001</v>
       </c>
     </row>
     <row r="18" spans="1:18">
@@ -11518,7 +11518,7 @@
         <v>0.508</v>
       </c>
       <c r="I23" s="3">
-        <v>0.508</v>
+        <v>0.5080000000000001</v>
       </c>
       <c r="J23" s="3">
         <v>0.5079999999999999</v>
@@ -11542,10 +11542,10 @@
         <v>0.508</v>
       </c>
       <c r="Q23" s="3">
+        <v>0.5079999999999999</v>
+      </c>
+      <c r="R23" s="3">
         <v>0.508</v>
-      </c>
-      <c r="R23" s="3">
-        <v>0.5079999999999999</v>
       </c>
     </row>
     <row r="24" spans="1:18">
@@ -11742,13 +11742,13 @@
         <v>0.3538</v>
       </c>
       <c r="I27" s="3">
-        <v>0.3538</v>
+        <v>0.3538000000000001</v>
       </c>
       <c r="J27" s="3">
-        <v>0.3538</v>
+        <v>0.3537999999999999</v>
       </c>
       <c r="K27" s="3">
-        <v>0.3538</v>
+        <v>0.3537999999999999</v>
       </c>
       <c r="L27" s="3">
         <v>0.3538</v>
@@ -11763,10 +11763,10 @@
         <v>0.3537999999999999</v>
       </c>
       <c r="P27" s="3">
-        <v>0.3538</v>
+        <v>0.3538000000000001</v>
       </c>
       <c r="Q27" s="3">
-        <v>0.3538000000000001</v>
+        <v>0.3537999999999999</v>
       </c>
       <c r="R27" s="3">
         <v>0.3538</v>
@@ -12078,7 +12078,7 @@
         <v>0.8070000000000001</v>
       </c>
       <c r="I33" s="3">
-        <v>0.8070000000000001</v>
+        <v>0.8070000000000002</v>
       </c>
       <c r="J33" s="3">
         <v>0.8069999999999999</v>
@@ -12102,7 +12102,7 @@
         <v>0.8070000000000001</v>
       </c>
       <c r="Q33" s="3">
-        <v>0.8070000000000001</v>
+        <v>0.8069999999999999</v>
       </c>
       <c r="R33" s="3">
         <v>0.8070000000000001</v>
@@ -12134,13 +12134,13 @@
         <v>0.7319999999999999</v>
       </c>
       <c r="I34" s="3">
-        <v>0.732</v>
+        <v>0.7320000000000001</v>
       </c>
       <c r="J34" s="3">
         <v>0.7319999999999999</v>
       </c>
       <c r="K34" s="3">
-        <v>0.732</v>
+        <v>0.7319999999999999</v>
       </c>
       <c r="L34" s="3">
         <v>0.732</v>
@@ -12158,10 +12158,10 @@
         <v>0.732</v>
       </c>
       <c r="Q34" s="3">
+        <v>0.7319999999999999</v>
+      </c>
+      <c r="R34" s="3">
         <v>0.732</v>
-      </c>
-      <c r="R34" s="3">
-        <v>0.7319999999999999</v>
       </c>
     </row>
     <row r="35" spans="1:18">
@@ -12190,13 +12190,13 @@
         <v>0.316</v>
       </c>
       <c r="I35" s="3">
-        <v>0.316</v>
+        <v>0.3160000000000001</v>
       </c>
       <c r="J35" s="3">
         <v>0.3159999999999999</v>
       </c>
       <c r="K35" s="3">
-        <v>0.316</v>
+        <v>0.3159999999999999</v>
       </c>
       <c r="L35" s="3">
         <v>0.316</v>
@@ -12214,10 +12214,10 @@
         <v>0.316</v>
       </c>
       <c r="Q35" s="3">
-        <v>0.3160000000000001</v>
+        <v>0.3159999999999999</v>
       </c>
       <c r="R35" s="3">
-        <v>0.3159999999999999</v>
+        <v>0.316</v>
       </c>
     </row>
     <row r="36" spans="1:18">
@@ -12246,13 +12246,13 @@
         <v>0.597</v>
       </c>
       <c r="I36" s="3">
-        <v>0.597</v>
+        <v>0.5970000000000001</v>
       </c>
       <c r="J36" s="3">
         <v>0.5969999999999999</v>
       </c>
       <c r="K36" s="3">
-        <v>0.597</v>
+        <v>0.5969999999999999</v>
       </c>
       <c r="L36" s="3">
         <v>0.597</v>
@@ -12273,7 +12273,7 @@
         <v>0.597</v>
       </c>
       <c r="R36" s="3">
-        <v>0.5969999999999999</v>
+        <v>0.597</v>
       </c>
     </row>
     <row r="37" spans="1:18">
@@ -12302,7 +12302,7 @@
         <v>0.199</v>
       </c>
       <c r="I37" s="3">
-        <v>0.199</v>
+        <v>0.1990000000000001</v>
       </c>
       <c r="J37" s="3">
         <v>0.199</v>
@@ -13254,13 +13254,13 @@
         <v>4795699.531576274</v>
       </c>
       <c r="I54" s="3">
-        <v>4882894.068514024</v>
+        <v>4882894.068514025</v>
       </c>
       <c r="J54" s="3">
-        <v>4970088.605451776</v>
+        <v>4970088.605451775</v>
       </c>
       <c r="K54" s="3">
-        <v>5079081.776623963</v>
+        <v>5079081.776623962</v>
       </c>
       <c r="L54" s="3">
         <v>5188074.94779615</v>
@@ -13275,10 +13275,10 @@
         <v>5515054.461312715</v>
       </c>
       <c r="P54" s="3">
-        <v>5624047.632484903</v>
+        <v>5624047.632484904</v>
       </c>
       <c r="Q54" s="3">
-        <v>5733040.803657092</v>
+        <v>5733040.803657091</v>
       </c>
       <c r="R54" s="3">
         <v>5863832.609063718</v>
@@ -13646,7 +13646,7 @@
         <v>32177163.57078648</v>
       </c>
       <c r="I61" s="3">
-        <v>32944238.48461909</v>
+        <v>32944238.4846191</v>
       </c>
       <c r="J61" s="3">
         <v>33760488.74849692</v>
@@ -13673,7 +13673,7 @@
         <v>40606387.29998831</v>
       </c>
       <c r="R61" s="3">
-        <v>41711835.89346581</v>
+        <v>41711835.89346582</v>
       </c>
     </row>
     <row r="62" spans="1:18">
@@ -13873,7 +13873,7 @@
         <v>3522225.859247135</v>
       </c>
       <c r="J65" s="3">
-        <v>3585122.749590835</v>
+        <v>3585122.749590834</v>
       </c>
       <c r="K65" s="3">
         <v>3663743.862520458</v>
@@ -13891,10 +13891,10 @@
         <v>3978228.314238951</v>
       </c>
       <c r="P65" s="3">
-        <v>4056849.427168575</v>
+        <v>4056849.427168576</v>
       </c>
       <c r="Q65" s="3">
-        <v>4135470.540098201</v>
+        <v>4135470.5400982</v>
       </c>
       <c r="R65" s="3">
         <v>4229815.875613748</v>
@@ -14262,7 +14262,7 @@
         <v>15988110.05553604</v>
       </c>
       <c r="I72" s="3">
-        <v>16369252.35591988</v>
+        <v>16369252.35591989</v>
       </c>
       <c r="J72" s="3">
         <v>16774828.78353227</v>
@@ -14318,13 +14318,13 @@
         <v>605839677.3321218</v>
       </c>
       <c r="I73" s="3">
-        <v>620282355.5148512</v>
+        <v>620282355.5148513</v>
       </c>
       <c r="J73" s="3">
         <v>635650919.4779898</v>
       </c>
       <c r="K73" s="3">
-        <v>651921419.9578193</v>
+        <v>651921419.9578192</v>
       </c>
       <c r="L73" s="3">
         <v>669019995.3863199</v>
@@ -14342,10 +14342,10 @@
         <v>744319030.9808786</v>
       </c>
       <c r="Q73" s="3">
-        <v>764547208.3121463</v>
+        <v>764547208.3121461</v>
       </c>
       <c r="R73" s="3">
-        <v>785360870.7005765</v>
+        <v>785360870.7005768</v>
       </c>
     </row>
     <row r="74" spans="1:18">
@@ -14374,13 +14374,13 @@
         <v>449137754.7021943</v>
       </c>
       <c r="I74" s="3">
-        <v>459844798.6505909</v>
+        <v>459844798.650591</v>
       </c>
       <c r="J74" s="3">
         <v>471238245.7450391</v>
       </c>
       <c r="K74" s="3">
-        <v>483300341.2577857</v>
+        <v>483300341.2577856</v>
       </c>
       <c r="L74" s="3">
         <v>495976328.0970446</v>
@@ -14401,7 +14401,7 @@
         <v>566795192.4464384</v>
       </c>
       <c r="R74" s="3">
-        <v>582225349.8660299</v>
+        <v>582225349.86603</v>
       </c>
     </row>
     <row r="75" spans="1:18">
@@ -14436,7 +14436,7 @@
         <v>516841946.9461719</v>
       </c>
       <c r="K75" s="3">
-        <v>530071342.0246682</v>
+        <v>530071342.0246681</v>
       </c>
       <c r="L75" s="3">
         <v>543974037.2677264</v>
@@ -14457,7 +14457,7 @@
         <v>621646340.1025454</v>
       </c>
       <c r="R75" s="3">
-        <v>638569738.5627426</v>
+        <v>638569738.5627427</v>
       </c>
     </row>
     <row r="76" spans="1:18">
@@ -14474,10 +14474,10 @@
         <v>47</v>
       </c>
       <c r="E76" s="3">
-        <v>4346927.29696232</v>
+        <v>4346927.296962321</v>
       </c>
       <c r="F76" s="3">
-        <v>4346927.29696232</v>
+        <v>4346927.296962321</v>
       </c>
       <c r="G76" s="3">
         <v>4371726.161968159</v>
@@ -14811,7 +14811,7 @@
         <v>88701198676.77414</v>
       </c>
       <c r="J2" s="3">
-        <v>89927895248.36372</v>
+        <v>89927895248.36375</v>
       </c>
       <c r="K2" s="3">
         <v>91261290518.62175</v>
@@ -14820,19 +14820,19 @@
         <v>92865701998.12115</v>
       </c>
       <c r="M2" s="3">
-        <v>94538504990.61125</v>
+        <v>94538504990.61127</v>
       </c>
       <c r="N2" s="3">
-        <v>96308830600.54324</v>
+        <v>96308830600.54327</v>
       </c>
       <c r="O2" s="3">
-        <v>98157598152.15562</v>
+        <v>98157598152.15565</v>
       </c>
       <c r="P2" s="3">
         <v>100132395051.2629</v>
       </c>
       <c r="Q2" s="3">
-        <v>102100002580.3574</v>
+        <v>102100002580.3573</v>
       </c>
       <c r="R2" s="3">
         <v>1200315528825.385</v>
@@ -14864,7 +14864,7 @@
         <v>23755539227.70131</v>
       </c>
       <c r="I3" s="3">
-        <v>24193542646.22192</v>
+        <v>24193542646.22191</v>
       </c>
       <c r="J3" s="3">
         <v>24663022792.21271</v>
@@ -14876,22 +14876,22 @@
         <v>25629772914.10549</v>
       </c>
       <c r="M3" s="3">
-        <v>26148034679.62643</v>
+        <v>26148034679.62644</v>
       </c>
       <c r="N3" s="3">
         <v>26663852858.32975</v>
       </c>
       <c r="O3" s="3">
-        <v>27183205214.17332</v>
+        <v>27183205214.17334</v>
       </c>
       <c r="P3" s="3">
         <v>27767491490.77292</v>
       </c>
       <c r="Q3" s="3">
-        <v>28310005492.26731</v>
+        <v>28310005492.2673</v>
       </c>
       <c r="R3" s="3">
-        <v>328637162409.901</v>
+        <v>328637162409.9009</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -14979,19 +14979,19 @@
         <v>60445818498.28165</v>
       </c>
       <c r="J5" s="3">
-        <v>61118607432.16673</v>
+        <v>61118607432.16676</v>
       </c>
       <c r="K5" s="3">
-        <v>61955336931.67776</v>
+        <v>61955336931.67777</v>
       </c>
       <c r="L5" s="3">
         <v>62920935836.47665</v>
       </c>
       <c r="M5" s="3">
-        <v>63986344444.21933</v>
+        <v>63986344444.21935</v>
       </c>
       <c r="N5" s="3">
-        <v>65153685279.96465</v>
+        <v>65153685279.96468</v>
       </c>
       <c r="O5" s="3">
         <v>66395700215.58045</v>
@@ -15003,7 +15003,7 @@
         <v>69020007427.4411</v>
       </c>
       <c r="R5" s="3">
-        <v>816497274303.5044</v>
+        <v>816497274303.5046</v>
       </c>
     </row>
     <row r="6" spans="1:18">
@@ -15265,7 +15265,7 @@
         <v>95741.96454501257</v>
       </c>
       <c r="L10" s="3">
-        <v>98115.73226100462</v>
+        <v>98115.73226100461</v>
       </c>
       <c r="M10" s="3">
         <v>100093.8720243313</v>
@@ -15274,7 +15274,7 @@
         <v>102072.011787658</v>
       </c>
       <c r="O10" s="3">
-        <v>104050.1515509847</v>
+        <v>104050.1515509848</v>
       </c>
       <c r="P10" s="3">
         <v>106423.9192669768</v>
@@ -15346,7 +15346,7 @@
         <v>95974517964.467</v>
       </c>
       <c r="O12" s="3">
-        <v>97819499130.80617</v>
+        <v>97819499130.80615</v>
       </c>
       <c r="P12" s="3">
         <v>99788108892.54088</v>
@@ -15549,10 +15549,10 @@
         <v>557356873.2126849</v>
       </c>
       <c r="H16" s="3">
-        <v>563519109.370102</v>
+        <v>563519109.3701019</v>
       </c>
       <c r="I16" s="3">
-        <v>571309335.4406751</v>
+        <v>571309335.4406749</v>
       </c>
       <c r="J16" s="3">
         <v>580527636.1331575</v>
@@ -15596,13 +15596,13 @@
         <v>0</v>
       </c>
       <c r="E17" s="3">
-        <v>385238536.7356724</v>
+        <v>385238536.7356723</v>
       </c>
       <c r="F17" s="3">
         <v>392281478.6568038</v>
       </c>
       <c r="G17" s="3">
-        <v>399472639.4038136</v>
+        <v>399472639.4038135</v>
       </c>
       <c r="H17" s="3">
         <v>406622307.2251863</v>
@@ -15632,7 +15632,7 @@
         <v>479519514.6398069</v>
       </c>
       <c r="Q17" s="3">
-        <v>488613223.7380732</v>
+        <v>488613223.738073</v>
       </c>
       <c r="R17" s="3">
         <v>5645174654.467421</v>
@@ -15682,7 +15682,7 @@
         <v>315476169.9169589</v>
       </c>
       <c r="O18" s="3">
-        <v>321590049.1789155</v>
+        <v>321590049.1789154</v>
       </c>
       <c r="P18" s="3">
         <v>328926704.2932634</v>
@@ -15785,7 +15785,7 @@
         <v>95741.96454501257</v>
       </c>
       <c r="L20" s="3">
-        <v>98115.73226100462</v>
+        <v>98115.73226100461</v>
       </c>
       <c r="M20" s="3">
         <v>100093.8720243313</v>
@@ -15794,7 +15794,7 @@
         <v>102072.011787658</v>
       </c>
       <c r="O20" s="3">
-        <v>104050.1515509847</v>
+        <v>104050.1515509848</v>
       </c>
       <c r="P20" s="3">
         <v>106423.9192669768</v>
@@ -16034,7 +16034,7 @@
         <v>65245965949.53699</v>
       </c>
       <c r="O25" s="3">
-        <v>66492264515.64706</v>
+        <v>66492264515.64705</v>
       </c>
       <c r="P25" s="3">
         <v>67785699713.84539</v>
@@ -16305,7 +16305,7 @@
         <v>95741.96454501257</v>
       </c>
       <c r="L30" s="3">
-        <v>98115.73226100462</v>
+        <v>98115.73226100461</v>
       </c>
       <c r="M30" s="3">
         <v>100093.8720243313</v>
@@ -16314,7 +16314,7 @@
         <v>102072.011787658</v>
       </c>
       <c r="O30" s="3">
-        <v>104050.1515509847</v>
+        <v>104050.1515509848</v>
       </c>
       <c r="P30" s="3">
         <v>106423.9192669768</v>
@@ -16362,7 +16362,7 @@
         <v>85895405920.56883</v>
       </c>
       <c r="G32" s="3">
-        <v>86364575388.29008</v>
+        <v>86364575388.2901</v>
       </c>
       <c r="H32" s="3">
         <v>86938926959.89204</v>
@@ -16371,7 +16371,7 @@
         <v>87800519013.16684</v>
       </c>
       <c r="J32" s="3">
-        <v>88899629757.35506</v>
+        <v>88899629757.35507</v>
       </c>
       <c r="K32" s="3">
         <v>90133707262.71797</v>
@@ -16383,13 +16383,13 @@
         <v>93267972872.38805</v>
       </c>
       <c r="N32" s="3">
-        <v>94984033754.31358</v>
+        <v>94984033754.3136</v>
       </c>
       <c r="O32" s="3">
         <v>96785568554.07823</v>
       </c>
       <c r="P32" s="3">
-        <v>98718105551.78349</v>
+        <v>98718105551.78351</v>
       </c>
       <c r="Q32" s="3">
         <v>100646733749.5054</v>
@@ -16418,7 +16418,7 @@
         <v>23020619409.36172</v>
       </c>
       <c r="G33" s="3">
-        <v>23333356329.56184</v>
+        <v>23333356329.56185</v>
       </c>
       <c r="H33" s="3">
         <v>23685494391.55053</v>
@@ -16427,13 +16427,13 @@
         <v>24118589225.29538</v>
       </c>
       <c r="J33" s="3">
-        <v>24584011399.60011</v>
+        <v>24584011399.60012</v>
       </c>
       <c r="K33" s="3">
-        <v>25005033297.81782</v>
+        <v>25005033297.81783</v>
       </c>
       <c r="L33" s="3">
-        <v>25544485278.98873</v>
+        <v>25544485278.98874</v>
       </c>
       <c r="M33" s="3">
         <v>26060043497.2495</v>
@@ -16445,13 +16445,13 @@
         <v>27090487159.6801</v>
       </c>
       <c r="P33" s="3">
-        <v>27672582611.4846</v>
+        <v>27672582611.48461</v>
       </c>
       <c r="Q33" s="3">
-        <v>28212898382.31876</v>
+        <v>28212898382.31877</v>
       </c>
       <c r="R33" s="3">
-        <v>327646358028.0221</v>
+        <v>327646358028.0222</v>
       </c>
     </row>
     <row r="34" spans="1:18">
@@ -16530,7 +16530,7 @@
         <v>59039345928.99995</v>
       </c>
       <c r="G35" s="3">
-        <v>59138963566.47988</v>
+        <v>59138963566.47987</v>
       </c>
       <c r="H35" s="3">
         <v>59293621663.45361</v>
@@ -16557,10 +16557,10 @@
         <v>65138225377.09432</v>
       </c>
       <c r="P35" s="3">
-        <v>66388433742.53746</v>
+        <v>66388433742.53744</v>
       </c>
       <c r="Q35" s="3">
-        <v>67686706279.47561</v>
+        <v>67686706279.47553</v>
       </c>
       <c r="R35" s="3">
         <v>804970043425.6864</v>
@@ -16586,7 +16586,7 @@
         <v>527451129.4141288</v>
       </c>
       <c r="G36" s="3">
-        <v>518813093.6073348</v>
+        <v>518813093.6073347</v>
       </c>
       <c r="H36" s="3">
         <v>524317116.5250738</v>
@@ -16595,10 +16595,10 @@
         <v>531344989.3000982</v>
       </c>
       <c r="J36" s="3">
-        <v>539807724.5950991</v>
+        <v>539807724.5950989</v>
       </c>
       <c r="K36" s="3">
-        <v>548923616.3308256</v>
+        <v>548923616.3308254</v>
       </c>
       <c r="L36" s="3">
         <v>558987325.3784565</v>
@@ -16619,7 +16619,7 @@
         <v>616448458.1270918</v>
       </c>
       <c r="R36" s="3">
-        <v>7243012769.993534</v>
+        <v>7243012769.993532</v>
       </c>
     </row>
     <row r="37" spans="1:18">
@@ -16642,7 +16642,7 @@
         <v>392945857.3348823</v>
       </c>
       <c r="G37" s="3">
-        <v>400152939.2419666</v>
+        <v>400152939.2419663</v>
       </c>
       <c r="H37" s="3">
         <v>407315039.0762282</v>
@@ -16651,31 +16651,31 @@
         <v>416091517.7225049</v>
       </c>
       <c r="J37" s="3">
-        <v>425028473.6309438</v>
+        <v>425028473.6309436</v>
       </c>
       <c r="K37" s="3">
-        <v>432358838.1178977</v>
+        <v>432358838.1178975</v>
       </c>
       <c r="L37" s="3">
-        <v>442764072.7584697</v>
+        <v>442764072.7584693</v>
       </c>
       <c r="M37" s="3">
-        <v>451862478.5214282</v>
+        <v>451862478.521428</v>
       </c>
       <c r="N37" s="3">
-        <v>460821142.0871657</v>
+        <v>460821142.0871655</v>
       </c>
       <c r="O37" s="3">
         <v>469770382.800914</v>
       </c>
       <c r="P37" s="3">
-        <v>480336398.6116697</v>
+        <v>480336398.6116696</v>
       </c>
       <c r="Q37" s="3">
         <v>489445644.028509</v>
       </c>
       <c r="R37" s="3">
-        <v>5654729650.536949</v>
+        <v>5654729650.536948</v>
       </c>
     </row>
     <row r="38" spans="1:18">
@@ -16825,7 +16825,7 @@
         <v>95741.96454501257</v>
       </c>
       <c r="L40" s="3">
-        <v>98115.73226100462</v>
+        <v>98115.73226100461</v>
       </c>
       <c r="M40" s="3">
         <v>100093.8720243313</v>
@@ -16834,7 +16834,7 @@
         <v>102072.011787658</v>
       </c>
       <c r="O40" s="3">
-        <v>104050.1515509847</v>
+        <v>104050.1515509848</v>
       </c>
       <c r="P40" s="3">
         <v>106423.9192669768</v>
@@ -16879,25 +16879,25 @@
         <v>85057136474.33154</v>
       </c>
       <c r="F42" s="3">
-        <v>85484028213.05547</v>
+        <v>85484028213.05548</v>
       </c>
       <c r="G42" s="3">
-        <v>85926306065.71637</v>
+        <v>85926306065.71635</v>
       </c>
       <c r="H42" s="3">
-        <v>86476133190.75908</v>
+        <v>86476133190.75911</v>
       </c>
       <c r="I42" s="3">
-        <v>87317405216.70778</v>
+        <v>87317405216.70782</v>
       </c>
       <c r="J42" s="3">
         <v>88399490423.86102</v>
       </c>
       <c r="K42" s="3">
-        <v>89620382625.6403</v>
+        <v>89620382625.64032</v>
       </c>
       <c r="L42" s="3">
-        <v>91130812571.15929</v>
+        <v>91130812571.15927</v>
       </c>
       <c r="M42" s="3">
         <v>92726452158.05679</v>
@@ -16909,13 +16909,13 @@
         <v>96220009708.43658</v>
       </c>
       <c r="P42" s="3">
-        <v>98139205653.85805</v>
+        <v>98139205653.85806</v>
       </c>
       <c r="Q42" s="3">
         <v>100056275943.8316</v>
       </c>
       <c r="R42" s="3">
-        <v>1180983954673.317</v>
+        <v>1180983954673.318</v>
       </c>
     </row>
     <row r="43" spans="1:18">
@@ -16935,10 +16935,10 @@
         <v>22377101653.58879</v>
       </c>
       <c r="F43" s="3">
-        <v>22646257697.5076</v>
+        <v>22646257697.50761</v>
       </c>
       <c r="G43" s="3">
-        <v>22950892020.05472</v>
+        <v>22950892020.05471</v>
       </c>
       <c r="H43" s="3">
         <v>23296485172.74183</v>
@@ -16947,7 +16947,7 @@
         <v>23721253905.77665</v>
       </c>
       <c r="J43" s="3">
-        <v>24178182872.92615</v>
+        <v>24178182872.92614</v>
       </c>
       <c r="K43" s="3">
         <v>24592501677.64723</v>
@@ -16956,7 +16956,7 @@
         <v>25121871234.73149</v>
       </c>
       <c r="M43" s="3">
-        <v>25628782310.22328</v>
+        <v>25628782310.22327</v>
       </c>
       <c r="N43" s="3">
         <v>26133721163.89852</v>
@@ -17053,37 +17053,37 @@
         <v>59033014017.88582</v>
       </c>
       <c r="H45" s="3">
-        <v>59126670346.97045</v>
+        <v>59126670346.97044</v>
       </c>
       <c r="I45" s="3">
         <v>59423895164.46609</v>
       </c>
       <c r="J45" s="3">
-        <v>59933955034.50418</v>
+        <v>59933955034.50415</v>
       </c>
       <c r="K45" s="3">
         <v>60644433705.06557</v>
       </c>
       <c r="L45" s="3">
-        <v>61510573912.44298</v>
+        <v>61510573912.44295</v>
       </c>
       <c r="M45" s="3">
-        <v>62495711573.7495</v>
+        <v>62495711573.74945</v>
       </c>
       <c r="N45" s="3">
-        <v>63595717737.2211</v>
+        <v>63595717737.22106</v>
       </c>
       <c r="O45" s="3">
         <v>64779539770.52294</v>
       </c>
       <c r="P45" s="3">
-        <v>66017723973.9257</v>
+        <v>66017723973.92571</v>
       </c>
       <c r="Q45" s="3">
-        <v>67305092236.35567</v>
+        <v>67305092236.35569</v>
       </c>
       <c r="R45" s="3">
-        <v>801779532571.8883</v>
+        <v>801779532571.8881</v>
       </c>
     </row>
     <row r="46" spans="1:18">
@@ -17112,7 +17112,7 @@
         <v>523291763.6234319</v>
       </c>
       <c r="I46" s="3">
-        <v>530463814.8859394</v>
+        <v>530463814.8859393</v>
       </c>
       <c r="J46" s="3">
         <v>538905779.0555878</v>
@@ -17124,22 +17124,22 @@
         <v>557914206.4967624</v>
       </c>
       <c r="M46" s="3">
-        <v>568658375.2865748</v>
+        <v>568658375.2865747</v>
       </c>
       <c r="N46" s="3">
-        <v>579769263.6840978</v>
+        <v>579769263.6840976</v>
       </c>
       <c r="O46" s="3">
-        <v>591116804.7437401</v>
+        <v>591116804.7437402</v>
       </c>
       <c r="P46" s="3">
         <v>603005742.5428466</v>
       </c>
       <c r="Q46" s="3">
-        <v>615148423.2289232</v>
+        <v>615148423.2289233</v>
       </c>
       <c r="R46" s="3">
-        <v>7229219167.00788</v>
+        <v>7229219167.007881</v>
       </c>
     </row>
     <row r="47" spans="1:18">
@@ -17168,22 +17168,22 @@
         <v>406622307.2252215</v>
       </c>
       <c r="I47" s="3">
-        <v>415383882.3480309</v>
+        <v>415383882.3480308</v>
       </c>
       <c r="J47" s="3">
         <v>424305638.2157612</v>
       </c>
       <c r="K47" s="3">
-        <v>431623487.9511803</v>
+        <v>431623487.9511804</v>
       </c>
       <c r="L47" s="3">
         <v>442011103.9804206</v>
       </c>
       <c r="M47" s="3">
-        <v>451093996.5761472</v>
+        <v>451093996.5761469</v>
       </c>
       <c r="N47" s="3">
-        <v>460037414.8552002</v>
+        <v>460037414.8552001</v>
       </c>
       <c r="O47" s="3">
         <v>468971430.1415914</v>
@@ -17215,13 +17215,13 @@
         <v>262896808.2641324</v>
       </c>
       <c r="F48" s="3">
-        <v>269010687.5260888</v>
+        <v>269010687.5260889</v>
       </c>
       <c r="G48" s="3">
         <v>273901790.9356542</v>
       </c>
       <c r="H48" s="3">
-        <v>278792894.3452193</v>
+        <v>278792894.3452194</v>
       </c>
       <c r="I48" s="3">
         <v>284906773.607176</v>
@@ -17233,7 +17233,7 @@
         <v>295911756.2786978</v>
       </c>
       <c r="L48" s="3">
-        <v>303248411.3930456</v>
+        <v>303248411.3930457</v>
       </c>
       <c r="M48" s="3">
         <v>309362290.6550022</v>
@@ -17345,7 +17345,7 @@
         <v>95741.96454501257</v>
       </c>
       <c r="L50" s="3">
-        <v>98115.73226100462</v>
+        <v>98115.73226100461</v>
       </c>
       <c r="M50" s="3">
         <v>100093.8720243313</v>
@@ -17354,7 +17354,7 @@
         <v>102072.011787658</v>
       </c>
       <c r="O50" s="3">
-        <v>104050.1515509847</v>
+        <v>104050.1515509848</v>
       </c>
       <c r="P50" s="3">
         <v>106423.9192669768</v>
@@ -17402,34 +17402,34 @@
         <v>86251606603.36079</v>
       </c>
       <c r="G52" s="3">
-        <v>86679891389.21921</v>
+        <v>86679891389.21919</v>
       </c>
       <c r="H52" s="3">
-        <v>87207863599.68184</v>
+        <v>87207863599.68181</v>
       </c>
       <c r="I52" s="3">
-        <v>88033238671.04494</v>
+        <v>88033238671.04492</v>
       </c>
       <c r="J52" s="3">
-        <v>89105795860.56511</v>
+        <v>89105795860.56508</v>
       </c>
       <c r="K52" s="3">
         <v>90319899897.96388</v>
       </c>
       <c r="L52" s="3">
-        <v>91834309048.09198</v>
+        <v>91834309048.09195</v>
       </c>
       <c r="M52" s="3">
-        <v>93434750595.03107</v>
+        <v>93434750595.03102</v>
       </c>
       <c r="N52" s="3">
-        <v>95145661437.24594</v>
+        <v>95145661437.2459</v>
       </c>
       <c r="O52" s="3">
-        <v>96944209261.95732</v>
+        <v>96944209261.95734</v>
       </c>
       <c r="P52" s="3">
-        <v>98876663864.7675</v>
+        <v>98876663864.76749</v>
       </c>
       <c r="Q52" s="3">
         <v>100804947842.6896</v>
@@ -17455,16 +17455,16 @@
         <v>23144087272.4607</v>
       </c>
       <c r="F53" s="3">
-        <v>23423424336.8319</v>
+        <v>23423424336.83191</v>
       </c>
       <c r="G53" s="3">
         <v>23740350604.92076</v>
       </c>
       <c r="H53" s="3">
-        <v>24095907314.52385</v>
+        <v>24095907314.52383</v>
       </c>
       <c r="I53" s="3">
-        <v>24534753196.9955</v>
+        <v>24534753196.99551</v>
       </c>
       <c r="J53" s="3">
         <v>25006758016.70269</v>
@@ -17573,22 +17573,22 @@
         <v>59156282253.31814</v>
       </c>
       <c r="H55" s="3">
-        <v>59316156278.25109</v>
+        <v>59316156278.2511</v>
       </c>
       <c r="I55" s="3">
-        <v>59668917117.21499</v>
+        <v>59668917117.215</v>
       </c>
       <c r="J55" s="3">
         <v>60222656707.84081</v>
       </c>
       <c r="K55" s="3">
-        <v>60967170321.25809</v>
+        <v>60967170321.25811</v>
       </c>
       <c r="L55" s="3">
         <v>61860058628.06026</v>
       </c>
       <c r="M55" s="3">
-        <v>62866652402.18303</v>
+        <v>62866652402.18304</v>
       </c>
       <c r="N55" s="3">
         <v>63984501298.11093</v>
@@ -17597,10 +17597,10 @@
         <v>65183604473.34687</v>
       </c>
       <c r="P55" s="3">
-        <v>66435217999.32922</v>
+        <v>66435217999.32925</v>
       </c>
       <c r="Q55" s="3">
-        <v>67734771192.65767</v>
+        <v>67734771192.65773</v>
       </c>
       <c r="R55" s="3">
         <v>805390310592.4091</v>
@@ -17626,7 +17626,7 @@
         <v>528582696.6969749</v>
       </c>
       <c r="G56" s="3">
-        <v>520449844.4483614</v>
+        <v>520449844.4483613</v>
       </c>
       <c r="H56" s="3">
         <v>526188216.4028171</v>
@@ -17635,13 +17635,13 @@
         <v>533400664.3937548</v>
       </c>
       <c r="J56" s="3">
-        <v>541926919.8652391</v>
+        <v>541926919.8652393</v>
       </c>
       <c r="K56" s="3">
         <v>551048487.7459986</v>
       </c>
       <c r="L56" s="3">
-        <v>561125279.6084211</v>
+        <v>561125279.608421</v>
       </c>
       <c r="M56" s="3">
         <v>571957321.4580852</v>
@@ -17656,7 +17656,7 @@
         <v>606542870.8691392</v>
       </c>
       <c r="Q56" s="3">
-        <v>618762046.1928821</v>
+        <v>618762046.1928822</v>
       </c>
       <c r="R56" s="3">
         <v>7268066293.262846</v>
@@ -17679,10 +17679,10 @@
         <v>386283396.1941368</v>
       </c>
       <c r="F57" s="3">
-        <v>393441419.4533958</v>
+        <v>393441419.4533957</v>
       </c>
       <c r="G57" s="3">
-        <v>400660363.2108887</v>
+        <v>400660363.2108886</v>
       </c>
       <c r="H57" s="3">
         <v>407831735.7899392</v>
@@ -17703,7 +17703,7 @@
         <v>452435669.6227673</v>
       </c>
       <c r="N57" s="3">
-        <v>461405706.1445109</v>
+        <v>461405706.144511</v>
       </c>
       <c r="O57" s="3">
         <v>470366304.1549186</v>
@@ -17732,10 +17732,10 @@
         <v>0</v>
       </c>
       <c r="E58" s="3">
-        <v>263734087.1758113</v>
+        <v>263734087.1758114</v>
       </c>
       <c r="F58" s="3">
-        <v>269867438.040365</v>
+        <v>269867438.0403651</v>
       </c>
       <c r="G58" s="3">
         <v>274774118.732008</v>
@@ -17753,7 +17753,7 @@
         <v>296854181.8444016</v>
       </c>
       <c r="L58" s="3">
-        <v>304214202.881866</v>
+        <v>304214202.8818661</v>
       </c>
       <c r="M58" s="3">
         <v>310347553.7464198</v>
@@ -17765,7 +17765,7 @@
         <v>322614255.4755274</v>
       </c>
       <c r="P58" s="3">
-        <v>329974276.5129918</v>
+        <v>329974276.5129919</v>
       </c>
       <c r="Q58" s="3">
         <v>336107627.3775457</v>
@@ -17865,7 +17865,7 @@
         <v>95741.96454501257</v>
       </c>
       <c r="L60" s="3">
-        <v>98115.73226100462</v>
+        <v>98115.73226100461</v>
       </c>
       <c r="M60" s="3">
         <v>100093.8720243313</v>
@@ -17874,7 +17874,7 @@
         <v>102072.011787658</v>
       </c>
       <c r="O60" s="3">
-        <v>104050.1515509847</v>
+        <v>104050.1515509848</v>
       </c>
       <c r="P60" s="3">
         <v>106423.9192669768</v>

</xml_diff>